<commit_message>
Invulformulier: voorsp/uitslag/pt kolomkoppen toegevoegd aan KO-rondes
</commit_message>
<xml_diff>
--- a/tempetoto2026_invulformulier.xlsx
+++ b/tempetoto2026_invulformulier.xlsx
@@ -1490,7 +1490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O203"/>
+  <dimension ref="A1:O208"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -3505,20 +3505,27 @@
         </is>
       </c>
     </row>
-    <row r="110" ht="16" customHeight="1">
-      <c r="A110" s="61" t="inlineStr">
-        <is>
-          <t>2A  –  2B</t>
-        </is>
-      </c>
-      <c r="E110" s="18" t="inlineStr"/>
-      <c r="F110" s="18" t="inlineStr"/>
-      <c r="G110" s="18" t="inlineStr"/>
+    <row r="110" ht="14" customHeight="1">
+      <c r="E110" s="13" t="inlineStr">
+        <is>
+          <t>voorsp.</t>
+        </is>
+      </c>
+      <c r="F110" s="13" t="inlineStr">
+        <is>
+          <t>uitslag</t>
+        </is>
+      </c>
+      <c r="G110" s="13" t="inlineStr">
+        <is>
+          <t>pt.</t>
+        </is>
+      </c>
     </row>
     <row r="111" ht="16" customHeight="1">
       <c r="A111" s="61" t="inlineStr">
         <is>
-          <t>1E  –  3e (A/B/C/D/F)</t>
+          <t>2A  –  2B</t>
         </is>
       </c>
       <c r="E111" s="18" t="inlineStr"/>
@@ -3528,7 +3535,7 @@
     <row r="112" ht="16" customHeight="1">
       <c r="A112" s="61" t="inlineStr">
         <is>
-          <t>1F  –  2C</t>
+          <t>1E  –  3e (A/B/C/D/F)</t>
         </is>
       </c>
       <c r="E112" s="18" t="inlineStr"/>
@@ -3538,7 +3545,7 @@
     <row r="113" ht="16" customHeight="1">
       <c r="A113" s="61" t="inlineStr">
         <is>
-          <t>1C  –  2F</t>
+          <t>1F  –  2C</t>
         </is>
       </c>
       <c r="E113" s="18" t="inlineStr"/>
@@ -3548,7 +3555,7 @@
     <row r="114" ht="16" customHeight="1">
       <c r="A114" s="61" t="inlineStr">
         <is>
-          <t>1I  –  3e (C/D/F/G/H)</t>
+          <t>1C  –  2F</t>
         </is>
       </c>
       <c r="E114" s="18" t="inlineStr"/>
@@ -3558,7 +3565,7 @@
     <row r="115" ht="16" customHeight="1">
       <c r="A115" s="61" t="inlineStr">
         <is>
-          <t>2E  –  2I</t>
+          <t>1I  –  3e (C/D/F/G/H)</t>
         </is>
       </c>
       <c r="E115" s="18" t="inlineStr"/>
@@ -3568,7 +3575,7 @@
     <row r="116" ht="16" customHeight="1">
       <c r="A116" s="61" t="inlineStr">
         <is>
-          <t>1A  –  3e (C/E/F/H/I)</t>
+          <t>2E  –  2I</t>
         </is>
       </c>
       <c r="E116" s="18" t="inlineStr"/>
@@ -3578,7 +3585,7 @@
     <row r="117" ht="16" customHeight="1">
       <c r="A117" s="61" t="inlineStr">
         <is>
-          <t>1L  –  3e (E/H/I/J/K)</t>
+          <t>1A  –  3e (C/E/F/H/I)</t>
         </is>
       </c>
       <c r="E117" s="18" t="inlineStr"/>
@@ -3588,7 +3595,7 @@
     <row r="118" ht="16" customHeight="1">
       <c r="A118" s="61" t="inlineStr">
         <is>
-          <t>1D  –  3e (B/E/F/I/J)</t>
+          <t>1L  –  3e (E/H/I/J/K)</t>
         </is>
       </c>
       <c r="E118" s="18" t="inlineStr"/>
@@ -3598,7 +3605,7 @@
     <row r="119" ht="16" customHeight="1">
       <c r="A119" s="61" t="inlineStr">
         <is>
-          <t>1G  –  3e (A/E/H/I/J)</t>
+          <t>1D  –  3e (B/E/F/I/J)</t>
         </is>
       </c>
       <c r="E119" s="18" t="inlineStr"/>
@@ -3608,7 +3615,7 @@
     <row r="120" ht="16" customHeight="1">
       <c r="A120" s="61" t="inlineStr">
         <is>
-          <t>2K  –  2L</t>
+          <t>1G  –  3e (A/E/H/I/J)</t>
         </is>
       </c>
       <c r="E120" s="18" t="inlineStr"/>
@@ -3618,7 +3625,7 @@
     <row r="121" ht="16" customHeight="1">
       <c r="A121" s="61" t="inlineStr">
         <is>
-          <t>1H  –  2J</t>
+          <t>2K  –  2L</t>
         </is>
       </c>
       <c r="E121" s="18" t="inlineStr"/>
@@ -3628,7 +3635,7 @@
     <row r="122" ht="16" customHeight="1">
       <c r="A122" s="61" t="inlineStr">
         <is>
-          <t>1B  –  3e (E/F/G/I/J)</t>
+          <t>1H  –  2J</t>
         </is>
       </c>
       <c r="E122" s="18" t="inlineStr"/>
@@ -3638,7 +3645,7 @@
     <row r="123" ht="16" customHeight="1">
       <c r="A123" s="61" t="inlineStr">
         <is>
-          <t>1J  –  2H</t>
+          <t>1B  –  3e (E/F/G/I/J)</t>
         </is>
       </c>
       <c r="E123" s="18" t="inlineStr"/>
@@ -3648,7 +3655,7 @@
     <row r="124" ht="16" customHeight="1">
       <c r="A124" s="61" t="inlineStr">
         <is>
-          <t>1K  –  3e (D/E/I/J/L)</t>
+          <t>1J  –  2H</t>
         </is>
       </c>
       <c r="E124" s="18" t="inlineStr"/>
@@ -3658,45 +3665,52 @@
     <row r="125" ht="16" customHeight="1">
       <c r="A125" s="61" t="inlineStr">
         <is>
-          <t>2D  –  2G</t>
+          <t>1K  –  3e (D/E/I/J/L)</t>
         </is>
       </c>
       <c r="E125" s="18" t="inlineStr"/>
       <c r="F125" s="18" t="inlineStr"/>
       <c r="G125" s="18" t="inlineStr"/>
     </row>
-    <row r="126" ht="6" customHeight="1"/>
-    <row r="127" ht="16" customHeight="1">
-      <c r="A127" s="10" t="inlineStr">
+    <row r="126" ht="16" customHeight="1">
+      <c r="A126" s="61" t="inlineStr">
+        <is>
+          <t>2D  –  2G</t>
+        </is>
+      </c>
+      <c r="E126" s="18" t="inlineStr"/>
+      <c r="F126" s="18" t="inlineStr"/>
+      <c r="G126" s="18" t="inlineStr"/>
+    </row>
+    <row r="127" ht="6" customHeight="1"/>
+    <row r="128" ht="16" customHeight="1">
+      <c r="A128" s="10" t="inlineStr">
         <is>
           <t>Ronde van 16  ·  toto 7 pt / exact +4 pt</t>
         </is>
       </c>
     </row>
-    <row r="128" ht="16" customHeight="1">
-      <c r="A128" s="61" t="inlineStr">
-        <is>
-          <t>W32-2  –  W32-5</t>
-        </is>
-      </c>
-      <c r="E128" s="18" t="inlineStr"/>
-      <c r="F128" s="18" t="inlineStr"/>
-      <c r="G128" s="18" t="inlineStr"/>
-    </row>
-    <row r="129" ht="16" customHeight="1">
-      <c r="A129" s="61" t="inlineStr">
-        <is>
-          <t>W32-1  –  W32-3</t>
-        </is>
-      </c>
-      <c r="E129" s="18" t="inlineStr"/>
-      <c r="F129" s="18" t="inlineStr"/>
-      <c r="G129" s="18" t="inlineStr"/>
+    <row r="129" ht="14" customHeight="1">
+      <c r="E129" s="13" t="inlineStr">
+        <is>
+          <t>voorsp.</t>
+        </is>
+      </c>
+      <c r="F129" s="13" t="inlineStr">
+        <is>
+          <t>uitslag</t>
+        </is>
+      </c>
+      <c r="G129" s="13" t="inlineStr">
+        <is>
+          <t>pt.</t>
+        </is>
+      </c>
     </row>
     <row r="130" ht="16" customHeight="1">
       <c r="A130" s="61" t="inlineStr">
         <is>
-          <t>W32-4  –  W32-6</t>
+          <t>W32-2  –  W32-5</t>
         </is>
       </c>
       <c r="E130" s="18" t="inlineStr"/>
@@ -3706,7 +3720,7 @@
     <row r="131" ht="16" customHeight="1">
       <c r="A131" s="61" t="inlineStr">
         <is>
-          <t>W32-7  –  W32-8</t>
+          <t>W32-1  –  W32-3</t>
         </is>
       </c>
       <c r="E131" s="18" t="inlineStr"/>
@@ -3716,7 +3730,7 @@
     <row r="132" ht="16" customHeight="1">
       <c r="A132" s="61" t="inlineStr">
         <is>
-          <t>W32-11  –  W32-12</t>
+          <t>W32-4  –  W32-6</t>
         </is>
       </c>
       <c r="E132" s="18" t="inlineStr"/>
@@ -3726,7 +3740,7 @@
     <row r="133" ht="16" customHeight="1">
       <c r="A133" s="61" t="inlineStr">
         <is>
-          <t>W32-9  –  W32-10</t>
+          <t>W32-7  –  W32-8</t>
         </is>
       </c>
       <c r="E133" s="18" t="inlineStr"/>
@@ -3736,7 +3750,7 @@
     <row r="134" ht="16" customHeight="1">
       <c r="A134" s="61" t="inlineStr">
         <is>
-          <t>W32-14  –  W32-16</t>
+          <t>W32-11  –  W32-12</t>
         </is>
       </c>
       <c r="E134" s="18" t="inlineStr"/>
@@ -3746,1200 +3760,1271 @@
     <row r="135" ht="16" customHeight="1">
       <c r="A135" s="61" t="inlineStr">
         <is>
-          <t>W32-13  –  W32-15</t>
+          <t>W32-9  –  W32-10</t>
         </is>
       </c>
       <c r="E135" s="18" t="inlineStr"/>
       <c r="F135" s="18" t="inlineStr"/>
       <c r="G135" s="18" t="inlineStr"/>
     </row>
-    <row r="136" ht="6" customHeight="1"/>
+    <row r="136" ht="16" customHeight="1">
+      <c r="A136" s="61" t="inlineStr">
+        <is>
+          <t>W32-14  –  W32-16</t>
+        </is>
+      </c>
+      <c r="E136" s="18" t="inlineStr"/>
+      <c r="F136" s="18" t="inlineStr"/>
+      <c r="G136" s="18" t="inlineStr"/>
+    </row>
     <row r="137" ht="16" customHeight="1">
-      <c r="A137" s="10" t="inlineStr">
+      <c r="A137" s="61" t="inlineStr">
+        <is>
+          <t>W32-13  –  W32-15</t>
+        </is>
+      </c>
+      <c r="E137" s="18" t="inlineStr"/>
+      <c r="F137" s="18" t="inlineStr"/>
+      <c r="G137" s="18" t="inlineStr"/>
+    </row>
+    <row r="138" ht="6" customHeight="1"/>
+    <row r="139" ht="16" customHeight="1">
+      <c r="A139" s="10" t="inlineStr">
         <is>
           <t>Kwartfinales  ·  toto 9 pt / exact +5 pt</t>
         </is>
       </c>
     </row>
-    <row r="138" ht="16" customHeight="1">
-      <c r="A138" s="61" t="inlineStr">
-        <is>
-          <t>W16-1  –  W16-2</t>
-        </is>
-      </c>
-      <c r="E138" s="18" t="inlineStr"/>
-      <c r="F138" s="18" t="inlineStr"/>
-      <c r="G138" s="18" t="inlineStr"/>
-    </row>
-    <row r="139" ht="16" customHeight="1">
-      <c r="A139" s="61" t="inlineStr">
-        <is>
-          <t>W16-5  –  W16-6</t>
-        </is>
-      </c>
-      <c r="E139" s="18" t="inlineStr"/>
-      <c r="F139" s="18" t="inlineStr"/>
-      <c r="G139" s="18" t="inlineStr"/>
-    </row>
-    <row r="140" ht="16" customHeight="1">
-      <c r="A140" s="61" t="inlineStr">
-        <is>
-          <t>W16-3  –  W16-4</t>
-        </is>
-      </c>
-      <c r="E140" s="18" t="inlineStr"/>
-      <c r="F140" s="18" t="inlineStr"/>
-      <c r="G140" s="18" t="inlineStr"/>
+    <row r="140" ht="14" customHeight="1">
+      <c r="E140" s="13" t="inlineStr">
+        <is>
+          <t>voorsp.</t>
+        </is>
+      </c>
+      <c r="F140" s="13" t="inlineStr">
+        <is>
+          <t>uitslag</t>
+        </is>
+      </c>
+      <c r="G140" s="13" t="inlineStr">
+        <is>
+          <t>pt.</t>
+        </is>
+      </c>
     </row>
     <row r="141" ht="16" customHeight="1">
       <c r="A141" s="61" t="inlineStr">
         <is>
-          <t>W16-7  –  W16-8</t>
+          <t>W16-1  –  W16-2</t>
         </is>
       </c>
       <c r="E141" s="18" t="inlineStr"/>
       <c r="F141" s="18" t="inlineStr"/>
       <c r="G141" s="18" t="inlineStr"/>
     </row>
-    <row r="142" ht="6" customHeight="1"/>
+    <row r="142" ht="16" customHeight="1">
+      <c r="A142" s="61" t="inlineStr">
+        <is>
+          <t>W16-5  –  W16-6</t>
+        </is>
+      </c>
+      <c r="E142" s="18" t="inlineStr"/>
+      <c r="F142" s="18" t="inlineStr"/>
+      <c r="G142" s="18" t="inlineStr"/>
+    </row>
     <row r="143" ht="16" customHeight="1">
-      <c r="A143" s="10" t="inlineStr">
-        <is>
-          <t>Halve finales  ·  toto 11 pt / exact +6 pt</t>
-        </is>
-      </c>
+      <c r="A143" s="61" t="inlineStr">
+        <is>
+          <t>W16-3  –  W16-4</t>
+        </is>
+      </c>
+      <c r="E143" s="18" t="inlineStr"/>
+      <c r="F143" s="18" t="inlineStr"/>
+      <c r="G143" s="18" t="inlineStr"/>
     </row>
     <row r="144" ht="16" customHeight="1">
       <c r="A144" s="61" t="inlineStr">
         <is>
-          <t>WKF-1  –  WKF-2</t>
+          <t>W16-7  –  W16-8</t>
         </is>
       </c>
       <c r="E144" s="18" t="inlineStr"/>
       <c r="F144" s="18" t="inlineStr"/>
       <c r="G144" s="18" t="inlineStr"/>
     </row>
-    <row r="145" ht="16" customHeight="1">
-      <c r="A145" s="61" t="inlineStr">
-        <is>
-          <t>WKF-3  –  WKF-4</t>
-        </is>
-      </c>
-      <c r="E145" s="18" t="inlineStr"/>
-      <c r="F145" s="18" t="inlineStr"/>
-      <c r="G145" s="18" t="inlineStr"/>
-    </row>
-    <row r="146" ht="6" customHeight="1"/>
-    <row r="147" ht="16" customHeight="1">
-      <c r="A147" s="10" t="inlineStr">
-        <is>
-          <t>Finale  ·  toto 13 pt / exact +7 pt</t>
+    <row r="145" ht="6" customHeight="1"/>
+    <row r="146" ht="16" customHeight="1">
+      <c r="A146" s="10" t="inlineStr">
+        <is>
+          <t>Halve finales  ·  toto 11 pt / exact +6 pt</t>
+        </is>
+      </c>
+    </row>
+    <row r="147" ht="14" customHeight="1">
+      <c r="E147" s="13" t="inlineStr">
+        <is>
+          <t>voorsp.</t>
+        </is>
+      </c>
+      <c r="F147" s="13" t="inlineStr">
+        <is>
+          <t>uitslag</t>
+        </is>
+      </c>
+      <c r="G147" s="13" t="inlineStr">
+        <is>
+          <t>pt.</t>
         </is>
       </c>
     </row>
     <row r="148" ht="16" customHeight="1">
       <c r="A148" s="61" t="inlineStr">
         <is>
-          <t>WHF-1  –  WHF-2</t>
+          <t>WKF-1  –  WKF-2</t>
         </is>
       </c>
       <c r="E148" s="18" t="inlineStr"/>
       <c r="F148" s="18" t="inlineStr"/>
       <c r="G148" s="18" t="inlineStr"/>
     </row>
-    <row r="149" ht="6" customHeight="1"/>
-    <row r="150" ht="8" customHeight="1"/>
-    <row r="151" ht="18" customHeight="1">
-      <c r="A151" s="4" t="inlineStr">
+    <row r="149" ht="16" customHeight="1">
+      <c r="A149" s="61" t="inlineStr">
+        <is>
+          <t>WKF-3  –  WKF-4</t>
+        </is>
+      </c>
+      <c r="E149" s="18" t="inlineStr"/>
+      <c r="F149" s="18" t="inlineStr"/>
+      <c r="G149" s="18" t="inlineStr"/>
+    </row>
+    <row r="150" ht="6" customHeight="1"/>
+    <row r="151" ht="16" customHeight="1">
+      <c r="A151" s="10" t="inlineStr">
+        <is>
+          <t>Finale  ·  toto 13 pt / exact +7 pt</t>
+        </is>
+      </c>
+    </row>
+    <row r="152" ht="14" customHeight="1">
+      <c r="E152" s="13" t="inlineStr">
+        <is>
+          <t>voorsp.</t>
+        </is>
+      </c>
+      <c r="F152" s="13" t="inlineStr">
+        <is>
+          <t>uitslag</t>
+        </is>
+      </c>
+      <c r="G152" s="13" t="inlineStr">
+        <is>
+          <t>pt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="153" ht="16" customHeight="1">
+      <c r="A153" s="61" t="inlineStr">
+        <is>
+          <t>WHF-1  –  WHF-2</t>
+        </is>
+      </c>
+      <c r="E153" s="18" t="inlineStr"/>
+      <c r="F153" s="18" t="inlineStr"/>
+      <c r="G153" s="18" t="inlineStr"/>
+    </row>
+    <row r="154" ht="6" customHeight="1"/>
+    <row r="155" ht="8" customHeight="1"/>
+    <row r="156" ht="18" customHeight="1">
+      <c r="A156" s="4" t="inlineStr">
         <is>
           <t>▶  VERRASSING — kies een land BUITEN de top-12 · punten schalen met ranking en ronde</t>
         </is>
       </c>
     </row>
-    <row r="152" ht="14" customHeight="1">
-      <c r="A152" s="13" t="inlineStr">
+    <row r="157" ht="14" customHeight="1">
+      <c r="A157" s="13" t="inlineStr">
         <is>
           <t>Land (outsider)</t>
         </is>
       </c>
-      <c r="E152" s="13" t="inlineStr">
+      <c r="E157" s="13" t="inlineStr">
         <is>
           <t>R16</t>
         </is>
       </c>
-      <c r="F152" s="13" t="inlineStr">
+      <c r="F157" s="13" t="inlineStr">
         <is>
           <t>KF</t>
         </is>
       </c>
-      <c r="G152" s="13" t="inlineStr">
+      <c r="G157" s="13" t="inlineStr">
         <is>
           <t>HF</t>
         </is>
       </c>
-      <c r="H152" s="13" t="inlineStr">
+      <c r="H157" s="13" t="inlineStr">
         <is>
           <t>Finale</t>
         </is>
       </c>
-      <c r="I152" s="13" t="inlineStr">
+      <c r="I157" s="13" t="inlineStr">
         <is>
           <t>Winnaar</t>
         </is>
-      </c>
-    </row>
-    <row r="153" ht="15" customHeight="1">
-      <c r="A153" s="15" t="inlineStr">
-        <is>
-          <t>Senegal</t>
-        </is>
-      </c>
-      <c r="E153" s="62" t="n">
-        <v>7</v>
-      </c>
-      <c r="F153" s="62" t="n">
-        <v>12</v>
-      </c>
-      <c r="G153" s="62" t="n">
-        <v>19</v>
-      </c>
-      <c r="H153" s="62" t="n">
-        <v>26</v>
-      </c>
-      <c r="I153" s="62" t="n">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="154" ht="15" customHeight="1">
-      <c r="A154" s="15" t="inlineStr">
-        <is>
-          <t>Mexico</t>
-        </is>
-      </c>
-      <c r="E154" s="62" t="n">
-        <v>7</v>
-      </c>
-      <c r="F154" s="62" t="n">
-        <v>13</v>
-      </c>
-      <c r="G154" s="62" t="n">
-        <v>19</v>
-      </c>
-      <c r="H154" s="62" t="n">
-        <v>27</v>
-      </c>
-      <c r="I154" s="62" t="n">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="155" ht="15" customHeight="1">
-      <c r="A155" s="15" t="inlineStr">
-        <is>
-          <t>Verenigde Staten</t>
-        </is>
-      </c>
-      <c r="E155" s="62" t="n">
-        <v>8</v>
-      </c>
-      <c r="F155" s="62" t="n">
-        <v>13</v>
-      </c>
-      <c r="G155" s="62" t="n">
-        <v>20</v>
-      </c>
-      <c r="H155" s="62" t="n">
-        <v>27</v>
-      </c>
-      <c r="I155" s="62" t="n">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="156" ht="15" customHeight="1">
-      <c r="A156" s="15" t="inlineStr">
-        <is>
-          <t>Uruguay</t>
-        </is>
-      </c>
-      <c r="E156" s="62" t="n">
-        <v>8</v>
-      </c>
-      <c r="F156" s="62" t="n">
-        <v>14</v>
-      </c>
-      <c r="G156" s="62" t="n">
-        <v>20</v>
-      </c>
-      <c r="H156" s="62" t="n">
-        <v>28</v>
-      </c>
-      <c r="I156" s="62" t="n">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="157" ht="15" customHeight="1">
-      <c r="A157" s="15" t="inlineStr">
-        <is>
-          <t>Japan</t>
-        </is>
-      </c>
-      <c r="E157" s="62" t="n">
-        <v>8</v>
-      </c>
-      <c r="F157" s="62" t="n">
-        <v>14</v>
-      </c>
-      <c r="G157" s="62" t="n">
-        <v>21</v>
-      </c>
-      <c r="H157" s="62" t="n">
-        <v>29</v>
-      </c>
-      <c r="I157" s="62" t="n">
-        <v>38</v>
       </c>
     </row>
     <row r="158" ht="15" customHeight="1">
       <c r="A158" s="15" t="inlineStr">
         <is>
-          <t>Zwitserland</t>
+          <t>Senegal</t>
         </is>
       </c>
       <c r="E158" s="62" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F158" s="62" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G158" s="62" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="H158" s="62" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="I158" s="62" t="n">
-        <v>39</v>
+        <v>34</v>
       </c>
     </row>
     <row r="159" ht="15" customHeight="1">
       <c r="A159" s="15" t="inlineStr">
         <is>
-          <t>Iran</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="E159" s="62" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F159" s="62" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="G159" s="62" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="H159" s="62" t="n">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="I159" s="62" t="n">
-        <v>41</v>
+        <v>35</v>
       </c>
     </row>
     <row r="160" ht="15" customHeight="1">
       <c r="A160" s="15" t="inlineStr">
         <is>
-          <t>Oostenrijk</t>
+          <t>Verenigde Staten</t>
         </is>
       </c>
       <c r="E160" s="62" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F160" s="62" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="G160" s="62" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="H160" s="62" t="n">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="I160" s="62" t="n">
-        <v>42</v>
+        <v>36</v>
       </c>
     </row>
     <row r="161" ht="15" customHeight="1">
       <c r="A161" s="15" t="inlineStr">
         <is>
-          <t>Zuid-Korea</t>
+          <t>Uruguay</t>
         </is>
       </c>
       <c r="E161" s="62" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F161" s="62" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="G161" s="62" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="H161" s="62" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="I161" s="62" t="n">
-        <v>43</v>
+        <v>37</v>
       </c>
     </row>
     <row r="162" ht="15" customHeight="1">
       <c r="A162" s="15" t="inlineStr">
         <is>
-          <t>Australië</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="E162" s="62" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F162" s="62" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="G162" s="62" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="H162" s="62" t="n">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="I162" s="62" t="n">
-        <v>43</v>
+        <v>38</v>
       </c>
     </row>
     <row r="163" ht="15" customHeight="1">
       <c r="A163" s="15" t="inlineStr">
         <is>
-          <t>Ecuador</t>
+          <t>Zwitserland</t>
         </is>
       </c>
       <c r="E163" s="62" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F163" s="62" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="G163" s="62" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="H163" s="62" t="n">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="I163" s="62" t="n">
-        <v>44</v>
+        <v>39</v>
       </c>
     </row>
     <row r="164" ht="15" customHeight="1">
       <c r="A164" s="15" t="inlineStr">
         <is>
-          <t>Noorwegen</t>
+          <t>Iran</t>
         </is>
       </c>
       <c r="E164" s="62" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F164" s="62" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G164" s="62" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="H164" s="62" t="n">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="I164" s="62" t="n">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="165" ht="15" customHeight="1">
       <c r="A165" s="15" t="inlineStr">
         <is>
-          <t>Panama</t>
+          <t>Oostenrijk</t>
         </is>
       </c>
       <c r="E165" s="62" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F165" s="62" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="G165" s="62" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="H165" s="62" t="n">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="I165" s="62" t="n">
-        <v>48</v>
+        <v>42</v>
       </c>
     </row>
     <row r="166" ht="15" customHeight="1">
       <c r="A166" s="15" t="inlineStr">
         <is>
-          <t>Egypte</t>
+          <t>Zuid-Korea</t>
         </is>
       </c>
       <c r="E166" s="62" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F166" s="62" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="G166" s="62" t="n">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="H166" s="62" t="n">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="I166" s="62" t="n">
-        <v>49</v>
+        <v>43</v>
       </c>
     </row>
     <row r="167" ht="15" customHeight="1">
       <c r="A167" s="15" t="inlineStr">
         <is>
-          <t>Algerije</t>
+          <t>Australië</t>
         </is>
       </c>
       <c r="E167" s="62" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F167" s="62" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="G167" s="62" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="H167" s="62" t="n">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="I167" s="62" t="n">
-        <v>52</v>
+        <v>43</v>
       </c>
     </row>
     <row r="168" ht="15" customHeight="1">
       <c r="A168" s="15" t="inlineStr">
         <is>
-          <t>Paraguay</t>
+          <t>Ecuador</t>
         </is>
       </c>
       <c r="E168" s="62" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F168" s="62" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="G168" s="62" t="n">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="H168" s="62" t="n">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="I168" s="62" t="n">
-        <v>53</v>
+        <v>44</v>
       </c>
     </row>
     <row r="169" ht="15" customHeight="1">
       <c r="A169" s="15" t="inlineStr">
         <is>
-          <t>Ivoorkust</t>
+          <t>Noorwegen</t>
         </is>
       </c>
       <c r="E169" s="62" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F169" s="62" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="G169" s="62" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="H169" s="62" t="n">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="I169" s="62" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
     </row>
     <row r="170" ht="15" customHeight="1">
       <c r="A170" s="15" t="inlineStr">
         <is>
-          <t>Tunesië</t>
+          <t>Panama</t>
         </is>
       </c>
       <c r="E170" s="62" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F170" s="62" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="G170" s="62" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="H170" s="62" t="n">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="I170" s="62" t="n">
-        <v>55</v>
+        <v>48</v>
       </c>
     </row>
     <row r="171" ht="15" customHeight="1">
       <c r="A171" s="15" t="inlineStr">
         <is>
-          <t>Schotland</t>
+          <t>Egypte</t>
         </is>
       </c>
       <c r="E171" s="62" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F171" s="62" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G171" s="62" t="n">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="H171" s="62" t="n">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="I171" s="62" t="n">
-        <v>56</v>
+        <v>49</v>
       </c>
     </row>
     <row r="172" ht="15" customHeight="1">
       <c r="A172" s="15" t="inlineStr">
         <is>
-          <t>Zweden</t>
+          <t>Algerije</t>
         </is>
       </c>
       <c r="E172" s="62" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F172" s="62" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="G172" s="62" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="H172" s="62" t="n">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="I172" s="62" t="n">
-        <v>57</v>
+        <v>52</v>
       </c>
     </row>
     <row r="173" ht="15" customHeight="1">
       <c r="A173" s="15" t="inlineStr">
         <is>
-          <t>Tsjechië</t>
+          <t>Paraguay</t>
         </is>
       </c>
       <c r="E173" s="62" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F173" s="62" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="G173" s="62" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="H173" s="62" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="I173" s="62" t="n">
-        <v>57</v>
+        <v>53</v>
       </c>
     </row>
     <row r="174" ht="15" customHeight="1">
       <c r="A174" s="15" t="inlineStr">
         <is>
-          <t>Qatar</t>
+          <t>Ivoorkust</t>
         </is>
       </c>
       <c r="E174" s="62" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F174" s="62" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="G174" s="62" t="n">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="H174" s="62" t="n">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="I174" s="62" t="n">
-        <v>61</v>
+        <v>55</v>
       </c>
     </row>
     <row r="175" ht="15" customHeight="1">
       <c r="A175" s="15" t="inlineStr">
         <is>
-          <t>Oezbekistan</t>
+          <t>Tunesië</t>
         </is>
       </c>
       <c r="E175" s="62" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F175" s="62" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="G175" s="62" t="n">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="H175" s="62" t="n">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="I175" s="62" t="n">
-        <v>63</v>
+        <v>55</v>
       </c>
     </row>
     <row r="176" ht="15" customHeight="1">
       <c r="A176" s="15" t="inlineStr">
         <is>
-          <t>DR Congo</t>
+          <t>Schotland</t>
         </is>
       </c>
       <c r="E176" s="62" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F176" s="62" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="G176" s="62" t="n">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="H176" s="62" t="n">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="I176" s="62" t="n">
-        <v>64</v>
+        <v>56</v>
       </c>
     </row>
     <row r="177" ht="15" customHeight="1">
       <c r="A177" s="15" t="inlineStr">
         <is>
-          <t>Saoedi-Arabië</t>
+          <t>Zweden</t>
         </is>
       </c>
       <c r="E177" s="62" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F177" s="62" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="G177" s="62" t="n">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="H177" s="62" t="n">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="I177" s="62" t="n">
-        <v>65</v>
+        <v>57</v>
       </c>
     </row>
     <row r="178" ht="15" customHeight="1">
       <c r="A178" s="15" t="inlineStr">
         <is>
-          <t>Irak</t>
+          <t>Tsjechië</t>
         </is>
       </c>
       <c r="E178" s="62" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F178" s="62" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="G178" s="62" t="n">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="H178" s="62" t="n">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="I178" s="62" t="n">
-        <v>65</v>
+        <v>57</v>
       </c>
     </row>
     <row r="179" ht="15" customHeight="1">
       <c r="A179" s="15" t="inlineStr">
         <is>
-          <t>Zuid-Afrika</t>
+          <t>Qatar</t>
         </is>
       </c>
       <c r="E179" s="62" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F179" s="62" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="G179" s="62" t="n">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="H179" s="62" t="n">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="I179" s="62" t="n">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="180" ht="15" customHeight="1">
       <c r="A180" s="15" t="inlineStr">
         <is>
-          <t>Jordanië</t>
+          <t>Oezbekistan</t>
         </is>
       </c>
       <c r="E180" s="62" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F180" s="62" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="G180" s="62" t="n">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="H180" s="62" t="n">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="I180" s="62" t="n">
-        <v>68</v>
+        <v>63</v>
       </c>
     </row>
     <row r="181" ht="15" customHeight="1">
       <c r="A181" s="15" t="inlineStr">
         <is>
-          <t>Kaapverdië</t>
+          <t>DR Congo</t>
         </is>
       </c>
       <c r="E181" s="62" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F181" s="62" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="G181" s="62" t="n">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="H181" s="62" t="n">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="I181" s="62" t="n">
-        <v>70</v>
+        <v>64</v>
       </c>
     </row>
     <row r="182" ht="15" customHeight="1">
       <c r="A182" s="15" t="inlineStr">
         <is>
-          <t>Ghana</t>
+          <t>Saoedi-Arabië</t>
         </is>
       </c>
       <c r="E182" s="62" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F182" s="62" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="G182" s="62" t="n">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="H182" s="62" t="n">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="I182" s="62" t="n">
-        <v>72</v>
+        <v>65</v>
       </c>
     </row>
     <row r="183" ht="15" customHeight="1">
       <c r="A183" s="15" t="inlineStr">
         <is>
-          <t>Bosnië-Herzegovina</t>
+          <t>Irak</t>
         </is>
       </c>
       <c r="E183" s="62" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F183" s="62" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="G183" s="62" t="n">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="H183" s="62" t="n">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="I183" s="62" t="n">
-        <v>72</v>
+        <v>65</v>
       </c>
     </row>
     <row r="184" ht="15" customHeight="1">
       <c r="A184" s="15" t="inlineStr">
         <is>
-          <t>Haïti</t>
+          <t>Zuid-Afrika</t>
         </is>
       </c>
       <c r="E184" s="62" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F184" s="62" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="G184" s="62" t="n">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="H184" s="62" t="n">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="I184" s="62" t="n">
-        <v>76</v>
+        <v>66</v>
       </c>
     </row>
     <row r="185" ht="15" customHeight="1">
       <c r="A185" s="15" t="inlineStr">
         <is>
-          <t>Nieuw-Zeeland</t>
+          <t>Jordanië</t>
         </is>
       </c>
       <c r="E185" s="62" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F185" s="62" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="G185" s="62" t="n">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="H185" s="62" t="n">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="I185" s="62" t="n">
-        <v>77</v>
+        <v>68</v>
       </c>
     </row>
     <row r="186" ht="15" customHeight="1">
       <c r="A186" s="15" t="inlineStr">
         <is>
-          <t>Curaçao</t>
+          <t>Kaapverdië</t>
         </is>
       </c>
       <c r="E186" s="62" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F186" s="62" t="n">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="G186" s="62" t="n">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="H186" s="62" t="n">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="I186" s="62" t="n">
-        <v>79</v>
+        <v>70</v>
       </c>
     </row>
     <row r="187" ht="15" customHeight="1">
       <c r="A187" s="15" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Ghana</t>
         </is>
       </c>
       <c r="E187" s="62" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F187" s="62" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="G187" s="62" t="n">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="H187" s="62" t="n">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="I187" s="62" t="n">
-        <v>61</v>
+        <v>72</v>
       </c>
     </row>
     <row r="188" ht="15" customHeight="1">
       <c r="A188" s="15" t="inlineStr">
         <is>
-          <t>Turkije</t>
+          <t>Bosnië-Herzegovina</t>
         </is>
       </c>
       <c r="E188" s="62" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F188" s="62" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="G188" s="62" t="n">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="H188" s="62" t="n">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="I188" s="62" t="n">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="189" ht="8" customHeight="1"/>
-    <row r="190" ht="18" customHeight="1">
-      <c r="A190" s="4" t="inlineStr">
-        <is>
-          <t>▶  DECEPTIE — kies een land UIT de top-12 · punten schalen met ranking en uitvalsronde</t>
-        </is>
-      </c>
-    </row>
-    <row r="191" ht="14" customHeight="1">
-      <c r="A191" s="13" t="inlineStr">
-        <is>
-          <t>Land (favoriet)</t>
-        </is>
-      </c>
-      <c r="E191" s="13" t="inlineStr">
-        <is>
-          <t>KF</t>
-        </is>
-      </c>
-      <c r="F191" s="13" t="inlineStr">
-        <is>
-          <t>R16</t>
-        </is>
-      </c>
-      <c r="G191" s="13" t="inlineStr">
-        <is>
-          <t>R32</t>
-        </is>
-      </c>
-      <c r="H191" s="13" t="inlineStr">
-        <is>
-          <t>Groep eruit</t>
-        </is>
+        <v>72</v>
+      </c>
+    </row>
+    <row r="189" ht="15" customHeight="1">
+      <c r="A189" s="15" t="inlineStr">
+        <is>
+          <t>Haïti</t>
+        </is>
+      </c>
+      <c r="E189" s="62" t="n">
+        <v>16</v>
+      </c>
+      <c r="F189" s="62" t="n">
+        <v>28</v>
+      </c>
+      <c r="G189" s="62" t="n">
+        <v>41</v>
+      </c>
+      <c r="H189" s="62" t="n">
+        <v>58</v>
+      </c>
+      <c r="I189" s="62" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="190" ht="15" customHeight="1">
+      <c r="A190" s="15" t="inlineStr">
+        <is>
+          <t>Nieuw-Zeeland</t>
+        </is>
+      </c>
+      <c r="E190" s="62" t="n">
+        <v>16</v>
+      </c>
+      <c r="F190" s="62" t="n">
+        <v>28</v>
+      </c>
+      <c r="G190" s="62" t="n">
+        <v>42</v>
+      </c>
+      <c r="H190" s="62" t="n">
+        <v>59</v>
+      </c>
+      <c r="I190" s="62" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="191" ht="15" customHeight="1">
+      <c r="A191" s="15" t="inlineStr">
+        <is>
+          <t>Curaçao</t>
+        </is>
+      </c>
+      <c r="E191" s="62" t="n">
+        <v>17</v>
+      </c>
+      <c r="F191" s="62" t="n">
+        <v>29</v>
+      </c>
+      <c r="G191" s="62" t="n">
+        <v>43</v>
+      </c>
+      <c r="H191" s="62" t="n">
+        <v>60</v>
+      </c>
+      <c r="I191" s="62" t="n">
+        <v>79</v>
       </c>
     </row>
     <row r="192" ht="15" customHeight="1">
       <c r="A192" s="15" t="inlineStr">
         <is>
-          <t>Frankrijk</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="E192" s="62" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="F192" s="62" t="n">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="G192" s="62" t="n">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="H192" s="62" t="n">
-        <v>30</v>
+        <v>46</v>
+      </c>
+      <c r="I192" s="62" t="n">
+        <v>61</v>
       </c>
     </row>
     <row r="193" ht="15" customHeight="1">
       <c r="A193" s="15" t="inlineStr">
         <is>
-          <t>Spanje</t>
+          <t>Turkije</t>
         </is>
       </c>
       <c r="E193" s="62" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="F193" s="62" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="G193" s="62" t="n">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="H193" s="62" t="n">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="194" ht="15" customHeight="1">
-      <c r="A194" s="15" t="inlineStr">
-        <is>
-          <t>Argentinië</t>
-        </is>
-      </c>
-      <c r="E194" s="62" t="n">
-        <v>6</v>
-      </c>
-      <c r="F194" s="62" t="n">
-        <v>12</v>
-      </c>
-      <c r="G194" s="62" t="n">
-        <v>17</v>
-      </c>
-      <c r="H194" s="62" t="n">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="195" ht="15" customHeight="1">
-      <c r="A195" s="15" t="inlineStr">
-        <is>
-          <t>Engeland</t>
-        </is>
-      </c>
-      <c r="E195" s="62" t="n">
-        <v>6</v>
-      </c>
-      <c r="F195" s="62" t="n">
-        <v>11</v>
-      </c>
-      <c r="G195" s="62" t="n">
-        <v>16</v>
-      </c>
-      <c r="H195" s="62" t="n">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="196" ht="15" customHeight="1">
-      <c r="A196" s="15" t="inlineStr">
-        <is>
-          <t>Portugal</t>
-        </is>
-      </c>
-      <c r="E196" s="62" t="n">
-        <v>6</v>
-      </c>
-      <c r="F196" s="62" t="n">
-        <v>10</v>
-      </c>
-      <c r="G196" s="62" t="n">
-        <v>15</v>
-      </c>
-      <c r="H196" s="62" t="n">
-        <v>22</v>
+        <v>46</v>
+      </c>
+      <c r="I193" s="62" t="n">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="194" ht="8" customHeight="1"/>
+    <row r="195" ht="18" customHeight="1">
+      <c r="A195" s="4" t="inlineStr">
+        <is>
+          <t>▶  DECEPTIE — kies een land UIT de top-12 · punten schalen met ranking en uitvalsronde</t>
+        </is>
+      </c>
+    </row>
+    <row r="196" ht="14" customHeight="1">
+      <c r="A196" s="13" t="inlineStr">
+        <is>
+          <t>Land (favoriet)</t>
+        </is>
+      </c>
+      <c r="E196" s="13" t="inlineStr">
+        <is>
+          <t>KF</t>
+        </is>
+      </c>
+      <c r="F196" s="13" t="inlineStr">
+        <is>
+          <t>R16</t>
+        </is>
+      </c>
+      <c r="G196" s="13" t="inlineStr">
+        <is>
+          <t>R32</t>
+        </is>
+      </c>
+      <c r="H196" s="13" t="inlineStr">
+        <is>
+          <t>Groep eruit</t>
+        </is>
       </c>
     </row>
     <row r="197" ht="15" customHeight="1">
       <c r="A197" s="15" t="inlineStr">
         <is>
-          <t>Brazilië</t>
+          <t>Frankrijk</t>
         </is>
       </c>
       <c r="E197" s="62" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F197" s="62" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="G197" s="62" t="n">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="H197" s="62" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
     </row>
     <row r="198" ht="15" customHeight="1">
       <c r="A198" s="15" t="inlineStr">
         <is>
-          <t>Nederland</t>
+          <t>Spanje</t>
         </is>
       </c>
       <c r="E198" s="62" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="F198" s="62" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="G198" s="62" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="H198" s="62" t="n">
-        <v>18</v>
+        <v>28</v>
       </c>
     </row>
     <row r="199" ht="15" customHeight="1">
       <c r="A199" s="15" t="inlineStr">
         <is>
-          <t>Marokko</t>
+          <t>Argentinië</t>
         </is>
       </c>
       <c r="E199" s="62" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F199" s="62" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="G199" s="62" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="H199" s="62" t="n">
-        <v>16</v>
+        <v>26</v>
       </c>
     </row>
     <row r="200" ht="15" customHeight="1">
       <c r="A200" s="15" t="inlineStr">
         <is>
-          <t>België</t>
+          <t>Engeland</t>
         </is>
       </c>
       <c r="E200" s="62" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F200" s="62" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="G200" s="62" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="H200" s="62" t="n">
-        <v>14</v>
+        <v>24</v>
       </c>
     </row>
     <row r="201" ht="15" customHeight="1">
       <c r="A201" s="15" t="inlineStr">
         <is>
-          <t>Duitsland</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="E201" s="62" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F201" s="62" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G201" s="62" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="H201" s="62" t="n">
-        <v>12</v>
+        <v>22</v>
       </c>
     </row>
     <row r="202" ht="15" customHeight="1">
       <c r="A202" s="15" t="inlineStr">
         <is>
-          <t>Kroatië</t>
+          <t>Brazilië</t>
         </is>
       </c>
       <c r="E202" s="62" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F202" s="62" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="G202" s="62" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="H202" s="62" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="203" ht="15" customHeight="1">
       <c r="A203" s="15" t="inlineStr">
         <is>
+          <t>Nederland</t>
+        </is>
+      </c>
+      <c r="E203" s="62" t="n">
+        <v>4</v>
+      </c>
+      <c r="F203" s="62" t="n">
+        <v>8</v>
+      </c>
+      <c r="G203" s="62" t="n">
+        <v>12</v>
+      </c>
+      <c r="H203" s="62" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="204" ht="15" customHeight="1">
+      <c r="A204" s="15" t="inlineStr">
+        <is>
+          <t>Marokko</t>
+        </is>
+      </c>
+      <c r="E204" s="62" t="n">
+        <v>4</v>
+      </c>
+      <c r="F204" s="62" t="n">
+        <v>7</v>
+      </c>
+      <c r="G204" s="62" t="n">
+        <v>11</v>
+      </c>
+      <c r="H204" s="62" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="205" ht="15" customHeight="1">
+      <c r="A205" s="15" t="inlineStr">
+        <is>
+          <t>België</t>
+        </is>
+      </c>
+      <c r="E205" s="62" t="n">
+        <v>4</v>
+      </c>
+      <c r="F205" s="62" t="n">
+        <v>6</v>
+      </c>
+      <c r="G205" s="62" t="n">
+        <v>9</v>
+      </c>
+      <c r="H205" s="62" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="206" ht="15" customHeight="1">
+      <c r="A206" s="15" t="inlineStr">
+        <is>
+          <t>Duitsland</t>
+        </is>
+      </c>
+      <c r="E206" s="62" t="n">
+        <v>3</v>
+      </c>
+      <c r="F206" s="62" t="n">
+        <v>6</v>
+      </c>
+      <c r="G206" s="62" t="n">
+        <v>8</v>
+      </c>
+      <c r="H206" s="62" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="207" ht="15" customHeight="1">
+      <c r="A207" s="15" t="inlineStr">
+        <is>
+          <t>Kroatië</t>
+        </is>
+      </c>
+      <c r="E207" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="F207" s="62" t="n">
+        <v>5</v>
+      </c>
+      <c r="G207" s="62" t="n">
+        <v>7</v>
+      </c>
+      <c r="H207" s="62" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="208" ht="15" customHeight="1">
+      <c r="A208" s="15" t="inlineStr">
+        <is>
           <t>Colombia</t>
         </is>
       </c>
-      <c r="E203" s="62" t="n">
+      <c r="E208" s="62" t="n">
         <v>2</v>
       </c>
-      <c r="F203" s="62" t="n">
+      <c r="F208" s="62" t="n">
         <v>3</v>
       </c>
-      <c r="G203" s="62" t="n">
+      <c r="G208" s="62" t="n">
         <v>4</v>
       </c>
-      <c r="H203" s="62" t="n">
+      <c r="H208" s="62" t="n">
         <v>6</v>
       </c>
     </row>
@@ -4957,7 +5042,6 @@
     <mergeCell ref="A200:D200"/>
     <mergeCell ref="A81:D81"/>
     <mergeCell ref="A112:D112"/>
-    <mergeCell ref="A152:D152"/>
     <mergeCell ref="A121:D121"/>
     <mergeCell ref="M81:O81"/>
     <mergeCell ref="A161:D161"/>
@@ -4989,21 +5073,25 @@
     <mergeCell ref="A164:D164"/>
     <mergeCell ref="A15:O15"/>
     <mergeCell ref="A24:O24"/>
-    <mergeCell ref="A154:D154"/>
+    <mergeCell ref="A149:D149"/>
     <mergeCell ref="M52:O52"/>
     <mergeCell ref="A163:D163"/>
     <mergeCell ref="A101:D101"/>
     <mergeCell ref="E92:G92"/>
-    <mergeCell ref="A195:D195"/>
+    <mergeCell ref="A204:D204"/>
+    <mergeCell ref="A146:O146"/>
     <mergeCell ref="I52:L52"/>
     <mergeCell ref="A188:D188"/>
+    <mergeCell ref="A126:D126"/>
     <mergeCell ref="A141:D141"/>
     <mergeCell ref="A16:O16"/>
     <mergeCell ref="A135:D135"/>
+    <mergeCell ref="A206:D206"/>
     <mergeCell ref="I44:L44"/>
     <mergeCell ref="A62:D62"/>
     <mergeCell ref="A108:O108"/>
     <mergeCell ref="A125:D125"/>
+    <mergeCell ref="A190:D190"/>
     <mergeCell ref="A18:O18"/>
     <mergeCell ref="I94:L94"/>
     <mergeCell ref="A117:D117"/>
@@ -5015,6 +5103,7 @@
     <mergeCell ref="A167:D167"/>
     <mergeCell ref="A151:O151"/>
     <mergeCell ref="E61:G61"/>
+    <mergeCell ref="A142:D142"/>
     <mergeCell ref="A11:D11"/>
     <mergeCell ref="A22:O22"/>
     <mergeCell ref="A182:D182"/>
@@ -5024,41 +5113,35 @@
     <mergeCell ref="I61:L61"/>
     <mergeCell ref="E72:G72"/>
     <mergeCell ref="A61:D61"/>
-    <mergeCell ref="A190:O190"/>
     <mergeCell ref="A28:O28"/>
     <mergeCell ref="A153:D153"/>
     <mergeCell ref="A162:D162"/>
     <mergeCell ref="M71:O71"/>
     <mergeCell ref="I54:L54"/>
-    <mergeCell ref="A128:D128"/>
     <mergeCell ref="I72:L72"/>
-    <mergeCell ref="A127:O127"/>
+    <mergeCell ref="A137:D137"/>
     <mergeCell ref="A177:D177"/>
+    <mergeCell ref="A208:D208"/>
     <mergeCell ref="A30:O30"/>
     <mergeCell ref="E71:G71"/>
+    <mergeCell ref="A136:D136"/>
     <mergeCell ref="A192:D192"/>
     <mergeCell ref="I71:L71"/>
     <mergeCell ref="A74:D74"/>
-    <mergeCell ref="A145:D145"/>
-    <mergeCell ref="A139:D139"/>
     <mergeCell ref="E8:G8"/>
     <mergeCell ref="G1:K1"/>
     <mergeCell ref="A179:D179"/>
     <mergeCell ref="A71:D71"/>
     <mergeCell ref="E82:G82"/>
-    <mergeCell ref="A129:D129"/>
-    <mergeCell ref="A194:D194"/>
     <mergeCell ref="A203:D203"/>
     <mergeCell ref="A116:D116"/>
     <mergeCell ref="A181:D181"/>
     <mergeCell ref="E10:G10"/>
     <mergeCell ref="A8:D8"/>
     <mergeCell ref="A91:D91"/>
-    <mergeCell ref="A137:O137"/>
+    <mergeCell ref="A184:D184"/>
     <mergeCell ref="A131:D131"/>
     <mergeCell ref="I82:L82"/>
-    <mergeCell ref="A184:D184"/>
-    <mergeCell ref="A140:D140"/>
     <mergeCell ref="A171:D171"/>
     <mergeCell ref="A52:D52"/>
     <mergeCell ref="A165:D165"/>
@@ -5067,12 +5150,14 @@
     <mergeCell ref="B31:O31"/>
     <mergeCell ref="A10:D10"/>
     <mergeCell ref="A115:D115"/>
-    <mergeCell ref="A155:D155"/>
+    <mergeCell ref="A139:O139"/>
     <mergeCell ref="A102:D102"/>
     <mergeCell ref="A173:D173"/>
     <mergeCell ref="E11:G11"/>
     <mergeCell ref="I74:L74"/>
     <mergeCell ref="B39:O39"/>
+    <mergeCell ref="A195:O195"/>
+    <mergeCell ref="A143:D143"/>
     <mergeCell ref="A92:D92"/>
     <mergeCell ref="A157:D157"/>
     <mergeCell ref="A166:D166"/>
@@ -5080,15 +5165,16 @@
     <mergeCell ref="A17:O17"/>
     <mergeCell ref="B23:O23"/>
     <mergeCell ref="M62:O62"/>
+    <mergeCell ref="A207:D207"/>
     <mergeCell ref="A109:O109"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A94:D94"/>
     <mergeCell ref="A168:D168"/>
     <mergeCell ref="E102:G102"/>
     <mergeCell ref="A19:O19"/>
+    <mergeCell ref="A205:D205"/>
     <mergeCell ref="A34:O34"/>
     <mergeCell ref="A133:D133"/>
-    <mergeCell ref="A143:O143"/>
     <mergeCell ref="A193:D193"/>
     <mergeCell ref="E62:G62"/>
     <mergeCell ref="A120:D120"/>
@@ -5102,8 +5188,8 @@
     <mergeCell ref="A185:D185"/>
     <mergeCell ref="I64:L64"/>
     <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A128:O128"/>
     <mergeCell ref="I51:L51"/>
-    <mergeCell ref="A156:D156"/>
     <mergeCell ref="A170:D170"/>
     <mergeCell ref="A21:O21"/>
     <mergeCell ref="A105:O105"/>
@@ -5118,12 +5204,10 @@
     <mergeCell ref="M91:O91"/>
     <mergeCell ref="E91:G91"/>
     <mergeCell ref="A123:D123"/>
-    <mergeCell ref="A138:D138"/>
-    <mergeCell ref="A147:O147"/>
     <mergeCell ref="A132:D132"/>
     <mergeCell ref="A197:D197"/>
-    <mergeCell ref="A110:D110"/>
     <mergeCell ref="A43:O43"/>
+    <mergeCell ref="A156:O156"/>
     <mergeCell ref="I101:L101"/>
     <mergeCell ref="A6:D6"/>
     <mergeCell ref="A119:D119"/>
@@ -5136,6 +5220,7 @@
     <mergeCell ref="A84:D84"/>
     <mergeCell ref="M92:O92"/>
     <mergeCell ref="A118:D118"/>
+    <mergeCell ref="A189:D189"/>
     <mergeCell ref="A158:D158"/>
     <mergeCell ref="E52:G52"/>
     <mergeCell ref="I102:L102"/>

</xml_diff>

<commit_message>
Invulformulier: KO koptekstrij volledig gevuld, voorsp/uitslag/pt niet meer weggedrukt
</commit_message>
<xml_diff>
--- a/tempetoto2026_invulformulier.xlsx
+++ b/tempetoto2026_invulformulier.xlsx
@@ -421,7 +421,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
@@ -514,6 +514,7 @@
     <xf numFmtId="0" fontId="12" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="8" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -3521,6 +3522,11 @@
       </c>
     </row>
     <row r="115" ht="14" customHeight="1">
+      <c r="A115" s="12" t="inlineStr">
+        <is>
+          <t>Wedstrijd</t>
+        </is>
+      </c>
       <c r="E115" s="12" t="inlineStr">
         <is>
           <t>voorsp.</t>
@@ -3536,9 +3542,17 @@
           <t>pt.</t>
         </is>
       </c>
+      <c r="H115" s="60" t="n"/>
+      <c r="I115" s="60" t="n"/>
+      <c r="J115" s="60" t="n"/>
+      <c r="K115" s="60" t="n"/>
+      <c r="L115" s="60" t="n"/>
+      <c r="M115" s="60" t="n"/>
+      <c r="N115" s="60" t="n"/>
+      <c r="O115" s="60" t="n"/>
     </row>
     <row r="116" ht="16" customHeight="1">
-      <c r="A116" s="60" t="inlineStr">
+      <c r="A116" s="61" t="inlineStr">
         <is>
           <t>2A  –  2B</t>
         </is>
@@ -3548,7 +3562,7 @@
       <c r="G116" s="17" t="inlineStr"/>
     </row>
     <row r="117" ht="16" customHeight="1">
-      <c r="A117" s="60" t="inlineStr">
+      <c r="A117" s="61" t="inlineStr">
         <is>
           <t>1E  –  3e (A/B/C/D/F)</t>
         </is>
@@ -3558,7 +3572,7 @@
       <c r="G117" s="17" t="inlineStr"/>
     </row>
     <row r="118" ht="16" customHeight="1">
-      <c r="A118" s="60" t="inlineStr">
+      <c r="A118" s="61" t="inlineStr">
         <is>
           <t>1F  –  2C</t>
         </is>
@@ -3568,7 +3582,7 @@
       <c r="G118" s="17" t="inlineStr"/>
     </row>
     <row r="119" ht="16" customHeight="1">
-      <c r="A119" s="60" t="inlineStr">
+      <c r="A119" s="61" t="inlineStr">
         <is>
           <t>1C  –  2F</t>
         </is>
@@ -3578,7 +3592,7 @@
       <c r="G119" s="17" t="inlineStr"/>
     </row>
     <row r="120" ht="16" customHeight="1">
-      <c r="A120" s="60" t="inlineStr">
+      <c r="A120" s="61" t="inlineStr">
         <is>
           <t>1I  –  3e (C/D/F/G/H)</t>
         </is>
@@ -3588,7 +3602,7 @@
       <c r="G120" s="17" t="inlineStr"/>
     </row>
     <row r="121" ht="16" customHeight="1">
-      <c r="A121" s="60" t="inlineStr">
+      <c r="A121" s="61" t="inlineStr">
         <is>
           <t>2E  –  2I</t>
         </is>
@@ -3598,7 +3612,7 @@
       <c r="G121" s="17" t="inlineStr"/>
     </row>
     <row r="122" ht="16" customHeight="1">
-      <c r="A122" s="60" t="inlineStr">
+      <c r="A122" s="61" t="inlineStr">
         <is>
           <t>1A  –  3e (C/E/F/H/I)</t>
         </is>
@@ -3608,7 +3622,7 @@
       <c r="G122" s="17" t="inlineStr"/>
     </row>
     <row r="123" ht="16" customHeight="1">
-      <c r="A123" s="60" t="inlineStr">
+      <c r="A123" s="61" t="inlineStr">
         <is>
           <t>1L  –  3e (E/H/I/J/K)</t>
         </is>
@@ -3618,7 +3632,7 @@
       <c r="G123" s="17" t="inlineStr"/>
     </row>
     <row r="124" ht="16" customHeight="1">
-      <c r="A124" s="60" t="inlineStr">
+      <c r="A124" s="61" t="inlineStr">
         <is>
           <t>1D  –  3e (B/E/F/I/J)</t>
         </is>
@@ -3628,7 +3642,7 @@
       <c r="G124" s="17" t="inlineStr"/>
     </row>
     <row r="125" ht="16" customHeight="1">
-      <c r="A125" s="60" t="inlineStr">
+      <c r="A125" s="61" t="inlineStr">
         <is>
           <t>1G  –  3e (A/E/H/I/J)</t>
         </is>
@@ -3638,7 +3652,7 @@
       <c r="G125" s="17" t="inlineStr"/>
     </row>
     <row r="126" ht="16" customHeight="1">
-      <c r="A126" s="60" t="inlineStr">
+      <c r="A126" s="61" t="inlineStr">
         <is>
           <t>2K  –  2L</t>
         </is>
@@ -3648,7 +3662,7 @@
       <c r="G126" s="17" t="inlineStr"/>
     </row>
     <row r="127" ht="16" customHeight="1">
-      <c r="A127" s="60" t="inlineStr">
+      <c r="A127" s="61" t="inlineStr">
         <is>
           <t>1H  –  2J</t>
         </is>
@@ -3658,7 +3672,7 @@
       <c r="G127" s="17" t="inlineStr"/>
     </row>
     <row r="128" ht="16" customHeight="1">
-      <c r="A128" s="60" t="inlineStr">
+      <c r="A128" s="61" t="inlineStr">
         <is>
           <t>1B  –  3e (E/F/G/I/J)</t>
         </is>
@@ -3668,7 +3682,7 @@
       <c r="G128" s="17" t="inlineStr"/>
     </row>
     <row r="129" ht="16" customHeight="1">
-      <c r="A129" s="60" t="inlineStr">
+      <c r="A129" s="61" t="inlineStr">
         <is>
           <t>1J  –  2H</t>
         </is>
@@ -3678,7 +3692,7 @@
       <c r="G129" s="17" t="inlineStr"/>
     </row>
     <row r="130" ht="16" customHeight="1">
-      <c r="A130" s="60" t="inlineStr">
+      <c r="A130" s="61" t="inlineStr">
         <is>
           <t>1K  –  3e (D/E/I/J/L)</t>
         </is>
@@ -3688,7 +3702,7 @@
       <c r="G130" s="17" t="inlineStr"/>
     </row>
     <row r="131" ht="16" customHeight="1">
-      <c r="A131" s="60" t="inlineStr">
+      <c r="A131" s="61" t="inlineStr">
         <is>
           <t>2D  –  2G</t>
         </is>
@@ -3706,6 +3720,11 @@
       </c>
     </row>
     <row r="134" ht="14" customHeight="1">
+      <c r="A134" s="12" t="inlineStr">
+        <is>
+          <t>Wedstrijd</t>
+        </is>
+      </c>
       <c r="E134" s="12" t="inlineStr">
         <is>
           <t>voorsp.</t>
@@ -3721,9 +3740,17 @@
           <t>pt.</t>
         </is>
       </c>
+      <c r="H134" s="60" t="n"/>
+      <c r="I134" s="60" t="n"/>
+      <c r="J134" s="60" t="n"/>
+      <c r="K134" s="60" t="n"/>
+      <c r="L134" s="60" t="n"/>
+      <c r="M134" s="60" t="n"/>
+      <c r="N134" s="60" t="n"/>
+      <c r="O134" s="60" t="n"/>
     </row>
     <row r="135" ht="16" customHeight="1">
-      <c r="A135" s="60" t="inlineStr">
+      <c r="A135" s="61" t="inlineStr">
         <is>
           <t>W32-2  –  W32-5</t>
         </is>
@@ -3733,7 +3760,7 @@
       <c r="G135" s="17" t="inlineStr"/>
     </row>
     <row r="136" ht="16" customHeight="1">
-      <c r="A136" s="60" t="inlineStr">
+      <c r="A136" s="61" t="inlineStr">
         <is>
           <t>W32-1  –  W32-3</t>
         </is>
@@ -3743,7 +3770,7 @@
       <c r="G136" s="17" t="inlineStr"/>
     </row>
     <row r="137" ht="16" customHeight="1">
-      <c r="A137" s="60" t="inlineStr">
+      <c r="A137" s="61" t="inlineStr">
         <is>
           <t>W32-4  –  W32-6</t>
         </is>
@@ -3753,7 +3780,7 @@
       <c r="G137" s="17" t="inlineStr"/>
     </row>
     <row r="138" ht="16" customHeight="1">
-      <c r="A138" s="60" t="inlineStr">
+      <c r="A138" s="61" t="inlineStr">
         <is>
           <t>W32-7  –  W32-8</t>
         </is>
@@ -3763,7 +3790,7 @@
       <c r="G138" s="17" t="inlineStr"/>
     </row>
     <row r="139" ht="16" customHeight="1">
-      <c r="A139" s="60" t="inlineStr">
+      <c r="A139" s="61" t="inlineStr">
         <is>
           <t>W32-11  –  W32-12</t>
         </is>
@@ -3773,7 +3800,7 @@
       <c r="G139" s="17" t="inlineStr"/>
     </row>
     <row r="140" ht="16" customHeight="1">
-      <c r="A140" s="60" t="inlineStr">
+      <c r="A140" s="61" t="inlineStr">
         <is>
           <t>W32-9  –  W32-10</t>
         </is>
@@ -3783,7 +3810,7 @@
       <c r="G140" s="17" t="inlineStr"/>
     </row>
     <row r="141" ht="16" customHeight="1">
-      <c r="A141" s="60" t="inlineStr">
+      <c r="A141" s="61" t="inlineStr">
         <is>
           <t>W32-14  –  W32-16</t>
         </is>
@@ -3793,7 +3820,7 @@
       <c r="G141" s="17" t="inlineStr"/>
     </row>
     <row r="142" ht="16" customHeight="1">
-      <c r="A142" s="60" t="inlineStr">
+      <c r="A142" s="61" t="inlineStr">
         <is>
           <t>W32-13  –  W32-15</t>
         </is>
@@ -3811,6 +3838,11 @@
       </c>
     </row>
     <row r="145" ht="14" customHeight="1">
+      <c r="A145" s="12" t="inlineStr">
+        <is>
+          <t>Wedstrijd</t>
+        </is>
+      </c>
       <c r="E145" s="12" t="inlineStr">
         <is>
           <t>voorsp.</t>
@@ -3826,9 +3858,17 @@
           <t>pt.</t>
         </is>
       </c>
+      <c r="H145" s="60" t="n"/>
+      <c r="I145" s="60" t="n"/>
+      <c r="J145" s="60" t="n"/>
+      <c r="K145" s="60" t="n"/>
+      <c r="L145" s="60" t="n"/>
+      <c r="M145" s="60" t="n"/>
+      <c r="N145" s="60" t="n"/>
+      <c r="O145" s="60" t="n"/>
     </row>
     <row r="146" ht="16" customHeight="1">
-      <c r="A146" s="60" t="inlineStr">
+      <c r="A146" s="61" t="inlineStr">
         <is>
           <t>W16-1  –  W16-2</t>
         </is>
@@ -3838,7 +3878,7 @@
       <c r="G146" s="17" t="inlineStr"/>
     </row>
     <row r="147" ht="16" customHeight="1">
-      <c r="A147" s="60" t="inlineStr">
+      <c r="A147" s="61" t="inlineStr">
         <is>
           <t>W16-5  –  W16-6</t>
         </is>
@@ -3848,7 +3888,7 @@
       <c r="G147" s="17" t="inlineStr"/>
     </row>
     <row r="148" ht="16" customHeight="1">
-      <c r="A148" s="60" t="inlineStr">
+      <c r="A148" s="61" t="inlineStr">
         <is>
           <t>W16-3  –  W16-4</t>
         </is>
@@ -3858,7 +3898,7 @@
       <c r="G148" s="17" t="inlineStr"/>
     </row>
     <row r="149" ht="16" customHeight="1">
-      <c r="A149" s="60" t="inlineStr">
+      <c r="A149" s="61" t="inlineStr">
         <is>
           <t>W16-7  –  W16-8</t>
         </is>
@@ -3876,6 +3916,11 @@
       </c>
     </row>
     <row r="152" ht="14" customHeight="1">
+      <c r="A152" s="12" t="inlineStr">
+        <is>
+          <t>Wedstrijd</t>
+        </is>
+      </c>
       <c r="E152" s="12" t="inlineStr">
         <is>
           <t>voorsp.</t>
@@ -3891,9 +3936,17 @@
           <t>pt.</t>
         </is>
       </c>
+      <c r="H152" s="60" t="n"/>
+      <c r="I152" s="60" t="n"/>
+      <c r="J152" s="60" t="n"/>
+      <c r="K152" s="60" t="n"/>
+      <c r="L152" s="60" t="n"/>
+      <c r="M152" s="60" t="n"/>
+      <c r="N152" s="60" t="n"/>
+      <c r="O152" s="60" t="n"/>
     </row>
     <row r="153" ht="16" customHeight="1">
-      <c r="A153" s="60" t="inlineStr">
+      <c r="A153" s="61" t="inlineStr">
         <is>
           <t>WKF-1  –  WKF-2</t>
         </is>
@@ -3903,7 +3956,7 @@
       <c r="G153" s="17" t="inlineStr"/>
     </row>
     <row r="154" ht="16" customHeight="1">
-      <c r="A154" s="60" t="inlineStr">
+      <c r="A154" s="61" t="inlineStr">
         <is>
           <t>WKF-3  –  WKF-4</t>
         </is>
@@ -3921,6 +3974,11 @@
       </c>
     </row>
     <row r="157" ht="14" customHeight="1">
+      <c r="A157" s="12" t="inlineStr">
+        <is>
+          <t>Wedstrijd</t>
+        </is>
+      </c>
       <c r="E157" s="12" t="inlineStr">
         <is>
           <t>voorsp.</t>
@@ -3936,9 +3994,17 @@
           <t>pt.</t>
         </is>
       </c>
+      <c r="H157" s="60" t="n"/>
+      <c r="I157" s="60" t="n"/>
+      <c r="J157" s="60" t="n"/>
+      <c r="K157" s="60" t="n"/>
+      <c r="L157" s="60" t="n"/>
+      <c r="M157" s="60" t="n"/>
+      <c r="N157" s="60" t="n"/>
+      <c r="O157" s="60" t="n"/>
     </row>
     <row r="158" ht="16" customHeight="1">
-      <c r="A158" s="60" t="inlineStr">
+      <c r="A158" s="61" t="inlineStr">
         <is>
           <t>WHF-1  –  WHF-2</t>
         </is>
@@ -3994,19 +4060,19 @@
           <t>Senegal</t>
         </is>
       </c>
-      <c r="E163" s="61" t="n">
+      <c r="E163" s="62" t="n">
         <v>7</v>
       </c>
-      <c r="F163" s="61" t="n">
+      <c r="F163" s="62" t="n">
         <v>12</v>
       </c>
-      <c r="G163" s="61" t="n">
+      <c r="G163" s="62" t="n">
         <v>19</v>
       </c>
-      <c r="H163" s="61" t="n">
+      <c r="H163" s="62" t="n">
         <v>26</v>
       </c>
-      <c r="I163" s="61" t="n">
+      <c r="I163" s="62" t="n">
         <v>34</v>
       </c>
     </row>
@@ -4016,19 +4082,19 @@
           <t>Mexico</t>
         </is>
       </c>
-      <c r="E164" s="61" t="n">
+      <c r="E164" s="62" t="n">
         <v>7</v>
       </c>
-      <c r="F164" s="61" t="n">
+      <c r="F164" s="62" t="n">
         <v>13</v>
       </c>
-      <c r="G164" s="61" t="n">
+      <c r="G164" s="62" t="n">
         <v>19</v>
       </c>
-      <c r="H164" s="61" t="n">
+      <c r="H164" s="62" t="n">
         <v>27</v>
       </c>
-      <c r="I164" s="61" t="n">
+      <c r="I164" s="62" t="n">
         <v>35</v>
       </c>
     </row>
@@ -4038,19 +4104,19 @@
           <t>Verenigde Staten</t>
         </is>
       </c>
-      <c r="E165" s="61" t="n">
+      <c r="E165" s="62" t="n">
         <v>8</v>
       </c>
-      <c r="F165" s="61" t="n">
+      <c r="F165" s="62" t="n">
         <v>13</v>
       </c>
-      <c r="G165" s="61" t="n">
+      <c r="G165" s="62" t="n">
         <v>20</v>
       </c>
-      <c r="H165" s="61" t="n">
+      <c r="H165" s="62" t="n">
         <v>27</v>
       </c>
-      <c r="I165" s="61" t="n">
+      <c r="I165" s="62" t="n">
         <v>36</v>
       </c>
     </row>
@@ -4060,19 +4126,19 @@
           <t>Uruguay</t>
         </is>
       </c>
-      <c r="E166" s="61" t="n">
+      <c r="E166" s="62" t="n">
         <v>8</v>
       </c>
-      <c r="F166" s="61" t="n">
+      <c r="F166" s="62" t="n">
         <v>14</v>
       </c>
-      <c r="G166" s="61" t="n">
+      <c r="G166" s="62" t="n">
         <v>20</v>
       </c>
-      <c r="H166" s="61" t="n">
+      <c r="H166" s="62" t="n">
         <v>28</v>
       </c>
-      <c r="I166" s="61" t="n">
+      <c r="I166" s="62" t="n">
         <v>37</v>
       </c>
     </row>
@@ -4082,19 +4148,19 @@
           <t>Japan</t>
         </is>
       </c>
-      <c r="E167" s="61" t="n">
+      <c r="E167" s="62" t="n">
         <v>8</v>
       </c>
-      <c r="F167" s="61" t="n">
+      <c r="F167" s="62" t="n">
         <v>14</v>
       </c>
-      <c r="G167" s="61" t="n">
+      <c r="G167" s="62" t="n">
         <v>21</v>
       </c>
-      <c r="H167" s="61" t="n">
+      <c r="H167" s="62" t="n">
         <v>29</v>
       </c>
-      <c r="I167" s="61" t="n">
+      <c r="I167" s="62" t="n">
         <v>38</v>
       </c>
     </row>
@@ -4104,19 +4170,19 @@
           <t>Zwitserland</t>
         </is>
       </c>
-      <c r="E168" s="61" t="n">
+      <c r="E168" s="62" t="n">
         <v>8</v>
       </c>
-      <c r="F168" s="61" t="n">
+      <c r="F168" s="62" t="n">
         <v>14</v>
       </c>
-      <c r="G168" s="61" t="n">
+      <c r="G168" s="62" t="n">
         <v>21</v>
       </c>
-      <c r="H168" s="61" t="n">
+      <c r="H168" s="62" t="n">
         <v>30</v>
       </c>
-      <c r="I168" s="61" t="n">
+      <c r="I168" s="62" t="n">
         <v>39</v>
       </c>
     </row>
@@ -4126,19 +4192,19 @@
           <t>Iran</t>
         </is>
       </c>
-      <c r="E169" s="61" t="n">
+      <c r="E169" s="62" t="n">
         <v>9</v>
       </c>
-      <c r="F169" s="61" t="n">
+      <c r="F169" s="62" t="n">
         <v>15</v>
       </c>
-      <c r="G169" s="61" t="n">
+      <c r="G169" s="62" t="n">
         <v>22</v>
       </c>
-      <c r="H169" s="61" t="n">
+      <c r="H169" s="62" t="n">
         <v>31</v>
       </c>
-      <c r="I169" s="61" t="n">
+      <c r="I169" s="62" t="n">
         <v>41</v>
       </c>
     </row>
@@ -4148,19 +4214,19 @@
           <t>Oostenrijk</t>
         </is>
       </c>
-      <c r="E170" s="61" t="n">
+      <c r="E170" s="62" t="n">
         <v>9</v>
       </c>
-      <c r="F170" s="61" t="n">
+      <c r="F170" s="62" t="n">
         <v>15</v>
       </c>
-      <c r="G170" s="61" t="n">
+      <c r="G170" s="62" t="n">
         <v>23</v>
       </c>
-      <c r="H170" s="61" t="n">
+      <c r="H170" s="62" t="n">
         <v>32</v>
       </c>
-      <c r="I170" s="61" t="n">
+      <c r="I170" s="62" t="n">
         <v>42</v>
       </c>
     </row>
@@ -4170,19 +4236,19 @@
           <t>Zuid-Korea</t>
         </is>
       </c>
-      <c r="E171" s="61" t="n">
+      <c r="E171" s="62" t="n">
         <v>9</v>
       </c>
-      <c r="F171" s="61" t="n">
+      <c r="F171" s="62" t="n">
         <v>16</v>
       </c>
-      <c r="G171" s="61" t="n">
+      <c r="G171" s="62" t="n">
         <v>23</v>
       </c>
-      <c r="H171" s="61" t="n">
+      <c r="H171" s="62" t="n">
         <v>32</v>
       </c>
-      <c r="I171" s="61" t="n">
+      <c r="I171" s="62" t="n">
         <v>43</v>
       </c>
     </row>
@@ -4192,19 +4258,19 @@
           <t>Australië</t>
         </is>
       </c>
-      <c r="E172" s="61" t="n">
+      <c r="E172" s="62" t="n">
         <v>9</v>
       </c>
-      <c r="F172" s="61" t="n">
+      <c r="F172" s="62" t="n">
         <v>16</v>
       </c>
-      <c r="G172" s="61" t="n">
+      <c r="G172" s="62" t="n">
         <v>24</v>
       </c>
-      <c r="H172" s="61" t="n">
+      <c r="H172" s="62" t="n">
         <v>33</v>
       </c>
-      <c r="I172" s="61" t="n">
+      <c r="I172" s="62" t="n">
         <v>43</v>
       </c>
     </row>
@@ -4214,19 +4280,19 @@
           <t>Ecuador</t>
         </is>
       </c>
-      <c r="E173" s="61" t="n">
+      <c r="E173" s="62" t="n">
         <v>9</v>
       </c>
-      <c r="F173" s="61" t="n">
+      <c r="F173" s="62" t="n">
         <v>16</v>
       </c>
-      <c r="G173" s="61" t="n">
+      <c r="G173" s="62" t="n">
         <v>24</v>
       </c>
-      <c r="H173" s="61" t="n">
+      <c r="H173" s="62" t="n">
         <v>34</v>
       </c>
-      <c r="I173" s="61" t="n">
+      <c r="I173" s="62" t="n">
         <v>44</v>
       </c>
     </row>
@@ -4236,19 +4302,19 @@
           <t>Noorwegen</t>
         </is>
       </c>
-      <c r="E174" s="61" t="n">
+      <c r="E174" s="62" t="n">
         <v>10</v>
       </c>
-      <c r="F174" s="61" t="n">
+      <c r="F174" s="62" t="n">
         <v>16</v>
       </c>
-      <c r="G174" s="61" t="n">
+      <c r="G174" s="62" t="n">
         <v>25</v>
       </c>
-      <c r="H174" s="61" t="n">
+      <c r="H174" s="62" t="n">
         <v>34</v>
       </c>
-      <c r="I174" s="61" t="n">
+      <c r="I174" s="62" t="n">
         <v>45</v>
       </c>
     </row>
@@ -4258,19 +4324,19 @@
           <t>Panama</t>
         </is>
       </c>
-      <c r="E175" s="61" t="n">
+      <c r="E175" s="62" t="n">
         <v>10</v>
       </c>
-      <c r="F175" s="61" t="n">
+      <c r="F175" s="62" t="n">
         <v>17</v>
       </c>
-      <c r="G175" s="61" t="n">
+      <c r="G175" s="62" t="n">
         <v>26</v>
       </c>
-      <c r="H175" s="61" t="n">
+      <c r="H175" s="62" t="n">
         <v>36</v>
       </c>
-      <c r="I175" s="61" t="n">
+      <c r="I175" s="62" t="n">
         <v>48</v>
       </c>
     </row>
@@ -4280,19 +4346,19 @@
           <t>Egypte</t>
         </is>
       </c>
-      <c r="E176" s="61" t="n">
+      <c r="E176" s="62" t="n">
         <v>10</v>
       </c>
-      <c r="F176" s="61" t="n">
+      <c r="F176" s="62" t="n">
         <v>18</v>
       </c>
-      <c r="G176" s="61" t="n">
+      <c r="G176" s="62" t="n">
         <v>27</v>
       </c>
-      <c r="H176" s="61" t="n">
+      <c r="H176" s="62" t="n">
         <v>37</v>
       </c>
-      <c r="I176" s="61" t="n">
+      <c r="I176" s="62" t="n">
         <v>49</v>
       </c>
     </row>
@@ -4302,19 +4368,19 @@
           <t>Algerije</t>
         </is>
       </c>
-      <c r="E177" s="61" t="n">
+      <c r="E177" s="62" t="n">
         <v>11</v>
       </c>
-      <c r="F177" s="61" t="n">
+      <c r="F177" s="62" t="n">
         <v>19</v>
       </c>
-      <c r="G177" s="61" t="n">
+      <c r="G177" s="62" t="n">
         <v>28</v>
       </c>
-      <c r="H177" s="61" t="n">
+      <c r="H177" s="62" t="n">
         <v>40</v>
       </c>
-      <c r="I177" s="61" t="n">
+      <c r="I177" s="62" t="n">
         <v>52</v>
       </c>
     </row>
@@ -4324,19 +4390,19 @@
           <t>Paraguay</t>
         </is>
       </c>
-      <c r="E178" s="61" t="n">
+      <c r="E178" s="62" t="n">
         <v>11</v>
       </c>
-      <c r="F178" s="61" t="n">
+      <c r="F178" s="62" t="n">
         <v>19</v>
       </c>
-      <c r="G178" s="61" t="n">
+      <c r="G178" s="62" t="n">
         <v>29</v>
       </c>
-      <c r="H178" s="61" t="n">
+      <c r="H178" s="62" t="n">
         <v>41</v>
       </c>
-      <c r="I178" s="61" t="n">
+      <c r="I178" s="62" t="n">
         <v>53</v>
       </c>
     </row>
@@ -4346,19 +4412,19 @@
           <t>Ivoorkust</t>
         </is>
       </c>
-      <c r="E179" s="61" t="n">
+      <c r="E179" s="62" t="n">
         <v>12</v>
       </c>
-      <c r="F179" s="61" t="n">
+      <c r="F179" s="62" t="n">
         <v>20</v>
       </c>
-      <c r="G179" s="61" t="n">
+      <c r="G179" s="62" t="n">
         <v>30</v>
       </c>
-      <c r="H179" s="61" t="n">
+      <c r="H179" s="62" t="n">
         <v>41</v>
       </c>
-      <c r="I179" s="61" t="n">
+      <c r="I179" s="62" t="n">
         <v>55</v>
       </c>
     </row>
@@ -4368,19 +4434,19 @@
           <t>Tunesië</t>
         </is>
       </c>
-      <c r="E180" s="61" t="n">
+      <c r="E180" s="62" t="n">
         <v>12</v>
       </c>
-      <c r="F180" s="61" t="n">
+      <c r="F180" s="62" t="n">
         <v>20</v>
       </c>
-      <c r="G180" s="61" t="n">
+      <c r="G180" s="62" t="n">
         <v>30</v>
       </c>
-      <c r="H180" s="61" t="n">
+      <c r="H180" s="62" t="n">
         <v>42</v>
       </c>
-      <c r="I180" s="61" t="n">
+      <c r="I180" s="62" t="n">
         <v>55</v>
       </c>
     </row>
@@ -4390,19 +4456,19 @@
           <t>Schotland</t>
         </is>
       </c>
-      <c r="E181" s="61" t="n">
+      <c r="E181" s="62" t="n">
         <v>12</v>
       </c>
-      <c r="F181" s="61" t="n">
+      <c r="F181" s="62" t="n">
         <v>20</v>
       </c>
-      <c r="G181" s="61" t="n">
+      <c r="G181" s="62" t="n">
         <v>31</v>
       </c>
-      <c r="H181" s="61" t="n">
+      <c r="H181" s="62" t="n">
         <v>42</v>
       </c>
-      <c r="I181" s="61" t="n">
+      <c r="I181" s="62" t="n">
         <v>56</v>
       </c>
     </row>
@@ -4412,19 +4478,19 @@
           <t>Zweden</t>
         </is>
       </c>
-      <c r="E182" s="61" t="n">
+      <c r="E182" s="62" t="n">
         <v>12</v>
       </c>
-      <c r="F182" s="61" t="n">
+      <c r="F182" s="62" t="n">
         <v>21</v>
       </c>
-      <c r="G182" s="61" t="n">
+      <c r="G182" s="62" t="n">
         <v>31</v>
       </c>
-      <c r="H182" s="61" t="n">
+      <c r="H182" s="62" t="n">
         <v>43</v>
       </c>
-      <c r="I182" s="61" t="n">
+      <c r="I182" s="62" t="n">
         <v>57</v>
       </c>
     </row>
@@ -4434,19 +4500,19 @@
           <t>Tsjechië</t>
         </is>
       </c>
-      <c r="E183" s="61" t="n">
+      <c r="E183" s="62" t="n">
         <v>12</v>
       </c>
-      <c r="F183" s="61" t="n">
+      <c r="F183" s="62" t="n">
         <v>21</v>
       </c>
-      <c r="G183" s="61" t="n">
+      <c r="G183" s="62" t="n">
         <v>31</v>
       </c>
-      <c r="H183" s="61" t="n">
+      <c r="H183" s="62" t="n">
         <v>43</v>
       </c>
-      <c r="I183" s="61" t="n">
+      <c r="I183" s="62" t="n">
         <v>57</v>
       </c>
     </row>
@@ -4456,19 +4522,19 @@
           <t>Qatar</t>
         </is>
       </c>
-      <c r="E184" s="61" t="n">
+      <c r="E184" s="62" t="n">
         <v>13</v>
       </c>
-      <c r="F184" s="61" t="n">
+      <c r="F184" s="62" t="n">
         <v>22</v>
       </c>
-      <c r="G184" s="61" t="n">
+      <c r="G184" s="62" t="n">
         <v>33</v>
       </c>
-      <c r="H184" s="61" t="n">
+      <c r="H184" s="62" t="n">
         <v>46</v>
       </c>
-      <c r="I184" s="61" t="n">
+      <c r="I184" s="62" t="n">
         <v>61</v>
       </c>
     </row>
@@ -4478,19 +4544,19 @@
           <t>Oezbekistan</t>
         </is>
       </c>
-      <c r="E185" s="61" t="n">
+      <c r="E185" s="62" t="n">
         <v>13</v>
       </c>
-      <c r="F185" s="61" t="n">
+      <c r="F185" s="62" t="n">
         <v>23</v>
       </c>
-      <c r="G185" s="61" t="n">
+      <c r="G185" s="62" t="n">
         <v>34</v>
       </c>
-      <c r="H185" s="61" t="n">
+      <c r="H185" s="62" t="n">
         <v>47</v>
       </c>
-      <c r="I185" s="61" t="n">
+      <c r="I185" s="62" t="n">
         <v>63</v>
       </c>
     </row>
@@ -4500,19 +4566,19 @@
           <t>DR Congo</t>
         </is>
       </c>
-      <c r="E186" s="61" t="n">
+      <c r="E186" s="62" t="n">
         <v>14</v>
       </c>
-      <c r="F186" s="61" t="n">
+      <c r="F186" s="62" t="n">
         <v>23</v>
       </c>
-      <c r="G186" s="61" t="n">
+      <c r="G186" s="62" t="n">
         <v>35</v>
       </c>
-      <c r="H186" s="61" t="n">
+      <c r="H186" s="62" t="n">
         <v>48</v>
       </c>
-      <c r="I186" s="61" t="n">
+      <c r="I186" s="62" t="n">
         <v>64</v>
       </c>
     </row>
@@ -4522,19 +4588,19 @@
           <t>Saoedi-Arabië</t>
         </is>
       </c>
-      <c r="E187" s="61" t="n">
+      <c r="E187" s="62" t="n">
         <v>14</v>
       </c>
-      <c r="F187" s="61" t="n">
+      <c r="F187" s="62" t="n">
         <v>24</v>
       </c>
-      <c r="G187" s="61" t="n">
+      <c r="G187" s="62" t="n">
         <v>35</v>
       </c>
-      <c r="H187" s="61" t="n">
+      <c r="H187" s="62" t="n">
         <v>49</v>
       </c>
-      <c r="I187" s="61" t="n">
+      <c r="I187" s="62" t="n">
         <v>65</v>
       </c>
     </row>
@@ -4544,19 +4610,19 @@
           <t>Irak</t>
         </is>
       </c>
-      <c r="E188" s="61" t="n">
+      <c r="E188" s="62" t="n">
         <v>14</v>
       </c>
-      <c r="F188" s="61" t="n">
+      <c r="F188" s="62" t="n">
         <v>24</v>
       </c>
-      <c r="G188" s="61" t="n">
+      <c r="G188" s="62" t="n">
         <v>36</v>
       </c>
-      <c r="H188" s="61" t="n">
+      <c r="H188" s="62" t="n">
         <v>49</v>
       </c>
-      <c r="I188" s="61" t="n">
+      <c r="I188" s="62" t="n">
         <v>65</v>
       </c>
     </row>
@@ -4566,19 +4632,19 @@
           <t>Zuid-Afrika</t>
         </is>
       </c>
-      <c r="E189" s="61" t="n">
+      <c r="E189" s="62" t="n">
         <v>14</v>
       </c>
-      <c r="F189" s="61" t="n">
+      <c r="F189" s="62" t="n">
         <v>24</v>
       </c>
-      <c r="G189" s="61" t="n">
+      <c r="G189" s="62" t="n">
         <v>36</v>
       </c>
-      <c r="H189" s="61" t="n">
+      <c r="H189" s="62" t="n">
         <v>50</v>
       </c>
-      <c r="I189" s="61" t="n">
+      <c r="I189" s="62" t="n">
         <v>66</v>
       </c>
     </row>
@@ -4588,19 +4654,19 @@
           <t>Jordanië</t>
         </is>
       </c>
-      <c r="E190" s="61" t="n">
+      <c r="E190" s="62" t="n">
         <v>14</v>
       </c>
-      <c r="F190" s="61" t="n">
+      <c r="F190" s="62" t="n">
         <v>25</v>
       </c>
-      <c r="G190" s="61" t="n">
+      <c r="G190" s="62" t="n">
         <v>37</v>
       </c>
-      <c r="H190" s="61" t="n">
+      <c r="H190" s="62" t="n">
         <v>51</v>
       </c>
-      <c r="I190" s="61" t="n">
+      <c r="I190" s="62" t="n">
         <v>68</v>
       </c>
     </row>
@@ -4610,19 +4676,19 @@
           <t>Kaapverdië</t>
         </is>
       </c>
-      <c r="E191" s="61" t="n">
+      <c r="E191" s="62" t="n">
         <v>15</v>
       </c>
-      <c r="F191" s="61" t="n">
+      <c r="F191" s="62" t="n">
         <v>26</v>
       </c>
-      <c r="G191" s="61" t="n">
+      <c r="G191" s="62" t="n">
         <v>38</v>
       </c>
-      <c r="H191" s="61" t="n">
+      <c r="H191" s="62" t="n">
         <v>53</v>
       </c>
-      <c r="I191" s="61" t="n">
+      <c r="I191" s="62" t="n">
         <v>70</v>
       </c>
     </row>
@@ -4632,19 +4698,19 @@
           <t>Ghana</t>
         </is>
       </c>
-      <c r="E192" s="61" t="n">
+      <c r="E192" s="62" t="n">
         <v>15</v>
       </c>
-      <c r="F192" s="61" t="n">
+      <c r="F192" s="62" t="n">
         <v>26</v>
       </c>
-      <c r="G192" s="61" t="n">
+      <c r="G192" s="62" t="n">
         <v>39</v>
       </c>
-      <c r="H192" s="61" t="n">
+      <c r="H192" s="62" t="n">
         <v>54</v>
       </c>
-      <c r="I192" s="61" t="n">
+      <c r="I192" s="62" t="n">
         <v>72</v>
       </c>
     </row>
@@ -4654,19 +4720,19 @@
           <t>Bosnië-Herzegovina</t>
         </is>
       </c>
-      <c r="E193" s="61" t="n">
+      <c r="E193" s="62" t="n">
         <v>15</v>
       </c>
-      <c r="F193" s="61" t="n">
+      <c r="F193" s="62" t="n">
         <v>26</v>
       </c>
-      <c r="G193" s="61" t="n">
+      <c r="G193" s="62" t="n">
         <v>39</v>
       </c>
-      <c r="H193" s="61" t="n">
+      <c r="H193" s="62" t="n">
         <v>55</v>
       </c>
-      <c r="I193" s="61" t="n">
+      <c r="I193" s="62" t="n">
         <v>72</v>
       </c>
     </row>
@@ -4676,19 +4742,19 @@
           <t>Haïti</t>
         </is>
       </c>
-      <c r="E194" s="61" t="n">
+      <c r="E194" s="62" t="n">
         <v>16</v>
       </c>
-      <c r="F194" s="61" t="n">
+      <c r="F194" s="62" t="n">
         <v>28</v>
       </c>
-      <c r="G194" s="61" t="n">
+      <c r="G194" s="62" t="n">
         <v>41</v>
       </c>
-      <c r="H194" s="61" t="n">
+      <c r="H194" s="62" t="n">
         <v>58</v>
       </c>
-      <c r="I194" s="61" t="n">
+      <c r="I194" s="62" t="n">
         <v>76</v>
       </c>
     </row>
@@ -4698,19 +4764,19 @@
           <t>Nieuw-Zeeland</t>
         </is>
       </c>
-      <c r="E195" s="61" t="n">
+      <c r="E195" s="62" t="n">
         <v>16</v>
       </c>
-      <c r="F195" s="61" t="n">
+      <c r="F195" s="62" t="n">
         <v>28</v>
       </c>
-      <c r="G195" s="61" t="n">
+      <c r="G195" s="62" t="n">
         <v>42</v>
       </c>
-      <c r="H195" s="61" t="n">
+      <c r="H195" s="62" t="n">
         <v>59</v>
       </c>
-      <c r="I195" s="61" t="n">
+      <c r="I195" s="62" t="n">
         <v>77</v>
       </c>
     </row>
@@ -4720,19 +4786,19 @@
           <t>Curaçao</t>
         </is>
       </c>
-      <c r="E196" s="61" t="n">
+      <c r="E196" s="62" t="n">
         <v>17</v>
       </c>
-      <c r="F196" s="61" t="n">
+      <c r="F196" s="62" t="n">
         <v>29</v>
       </c>
-      <c r="G196" s="61" t="n">
+      <c r="G196" s="62" t="n">
         <v>43</v>
       </c>
-      <c r="H196" s="61" t="n">
+      <c r="H196" s="62" t="n">
         <v>60</v>
       </c>
-      <c r="I196" s="61" t="n">
+      <c r="I196" s="62" t="n">
         <v>79</v>
       </c>
     </row>
@@ -4742,19 +4808,19 @@
           <t>Canada</t>
         </is>
       </c>
-      <c r="E197" s="61" t="n">
+      <c r="E197" s="62" t="n">
         <v>13</v>
       </c>
-      <c r="F197" s="61" t="n">
+      <c r="F197" s="62" t="n">
         <v>22</v>
       </c>
-      <c r="G197" s="61" t="n">
+      <c r="G197" s="62" t="n">
         <v>33</v>
       </c>
-      <c r="H197" s="61" t="n">
+      <c r="H197" s="62" t="n">
         <v>46</v>
       </c>
-      <c r="I197" s="61" t="n">
+      <c r="I197" s="62" t="n">
         <v>61</v>
       </c>
     </row>
@@ -4764,19 +4830,19 @@
           <t>Turkije</t>
         </is>
       </c>
-      <c r="E198" s="61" t="n">
+      <c r="E198" s="62" t="n">
         <v>13</v>
       </c>
-      <c r="F198" s="61" t="n">
+      <c r="F198" s="62" t="n">
         <v>22</v>
       </c>
-      <c r="G198" s="61" t="n">
+      <c r="G198" s="62" t="n">
         <v>33</v>
       </c>
-      <c r="H198" s="61" t="n">
+      <c r="H198" s="62" t="n">
         <v>46</v>
       </c>
-      <c r="I198" s="61" t="n">
+      <c r="I198" s="62" t="n">
         <v>61</v>
       </c>
     </row>
@@ -4821,16 +4887,16 @@
           <t>Frankrijk</t>
         </is>
       </c>
-      <c r="E202" s="61" t="n">
+      <c r="E202" s="62" t="n">
         <v>8</v>
       </c>
-      <c r="F202" s="61" t="n">
+      <c r="F202" s="62" t="n">
         <v>14</v>
       </c>
-      <c r="G202" s="61" t="n">
+      <c r="G202" s="62" t="n">
         <v>20</v>
       </c>
-      <c r="H202" s="61" t="n">
+      <c r="H202" s="62" t="n">
         <v>30</v>
       </c>
     </row>
@@ -4840,16 +4906,16 @@
           <t>Spanje</t>
         </is>
       </c>
-      <c r="E203" s="61" t="n">
+      <c r="E203" s="62" t="n">
         <v>7</v>
       </c>
-      <c r="F203" s="61" t="n">
+      <c r="F203" s="62" t="n">
         <v>13</v>
       </c>
-      <c r="G203" s="61" t="n">
+      <c r="G203" s="62" t="n">
         <v>19</v>
       </c>
-      <c r="H203" s="61" t="n">
+      <c r="H203" s="62" t="n">
         <v>28</v>
       </c>
     </row>
@@ -4859,16 +4925,16 @@
           <t>Argentinië</t>
         </is>
       </c>
-      <c r="E204" s="61" t="n">
+      <c r="E204" s="62" t="n">
         <v>6</v>
       </c>
-      <c r="F204" s="61" t="n">
+      <c r="F204" s="62" t="n">
         <v>12</v>
       </c>
-      <c r="G204" s="61" t="n">
+      <c r="G204" s="62" t="n">
         <v>17</v>
       </c>
-      <c r="H204" s="61" t="n">
+      <c r="H204" s="62" t="n">
         <v>26</v>
       </c>
     </row>
@@ -4878,16 +4944,16 @@
           <t>Engeland</t>
         </is>
       </c>
-      <c r="E205" s="61" t="n">
+      <c r="E205" s="62" t="n">
         <v>6</v>
       </c>
-      <c r="F205" s="61" t="n">
+      <c r="F205" s="62" t="n">
         <v>11</v>
       </c>
-      <c r="G205" s="61" t="n">
+      <c r="G205" s="62" t="n">
         <v>16</v>
       </c>
-      <c r="H205" s="61" t="n">
+      <c r="H205" s="62" t="n">
         <v>24</v>
       </c>
     </row>
@@ -4897,16 +4963,16 @@
           <t>Portugal</t>
         </is>
       </c>
-      <c r="E206" s="61" t="n">
+      <c r="E206" s="62" t="n">
         <v>6</v>
       </c>
-      <c r="F206" s="61" t="n">
+      <c r="F206" s="62" t="n">
         <v>10</v>
       </c>
-      <c r="G206" s="61" t="n">
+      <c r="G206" s="62" t="n">
         <v>15</v>
       </c>
-      <c r="H206" s="61" t="n">
+      <c r="H206" s="62" t="n">
         <v>22</v>
       </c>
     </row>
@@ -4916,16 +4982,16 @@
           <t>Brazilië</t>
         </is>
       </c>
-      <c r="E207" s="61" t="n">
+      <c r="E207" s="62" t="n">
         <v>5</v>
       </c>
-      <c r="F207" s="61" t="n">
+      <c r="F207" s="62" t="n">
         <v>9</v>
       </c>
-      <c r="G207" s="61" t="n">
+      <c r="G207" s="62" t="n">
         <v>13</v>
       </c>
-      <c r="H207" s="61" t="n">
+      <c r="H207" s="62" t="n">
         <v>20</v>
       </c>
     </row>
@@ -4935,16 +5001,16 @@
           <t>Nederland</t>
         </is>
       </c>
-      <c r="E208" s="61" t="n">
+      <c r="E208" s="62" t="n">
         <v>4</v>
       </c>
-      <c r="F208" s="61" t="n">
+      <c r="F208" s="62" t="n">
         <v>8</v>
       </c>
-      <c r="G208" s="61" t="n">
+      <c r="G208" s="62" t="n">
         <v>12</v>
       </c>
-      <c r="H208" s="61" t="n">
+      <c r="H208" s="62" t="n">
         <v>18</v>
       </c>
     </row>
@@ -4954,16 +5020,16 @@
           <t>Marokko</t>
         </is>
       </c>
-      <c r="E209" s="61" t="n">
+      <c r="E209" s="62" t="n">
         <v>4</v>
       </c>
-      <c r="F209" s="61" t="n">
+      <c r="F209" s="62" t="n">
         <v>7</v>
       </c>
-      <c r="G209" s="61" t="n">
+      <c r="G209" s="62" t="n">
         <v>11</v>
       </c>
-      <c r="H209" s="61" t="n">
+      <c r="H209" s="62" t="n">
         <v>16</v>
       </c>
     </row>
@@ -4973,16 +5039,16 @@
           <t>België</t>
         </is>
       </c>
-      <c r="E210" s="61" t="n">
+      <c r="E210" s="62" t="n">
         <v>4</v>
       </c>
-      <c r="F210" s="61" t="n">
+      <c r="F210" s="62" t="n">
         <v>6</v>
       </c>
-      <c r="G210" s="61" t="n">
+      <c r="G210" s="62" t="n">
         <v>9</v>
       </c>
-      <c r="H210" s="61" t="n">
+      <c r="H210" s="62" t="n">
         <v>14</v>
       </c>
     </row>
@@ -4992,16 +5058,16 @@
           <t>Duitsland</t>
         </is>
       </c>
-      <c r="E211" s="61" t="n">
+      <c r="E211" s="62" t="n">
         <v>3</v>
       </c>
-      <c r="F211" s="61" t="n">
+      <c r="F211" s="62" t="n">
         <v>6</v>
       </c>
-      <c r="G211" s="61" t="n">
+      <c r="G211" s="62" t="n">
         <v>8</v>
       </c>
-      <c r="H211" s="61" t="n">
+      <c r="H211" s="62" t="n">
         <v>12</v>
       </c>
     </row>
@@ -5011,16 +5077,16 @@
           <t>Kroatië</t>
         </is>
       </c>
-      <c r="E212" s="61" t="n">
+      <c r="E212" s="62" t="n">
         <v>2</v>
       </c>
-      <c r="F212" s="61" t="n">
+      <c r="F212" s="62" t="n">
         <v>5</v>
       </c>
-      <c r="G212" s="61" t="n">
+      <c r="G212" s="62" t="n">
         <v>7</v>
       </c>
-      <c r="H212" s="61" t="n">
+      <c r="H212" s="62" t="n">
         <v>10</v>
       </c>
     </row>
@@ -5030,25 +5096,27 @@
           <t>Colombia</t>
         </is>
       </c>
-      <c r="E213" s="61" t="n">
+      <c r="E213" s="62" t="n">
         <v>2</v>
       </c>
-      <c r="F213" s="61" t="n">
+      <c r="F213" s="62" t="n">
         <v>3</v>
       </c>
-      <c r="G213" s="61" t="n">
+      <c r="G213" s="62" t="n">
         <v>4</v>
       </c>
-      <c r="H213" s="61" t="n">
+      <c r="H213" s="62" t="n">
         <v>6</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="199">
+  <mergeCells count="204">
     <mergeCell ref="E13:G13"/>
     <mergeCell ref="A122:D122"/>
     <mergeCell ref="A97:D97"/>
     <mergeCell ref="A133:O133"/>
+    <mergeCell ref="A134:D134"/>
+    <mergeCell ref="A152:D152"/>
     <mergeCell ref="A121:D121"/>
     <mergeCell ref="E15:G15"/>
     <mergeCell ref="A13:D13"/>
@@ -5140,6 +5208,7 @@
     <mergeCell ref="I56:L56"/>
     <mergeCell ref="I96:L96"/>
     <mergeCell ref="M107:O107"/>
+    <mergeCell ref="A145:D145"/>
     <mergeCell ref="A192:D192"/>
     <mergeCell ref="B30:O30"/>
     <mergeCell ref="A139:D139"/>
@@ -5163,6 +5232,7 @@
     <mergeCell ref="E9:G9"/>
     <mergeCell ref="A10:D10"/>
     <mergeCell ref="B46:O46"/>
+    <mergeCell ref="A115:D115"/>
     <mergeCell ref="I59:L59"/>
     <mergeCell ref="I99:L99"/>
     <mergeCell ref="A173:D173"/>
@@ -5171,6 +5241,7 @@
     <mergeCell ref="A77:D77"/>
     <mergeCell ref="I69:L69"/>
     <mergeCell ref="A33:O33"/>
+    <mergeCell ref="A157:D157"/>
     <mergeCell ref="A166:D166"/>
     <mergeCell ref="A8:O8"/>
     <mergeCell ref="A49:D49"/>

</xml_diff>

<commit_message>
Groepswinnaar, runner-up en beste 8 nr3 zijn nu vrij invulbaar
Deelnemers vullen zelf per groep de verwachte winnaar en runner-up in
(dropdown beperkt tot de 4 teams van die groep), plus de 8 verwachte
beste nummers 3. Deze voorspellingen mogen afwijken van wat de
wedstrijdscores logisch opleveren. AGENT_INSTRUCTIONS.md: berekeningssectie
verwijderd (top2/best3 zijn nu altijd expliciet ingevuld).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tempetoto2026_invulformulier.xlsx
+++ b/tempetoto2026_invulformulier.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="14">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -87,12 +87,6 @@
       <name val="Calibri"/>
       <i val="1"/>
       <color rgb="00888888"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="00555555"/>
       <sz val="10"/>
     </font>
     <font>
@@ -421,7 +415,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
@@ -511,14 +505,11 @@
     <xf numFmtId="0" fontId="0" fillId="47" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="48" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="49" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="8" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="50" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="50" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -916,7 +907,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C48"/>
+  <dimension ref="A1:O48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -935,6 +926,66 @@
           <t>Frankrijk</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Brazilië</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Verenigde Staten</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Duitsland</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Nederland</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>België</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Spanje</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Frankrijk</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Argentinië</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Engeland</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -952,6 +1003,66 @@
           <t>Spanje</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Zuid-Afrika</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Zwitserland</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Marokko</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Paraguay</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Curaçao</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Egypte</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Kaapverdië</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Senegal</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Algerije</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>DR Congo</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Kroatië</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -969,6 +1080,66 @@
           <t>Argentinië</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Zuid-Korea</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Qatar</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Haïti</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Australië</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Ivoorkust</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Zweden</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Iran</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Saoedi-Arabië</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Noorwegen</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Oostenrijk</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Oezbekistan</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Ghana</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -984,6 +1155,66 @@
       <c r="C4" t="inlineStr">
         <is>
           <t>Engeland</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Tsjechië</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Bosnië-Herzegovina</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Schotland</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Turkije</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Tunesië</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Nieuw-Zeeland</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Uruguay</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Irak</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Jordanië</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Panama</t>
         </is>
       </c>
     </row>
@@ -1506,7 +1737,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A6:O213"/>
+  <dimension ref="A6:O214"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -1636,7 +1867,7 @@
     <row r="21" ht="40" customHeight="1">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>3.  Groepswinnaar, runner-up en beste nummers 3 worden AUTOMATISCH berekend uit je scores — je hoeft die niet in te vullen.</t>
+          <t>3.  Na je wedstrijdscores vul je per groep de groepswinnaar en runner-up in, én de 8 beste nummers 3. Dit zijn vrije voorspellingen — ze mogen afwijken van wat je scores logisch opleveren.</t>
         </is>
       </c>
     </row>
@@ -2057,21 +2288,17 @@
           <t>Groepswinnaar:</t>
         </is>
       </c>
-      <c r="E56" s="17" t="inlineStr">
-        <is>
-          <t>↳ niet invullen</t>
-        </is>
-      </c>
+      <c r="E56" s="5" t="n"/>
+      <c r="F56" s="17" t="inlineStr"/>
+      <c r="G56" s="17" t="inlineStr"/>
       <c r="I56" s="4" t="inlineStr">
         <is>
           <t>Groepswinnaar:</t>
         </is>
       </c>
-      <c r="M56" s="17" t="inlineStr">
-        <is>
-          <t>↳ niet invullen</t>
-        </is>
-      </c>
+      <c r="M56" s="5" t="n"/>
+      <c r="N56" s="17" t="inlineStr"/>
+      <c r="O56" s="17" t="inlineStr"/>
     </row>
     <row r="57" ht="17" customHeight="1">
       <c r="A57" s="4" t="inlineStr">
@@ -2079,21 +2306,17 @@
           <t>Runner-up:</t>
         </is>
       </c>
-      <c r="E57" s="17" t="inlineStr">
-        <is>
-          <t>↳ niet invullen</t>
-        </is>
-      </c>
+      <c r="E57" s="5" t="n"/>
+      <c r="F57" s="17" t="inlineStr"/>
+      <c r="G57" s="17" t="inlineStr"/>
       <c r="I57" s="4" t="inlineStr">
         <is>
           <t>Runner-up:</t>
         </is>
       </c>
-      <c r="M57" s="17" t="inlineStr">
-        <is>
-          <t>↳ niet invullen</t>
-        </is>
-      </c>
+      <c r="M57" s="5" t="n"/>
+      <c r="N57" s="17" t="inlineStr"/>
+      <c r="O57" s="17" t="inlineStr"/>
     </row>
     <row r="58" ht="6" customHeight="1"/>
     <row r="59" ht="16" customHeight="1">
@@ -2336,21 +2559,17 @@
           <t>Groepswinnaar:</t>
         </is>
       </c>
-      <c r="E66" s="17" t="inlineStr">
-        <is>
-          <t>↳ niet invullen</t>
-        </is>
-      </c>
+      <c r="E66" s="5" t="n"/>
+      <c r="F66" s="17" t="inlineStr"/>
+      <c r="G66" s="17" t="inlineStr"/>
       <c r="I66" s="4" t="inlineStr">
         <is>
           <t>Groepswinnaar:</t>
         </is>
       </c>
-      <c r="M66" s="17" t="inlineStr">
-        <is>
-          <t>↳ niet invullen</t>
-        </is>
-      </c>
+      <c r="M66" s="5" t="n"/>
+      <c r="N66" s="17" t="inlineStr"/>
+      <c r="O66" s="17" t="inlineStr"/>
     </row>
     <row r="67" ht="17" customHeight="1">
       <c r="A67" s="4" t="inlineStr">
@@ -2358,21 +2577,17 @@
           <t>Runner-up:</t>
         </is>
       </c>
-      <c r="E67" s="17" t="inlineStr">
-        <is>
-          <t>↳ niet invullen</t>
-        </is>
-      </c>
+      <c r="E67" s="5" t="n"/>
+      <c r="F67" s="17" t="inlineStr"/>
+      <c r="G67" s="17" t="inlineStr"/>
       <c r="I67" s="4" t="inlineStr">
         <is>
           <t>Runner-up:</t>
         </is>
       </c>
-      <c r="M67" s="17" t="inlineStr">
-        <is>
-          <t>↳ niet invullen</t>
-        </is>
-      </c>
+      <c r="M67" s="5" t="n"/>
+      <c r="N67" s="17" t="inlineStr"/>
+      <c r="O67" s="17" t="inlineStr"/>
     </row>
     <row r="68" ht="6" customHeight="1"/>
     <row r="69" ht="16" customHeight="1">
@@ -2615,21 +2830,17 @@
           <t>Groepswinnaar:</t>
         </is>
       </c>
-      <c r="E76" s="17" t="inlineStr">
-        <is>
-          <t>↳ niet invullen</t>
-        </is>
-      </c>
+      <c r="E76" s="5" t="n"/>
+      <c r="F76" s="17" t="inlineStr"/>
+      <c r="G76" s="17" t="inlineStr"/>
       <c r="I76" s="4" t="inlineStr">
         <is>
           <t>Groepswinnaar:</t>
         </is>
       </c>
-      <c r="M76" s="17" t="inlineStr">
-        <is>
-          <t>↳ niet invullen</t>
-        </is>
-      </c>
+      <c r="M76" s="5" t="n"/>
+      <c r="N76" s="17" t="inlineStr"/>
+      <c r="O76" s="17" t="inlineStr"/>
     </row>
     <row r="77" ht="17" customHeight="1">
       <c r="A77" s="4" t="inlineStr">
@@ -2637,21 +2848,17 @@
           <t>Runner-up:</t>
         </is>
       </c>
-      <c r="E77" s="17" t="inlineStr">
-        <is>
-          <t>↳ niet invullen</t>
-        </is>
-      </c>
+      <c r="E77" s="5" t="n"/>
+      <c r="F77" s="17" t="inlineStr"/>
+      <c r="G77" s="17" t="inlineStr"/>
       <c r="I77" s="4" t="inlineStr">
         <is>
           <t>Runner-up:</t>
         </is>
       </c>
-      <c r="M77" s="17" t="inlineStr">
-        <is>
-          <t>↳ niet invullen</t>
-        </is>
-      </c>
+      <c r="M77" s="5" t="n"/>
+      <c r="N77" s="17" t="inlineStr"/>
+      <c r="O77" s="17" t="inlineStr"/>
     </row>
     <row r="78" ht="6" customHeight="1"/>
     <row r="79" ht="16" customHeight="1">
@@ -2894,21 +3101,17 @@
           <t>Groepswinnaar:</t>
         </is>
       </c>
-      <c r="E86" s="17" t="inlineStr">
-        <is>
-          <t>↳ niet invullen</t>
-        </is>
-      </c>
+      <c r="E86" s="5" t="n"/>
+      <c r="F86" s="17" t="inlineStr"/>
+      <c r="G86" s="17" t="inlineStr"/>
       <c r="I86" s="4" t="inlineStr">
         <is>
           <t>Groepswinnaar:</t>
         </is>
       </c>
-      <c r="M86" s="17" t="inlineStr">
-        <is>
-          <t>↳ niet invullen</t>
-        </is>
-      </c>
+      <c r="M86" s="5" t="n"/>
+      <c r="N86" s="17" t="inlineStr"/>
+      <c r="O86" s="17" t="inlineStr"/>
     </row>
     <row r="87" ht="17" customHeight="1">
       <c r="A87" s="4" t="inlineStr">
@@ -2916,21 +3119,17 @@
           <t>Runner-up:</t>
         </is>
       </c>
-      <c r="E87" s="17" t="inlineStr">
-        <is>
-          <t>↳ niet invullen</t>
-        </is>
-      </c>
+      <c r="E87" s="5" t="n"/>
+      <c r="F87" s="17" t="inlineStr"/>
+      <c r="G87" s="17" t="inlineStr"/>
       <c r="I87" s="4" t="inlineStr">
         <is>
           <t>Runner-up:</t>
         </is>
       </c>
-      <c r="M87" s="17" t="inlineStr">
-        <is>
-          <t>↳ niet invullen</t>
-        </is>
-      </c>
+      <c r="M87" s="5" t="n"/>
+      <c r="N87" s="17" t="inlineStr"/>
+      <c r="O87" s="17" t="inlineStr"/>
     </row>
     <row r="88" ht="6" customHeight="1"/>
     <row r="89" ht="16" customHeight="1">
@@ -3173,21 +3372,17 @@
           <t>Groepswinnaar:</t>
         </is>
       </c>
-      <c r="E96" s="17" t="inlineStr">
-        <is>
-          <t>↳ niet invullen</t>
-        </is>
-      </c>
+      <c r="E96" s="5" t="n"/>
+      <c r="F96" s="17" t="inlineStr"/>
+      <c r="G96" s="17" t="inlineStr"/>
       <c r="I96" s="4" t="inlineStr">
         <is>
           <t>Groepswinnaar:</t>
         </is>
       </c>
-      <c r="M96" s="17" t="inlineStr">
-        <is>
-          <t>↳ niet invullen</t>
-        </is>
-      </c>
+      <c r="M96" s="5" t="n"/>
+      <c r="N96" s="17" t="inlineStr"/>
+      <c r="O96" s="17" t="inlineStr"/>
     </row>
     <row r="97" ht="17" customHeight="1">
       <c r="A97" s="4" t="inlineStr">
@@ -3195,21 +3390,17 @@
           <t>Runner-up:</t>
         </is>
       </c>
-      <c r="E97" s="17" t="inlineStr">
-        <is>
-          <t>↳ niet invullen</t>
-        </is>
-      </c>
+      <c r="E97" s="5" t="n"/>
+      <c r="F97" s="17" t="inlineStr"/>
+      <c r="G97" s="17" t="inlineStr"/>
       <c r="I97" s="4" t="inlineStr">
         <is>
           <t>Runner-up:</t>
         </is>
       </c>
-      <c r="M97" s="17" t="inlineStr">
-        <is>
-          <t>↳ niet invullen</t>
-        </is>
-      </c>
+      <c r="M97" s="5" t="n"/>
+      <c r="N97" s="17" t="inlineStr"/>
+      <c r="O97" s="17" t="inlineStr"/>
     </row>
     <row r="98" ht="6" customHeight="1"/>
     <row r="99" ht="16" customHeight="1">
@@ -3452,21 +3643,17 @@
           <t>Groepswinnaar:</t>
         </is>
       </c>
-      <c r="E106" s="17" t="inlineStr">
-        <is>
-          <t>↳ niet invullen</t>
-        </is>
-      </c>
+      <c r="E106" s="5" t="n"/>
+      <c r="F106" s="17" t="inlineStr"/>
+      <c r="G106" s="17" t="inlineStr"/>
       <c r="I106" s="4" t="inlineStr">
         <is>
           <t>Groepswinnaar:</t>
         </is>
       </c>
-      <c r="M106" s="17" t="inlineStr">
-        <is>
-          <t>↳ niet invullen</t>
-        </is>
-      </c>
+      <c r="M106" s="5" t="n"/>
+      <c r="N106" s="17" t="inlineStr"/>
+      <c r="O106" s="17" t="inlineStr"/>
     </row>
     <row r="107" ht="17" customHeight="1">
       <c r="A107" s="4" t="inlineStr">
@@ -3474,97 +3661,128 @@
           <t>Runner-up:</t>
         </is>
       </c>
-      <c r="E107" s="17" t="inlineStr">
-        <is>
-          <t>↳ niet invullen</t>
-        </is>
-      </c>
+      <c r="E107" s="5" t="n"/>
+      <c r="F107" s="17" t="inlineStr"/>
+      <c r="G107" s="17" t="inlineStr"/>
       <c r="I107" s="4" t="inlineStr">
         <is>
           <t>Runner-up:</t>
         </is>
       </c>
-      <c r="M107" s="17" t="inlineStr">
-        <is>
-          <t>↳ niet invullen</t>
-        </is>
-      </c>
+      <c r="M107" s="5" t="n"/>
+      <c r="N107" s="17" t="inlineStr"/>
+      <c r="O107" s="17" t="inlineStr"/>
     </row>
     <row r="108" ht="6" customHeight="1"/>
     <row r="109" ht="8" customHeight="1"/>
     <row r="110" ht="18" customHeight="1">
       <c r="A110" s="3" t="inlineStr">
         <is>
-          <t>▶  BESTE 8 NUMMERS 3  ·  niet invullen — wordt na inlevering door de agent berekend</t>
-        </is>
-      </c>
-    </row>
-    <row r="111" ht="40" customHeight="1">
-      <c r="A111" s="59" t="inlineStr">
-        <is>
-          <t>De 8 beste nummers 3 worden na inlevering van dit formulier automatisch berekend op basis van de punten en het doelsaldo van de nummer-3-landen in jouw groepsscores. De Excel zelf rekent dit NIET uit — je hoeft hier niets in te vullen.</t>
-        </is>
-      </c>
-    </row>
-    <row r="112" ht="8" customHeight="1"/>
-    <row r="113" ht="18" customHeight="1">
-      <c r="A113" s="3" t="inlineStr">
+          <t>▶  BESTE 8 NUMMERS 3  ·  vul in welke 8 nummers 3 jij verwacht dat doorgaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="18" customHeight="1">
+      <c r="A111" s="4" t="inlineStr">
+        <is>
+          <t>#1:</t>
+        </is>
+      </c>
+      <c r="C111" s="5" t="n"/>
+      <c r="E111" s="4" t="inlineStr">
+        <is>
+          <t>#2:</t>
+        </is>
+      </c>
+      <c r="G111" s="5" t="n"/>
+      <c r="I111" s="4" t="inlineStr">
+        <is>
+          <t>#3:</t>
+        </is>
+      </c>
+      <c r="K111" s="5" t="n"/>
+      <c r="M111" s="4" t="inlineStr">
+        <is>
+          <t>#4:</t>
+        </is>
+      </c>
+      <c r="O111" s="5" t="n"/>
+    </row>
+    <row r="112" ht="18" customHeight="1">
+      <c r="A112" s="4" t="inlineStr">
+        <is>
+          <t>#5:</t>
+        </is>
+      </c>
+      <c r="C112" s="5" t="n"/>
+      <c r="E112" s="4" t="inlineStr">
+        <is>
+          <t>#6:</t>
+        </is>
+      </c>
+      <c r="G112" s="5" t="n"/>
+      <c r="I112" s="4" t="inlineStr">
+        <is>
+          <t>#7:</t>
+        </is>
+      </c>
+      <c r="K112" s="5" t="n"/>
+      <c r="M112" s="4" t="inlineStr">
+        <is>
+          <t>#8:</t>
+        </is>
+      </c>
+      <c r="O112" s="5" t="n"/>
+    </row>
+    <row r="113" ht="8" customHeight="1"/>
+    <row r="114" ht="18" customHeight="1">
+      <c r="A114" s="3" t="inlineStr">
         <is>
           <t>▶  KNOCK-OUT  ·  grijze vakjes — invullen na de groepsfase, vóór elke ronde</t>
         </is>
       </c>
     </row>
-    <row r="114" ht="16" customHeight="1">
-      <c r="A114" s="9" t="inlineStr">
+    <row r="115" ht="16" customHeight="1">
+      <c r="A115" s="9" t="inlineStr">
         <is>
           <t>Ronde van 32  ·  toto 5 pt / exact +3 pt</t>
         </is>
       </c>
     </row>
-    <row r="115" ht="14" customHeight="1">
-      <c r="A115" s="12" t="inlineStr">
+    <row r="116" ht="14" customHeight="1">
+      <c r="A116" s="12" t="inlineStr">
         <is>
           <t>Wedstrijd</t>
         </is>
       </c>
-      <c r="E115" s="12" t="inlineStr">
+      <c r="E116" s="12" t="inlineStr">
         <is>
           <t>voorsp.</t>
         </is>
       </c>
-      <c r="F115" s="12" t="inlineStr">
+      <c r="F116" s="12" t="inlineStr">
         <is>
           <t>uitslag</t>
         </is>
       </c>
-      <c r="G115" s="12" t="inlineStr">
+      <c r="G116" s="12" t="inlineStr">
         <is>
           <t>pt.</t>
         </is>
       </c>
-      <c r="H115" s="60" t="n"/>
-      <c r="I115" s="60" t="n"/>
-      <c r="J115" s="60" t="n"/>
-      <c r="K115" s="60" t="n"/>
-      <c r="L115" s="60" t="n"/>
-      <c r="M115" s="60" t="n"/>
-      <c r="N115" s="60" t="n"/>
-      <c r="O115" s="60" t="n"/>
-    </row>
-    <row r="116" ht="16" customHeight="1">
-      <c r="A116" s="61" t="inlineStr">
+      <c r="H116" s="59" t="n"/>
+      <c r="I116" s="59" t="n"/>
+      <c r="J116" s="59" t="n"/>
+      <c r="K116" s="59" t="n"/>
+      <c r="L116" s="59" t="n"/>
+      <c r="M116" s="59" t="n"/>
+      <c r="N116" s="59" t="n"/>
+      <c r="O116" s="59" t="n"/>
+    </row>
+    <row r="117" ht="16" customHeight="1">
+      <c r="A117" s="60" t="inlineStr">
         <is>
           <t>2A  –  2B</t>
-        </is>
-      </c>
-      <c r="E116" s="17" t="inlineStr"/>
-      <c r="F116" s="17" t="inlineStr"/>
-      <c r="G116" s="17" t="inlineStr"/>
-    </row>
-    <row r="117" ht="16" customHeight="1">
-      <c r="A117" s="61" t="inlineStr">
-        <is>
-          <t>1E  –  3e (A/B/C/D/F)</t>
         </is>
       </c>
       <c r="E117" s="17" t="inlineStr"/>
@@ -3572,9 +3790,9 @@
       <c r="G117" s="17" t="inlineStr"/>
     </row>
     <row r="118" ht="16" customHeight="1">
-      <c r="A118" s="61" t="inlineStr">
-        <is>
-          <t>1F  –  2C</t>
+      <c r="A118" s="60" t="inlineStr">
+        <is>
+          <t>1E  –  3e (A/B/C/D/F)</t>
         </is>
       </c>
       <c r="E118" s="17" t="inlineStr"/>
@@ -3582,9 +3800,9 @@
       <c r="G118" s="17" t="inlineStr"/>
     </row>
     <row r="119" ht="16" customHeight="1">
-      <c r="A119" s="61" t="inlineStr">
-        <is>
-          <t>1C  –  2F</t>
+      <c r="A119" s="60" t="inlineStr">
+        <is>
+          <t>1F  –  2C</t>
         </is>
       </c>
       <c r="E119" s="17" t="inlineStr"/>
@@ -3592,9 +3810,9 @@
       <c r="G119" s="17" t="inlineStr"/>
     </row>
     <row r="120" ht="16" customHeight="1">
-      <c r="A120" s="61" t="inlineStr">
-        <is>
-          <t>1I  –  3e (C/D/F/G/H)</t>
+      <c r="A120" s="60" t="inlineStr">
+        <is>
+          <t>1C  –  2F</t>
         </is>
       </c>
       <c r="E120" s="17" t="inlineStr"/>
@@ -3602,9 +3820,9 @@
       <c r="G120" s="17" t="inlineStr"/>
     </row>
     <row r="121" ht="16" customHeight="1">
-      <c r="A121" s="61" t="inlineStr">
-        <is>
-          <t>2E  –  2I</t>
+      <c r="A121" s="60" t="inlineStr">
+        <is>
+          <t>1I  –  3e (C/D/F/G/H)</t>
         </is>
       </c>
       <c r="E121" s="17" t="inlineStr"/>
@@ -3612,9 +3830,9 @@
       <c r="G121" s="17" t="inlineStr"/>
     </row>
     <row r="122" ht="16" customHeight="1">
-      <c r="A122" s="61" t="inlineStr">
-        <is>
-          <t>1A  –  3e (C/E/F/H/I)</t>
+      <c r="A122" s="60" t="inlineStr">
+        <is>
+          <t>2E  –  2I</t>
         </is>
       </c>
       <c r="E122" s="17" t="inlineStr"/>
@@ -3622,9 +3840,9 @@
       <c r="G122" s="17" t="inlineStr"/>
     </row>
     <row r="123" ht="16" customHeight="1">
-      <c r="A123" s="61" t="inlineStr">
-        <is>
-          <t>1L  –  3e (E/H/I/J/K)</t>
+      <c r="A123" s="60" t="inlineStr">
+        <is>
+          <t>1A  –  3e (C/E/F/H/I)</t>
         </is>
       </c>
       <c r="E123" s="17" t="inlineStr"/>
@@ -3632,9 +3850,9 @@
       <c r="G123" s="17" t="inlineStr"/>
     </row>
     <row r="124" ht="16" customHeight="1">
-      <c r="A124" s="61" t="inlineStr">
-        <is>
-          <t>1D  –  3e (B/E/F/I/J)</t>
+      <c r="A124" s="60" t="inlineStr">
+        <is>
+          <t>1L  –  3e (E/H/I/J/K)</t>
         </is>
       </c>
       <c r="E124" s="17" t="inlineStr"/>
@@ -3642,9 +3860,9 @@
       <c r="G124" s="17" t="inlineStr"/>
     </row>
     <row r="125" ht="16" customHeight="1">
-      <c r="A125" s="61" t="inlineStr">
-        <is>
-          <t>1G  –  3e (A/E/H/I/J)</t>
+      <c r="A125" s="60" t="inlineStr">
+        <is>
+          <t>1D  –  3e (B/E/F/I/J)</t>
         </is>
       </c>
       <c r="E125" s="17" t="inlineStr"/>
@@ -3652,9 +3870,9 @@
       <c r="G125" s="17" t="inlineStr"/>
     </row>
     <row r="126" ht="16" customHeight="1">
-      <c r="A126" s="61" t="inlineStr">
-        <is>
-          <t>2K  –  2L</t>
+      <c r="A126" s="60" t="inlineStr">
+        <is>
+          <t>1G  –  3e (A/E/H/I/J)</t>
         </is>
       </c>
       <c r="E126" s="17" t="inlineStr"/>
@@ -3662,9 +3880,9 @@
       <c r="G126" s="17" t="inlineStr"/>
     </row>
     <row r="127" ht="16" customHeight="1">
-      <c r="A127" s="61" t="inlineStr">
-        <is>
-          <t>1H  –  2J</t>
+      <c r="A127" s="60" t="inlineStr">
+        <is>
+          <t>2K  –  2L</t>
         </is>
       </c>
       <c r="E127" s="17" t="inlineStr"/>
@@ -3672,9 +3890,9 @@
       <c r="G127" s="17" t="inlineStr"/>
     </row>
     <row r="128" ht="16" customHeight="1">
-      <c r="A128" s="61" t="inlineStr">
-        <is>
-          <t>1B  –  3e (E/F/G/I/J)</t>
+      <c r="A128" s="60" t="inlineStr">
+        <is>
+          <t>1H  –  2J</t>
         </is>
       </c>
       <c r="E128" s="17" t="inlineStr"/>
@@ -3682,9 +3900,9 @@
       <c r="G128" s="17" t="inlineStr"/>
     </row>
     <row r="129" ht="16" customHeight="1">
-      <c r="A129" s="61" t="inlineStr">
-        <is>
-          <t>1J  –  2H</t>
+      <c r="A129" s="60" t="inlineStr">
+        <is>
+          <t>1B  –  3e (E/F/G/I/J)</t>
         </is>
       </c>
       <c r="E129" s="17" t="inlineStr"/>
@@ -3692,9 +3910,9 @@
       <c r="G129" s="17" t="inlineStr"/>
     </row>
     <row r="130" ht="16" customHeight="1">
-      <c r="A130" s="61" t="inlineStr">
-        <is>
-          <t>1K  –  3e (D/E/I/J/L)</t>
+      <c r="A130" s="60" t="inlineStr">
+        <is>
+          <t>1J  –  2H</t>
         </is>
       </c>
       <c r="E130" s="17" t="inlineStr"/>
@@ -3702,67 +3920,67 @@
       <c r="G130" s="17" t="inlineStr"/>
     </row>
     <row r="131" ht="16" customHeight="1">
-      <c r="A131" s="61" t="inlineStr">
-        <is>
-          <t>2D  –  2G</t>
+      <c r="A131" s="60" t="inlineStr">
+        <is>
+          <t>1K  –  3e (D/E/I/J/L)</t>
         </is>
       </c>
       <c r="E131" s="17" t="inlineStr"/>
       <c r="F131" s="17" t="inlineStr"/>
       <c r="G131" s="17" t="inlineStr"/>
     </row>
-    <row r="132" ht="6" customHeight="1"/>
-    <row r="133" ht="16" customHeight="1">
-      <c r="A133" s="9" t="inlineStr">
+    <row r="132" ht="16" customHeight="1">
+      <c r="A132" s="60" t="inlineStr">
+        <is>
+          <t>2D  –  2G</t>
+        </is>
+      </c>
+      <c r="E132" s="17" t="inlineStr"/>
+      <c r="F132" s="17" t="inlineStr"/>
+      <c r="G132" s="17" t="inlineStr"/>
+    </row>
+    <row r="133" ht="6" customHeight="1"/>
+    <row r="134" ht="16" customHeight="1">
+      <c r="A134" s="9" t="inlineStr">
         <is>
           <t>Ronde van 16  ·  toto 7 pt / exact +4 pt</t>
         </is>
       </c>
     </row>
-    <row r="134" ht="14" customHeight="1">
-      <c r="A134" s="12" t="inlineStr">
+    <row r="135" ht="14" customHeight="1">
+      <c r="A135" s="12" t="inlineStr">
         <is>
           <t>Wedstrijd</t>
         </is>
       </c>
-      <c r="E134" s="12" t="inlineStr">
+      <c r="E135" s="12" t="inlineStr">
         <is>
           <t>voorsp.</t>
         </is>
       </c>
-      <c r="F134" s="12" t="inlineStr">
+      <c r="F135" s="12" t="inlineStr">
         <is>
           <t>uitslag</t>
         </is>
       </c>
-      <c r="G134" s="12" t="inlineStr">
+      <c r="G135" s="12" t="inlineStr">
         <is>
           <t>pt.</t>
         </is>
       </c>
-      <c r="H134" s="60" t="n"/>
-      <c r="I134" s="60" t="n"/>
-      <c r="J134" s="60" t="n"/>
-      <c r="K134" s="60" t="n"/>
-      <c r="L134" s="60" t="n"/>
-      <c r="M134" s="60" t="n"/>
-      <c r="N134" s="60" t="n"/>
-      <c r="O134" s="60" t="n"/>
-    </row>
-    <row r="135" ht="16" customHeight="1">
-      <c r="A135" s="61" t="inlineStr">
+      <c r="H135" s="59" t="n"/>
+      <c r="I135" s="59" t="n"/>
+      <c r="J135" s="59" t="n"/>
+      <c r="K135" s="59" t="n"/>
+      <c r="L135" s="59" t="n"/>
+      <c r="M135" s="59" t="n"/>
+      <c r="N135" s="59" t="n"/>
+      <c r="O135" s="59" t="n"/>
+    </row>
+    <row r="136" ht="16" customHeight="1">
+      <c r="A136" s="60" t="inlineStr">
         <is>
           <t>W32-2  –  W32-5</t>
-        </is>
-      </c>
-      <c r="E135" s="17" t="inlineStr"/>
-      <c r="F135" s="17" t="inlineStr"/>
-      <c r="G135" s="17" t="inlineStr"/>
-    </row>
-    <row r="136" ht="16" customHeight="1">
-      <c r="A136" s="61" t="inlineStr">
-        <is>
-          <t>W32-1  –  W32-3</t>
         </is>
       </c>
       <c r="E136" s="17" t="inlineStr"/>
@@ -3770,9 +3988,9 @@
       <c r="G136" s="17" t="inlineStr"/>
     </row>
     <row r="137" ht="16" customHeight="1">
-      <c r="A137" s="61" t="inlineStr">
-        <is>
-          <t>W32-4  –  W32-6</t>
+      <c r="A137" s="60" t="inlineStr">
+        <is>
+          <t>W32-1  –  W32-3</t>
         </is>
       </c>
       <c r="E137" s="17" t="inlineStr"/>
@@ -3780,9 +3998,9 @@
       <c r="G137" s="17" t="inlineStr"/>
     </row>
     <row r="138" ht="16" customHeight="1">
-      <c r="A138" s="61" t="inlineStr">
-        <is>
-          <t>W32-7  –  W32-8</t>
+      <c r="A138" s="60" t="inlineStr">
+        <is>
+          <t>W32-4  –  W32-6</t>
         </is>
       </c>
       <c r="E138" s="17" t="inlineStr"/>
@@ -3790,9 +4008,9 @@
       <c r="G138" s="17" t="inlineStr"/>
     </row>
     <row r="139" ht="16" customHeight="1">
-      <c r="A139" s="61" t="inlineStr">
-        <is>
-          <t>W32-11  –  W32-12</t>
+      <c r="A139" s="60" t="inlineStr">
+        <is>
+          <t>W32-7  –  W32-8</t>
         </is>
       </c>
       <c r="E139" s="17" t="inlineStr"/>
@@ -3800,9 +4018,9 @@
       <c r="G139" s="17" t="inlineStr"/>
     </row>
     <row r="140" ht="16" customHeight="1">
-      <c r="A140" s="61" t="inlineStr">
-        <is>
-          <t>W32-9  –  W32-10</t>
+      <c r="A140" s="60" t="inlineStr">
+        <is>
+          <t>W32-11  –  W32-12</t>
         </is>
       </c>
       <c r="E140" s="17" t="inlineStr"/>
@@ -3810,9 +4028,9 @@
       <c r="G140" s="17" t="inlineStr"/>
     </row>
     <row r="141" ht="16" customHeight="1">
-      <c r="A141" s="61" t="inlineStr">
-        <is>
-          <t>W32-14  –  W32-16</t>
+      <c r="A141" s="60" t="inlineStr">
+        <is>
+          <t>W32-9  –  W32-10</t>
         </is>
       </c>
       <c r="E141" s="17" t="inlineStr"/>
@@ -3820,67 +4038,67 @@
       <c r="G141" s="17" t="inlineStr"/>
     </row>
     <row r="142" ht="16" customHeight="1">
-      <c r="A142" s="61" t="inlineStr">
-        <is>
-          <t>W32-13  –  W32-15</t>
+      <c r="A142" s="60" t="inlineStr">
+        <is>
+          <t>W32-14  –  W32-16</t>
         </is>
       </c>
       <c r="E142" s="17" t="inlineStr"/>
       <c r="F142" s="17" t="inlineStr"/>
       <c r="G142" s="17" t="inlineStr"/>
     </row>
-    <row r="143" ht="6" customHeight="1"/>
-    <row r="144" ht="16" customHeight="1">
-      <c r="A144" s="9" t="inlineStr">
+    <row r="143" ht="16" customHeight="1">
+      <c r="A143" s="60" t="inlineStr">
+        <is>
+          <t>W32-13  –  W32-15</t>
+        </is>
+      </c>
+      <c r="E143" s="17" t="inlineStr"/>
+      <c r="F143" s="17" t="inlineStr"/>
+      <c r="G143" s="17" t="inlineStr"/>
+    </row>
+    <row r="144" ht="6" customHeight="1"/>
+    <row r="145" ht="16" customHeight="1">
+      <c r="A145" s="9" t="inlineStr">
         <is>
           <t>Kwartfinales  ·  toto 9 pt / exact +5 pt</t>
         </is>
       </c>
     </row>
-    <row r="145" ht="14" customHeight="1">
-      <c r="A145" s="12" t="inlineStr">
+    <row r="146" ht="14" customHeight="1">
+      <c r="A146" s="12" t="inlineStr">
         <is>
           <t>Wedstrijd</t>
         </is>
       </c>
-      <c r="E145" s="12" t="inlineStr">
+      <c r="E146" s="12" t="inlineStr">
         <is>
           <t>voorsp.</t>
         </is>
       </c>
-      <c r="F145" s="12" t="inlineStr">
+      <c r="F146" s="12" t="inlineStr">
         <is>
           <t>uitslag</t>
         </is>
       </c>
-      <c r="G145" s="12" t="inlineStr">
+      <c r="G146" s="12" t="inlineStr">
         <is>
           <t>pt.</t>
         </is>
       </c>
-      <c r="H145" s="60" t="n"/>
-      <c r="I145" s="60" t="n"/>
-      <c r="J145" s="60" t="n"/>
-      <c r="K145" s="60" t="n"/>
-      <c r="L145" s="60" t="n"/>
-      <c r="M145" s="60" t="n"/>
-      <c r="N145" s="60" t="n"/>
-      <c r="O145" s="60" t="n"/>
-    </row>
-    <row r="146" ht="16" customHeight="1">
-      <c r="A146" s="61" t="inlineStr">
+      <c r="H146" s="59" t="n"/>
+      <c r="I146" s="59" t="n"/>
+      <c r="J146" s="59" t="n"/>
+      <c r="K146" s="59" t="n"/>
+      <c r="L146" s="59" t="n"/>
+      <c r="M146" s="59" t="n"/>
+      <c r="N146" s="59" t="n"/>
+      <c r="O146" s="59" t="n"/>
+    </row>
+    <row r="147" ht="16" customHeight="1">
+      <c r="A147" s="60" t="inlineStr">
         <is>
           <t>W16-1  –  W16-2</t>
-        </is>
-      </c>
-      <c r="E146" s="17" t="inlineStr"/>
-      <c r="F146" s="17" t="inlineStr"/>
-      <c r="G146" s="17" t="inlineStr"/>
-    </row>
-    <row r="147" ht="16" customHeight="1">
-      <c r="A147" s="61" t="inlineStr">
-        <is>
-          <t>W16-5  –  W16-6</t>
         </is>
       </c>
       <c r="E147" s="17" t="inlineStr"/>
@@ -3888,9 +4106,9 @@
       <c r="G147" s="17" t="inlineStr"/>
     </row>
     <row r="148" ht="16" customHeight="1">
-      <c r="A148" s="61" t="inlineStr">
-        <is>
-          <t>W16-3  –  W16-4</t>
+      <c r="A148" s="60" t="inlineStr">
+        <is>
+          <t>W16-5  –  W16-6</t>
         </is>
       </c>
       <c r="E148" s="17" t="inlineStr"/>
@@ -3898,1243 +4116,1249 @@
       <c r="G148" s="17" t="inlineStr"/>
     </row>
     <row r="149" ht="16" customHeight="1">
-      <c r="A149" s="61" t="inlineStr">
-        <is>
-          <t>W16-7  –  W16-8</t>
+      <c r="A149" s="60" t="inlineStr">
+        <is>
+          <t>W16-3  –  W16-4</t>
         </is>
       </c>
       <c r="E149" s="17" t="inlineStr"/>
       <c r="F149" s="17" t="inlineStr"/>
       <c r="G149" s="17" t="inlineStr"/>
     </row>
-    <row r="150" ht="6" customHeight="1"/>
-    <row r="151" ht="16" customHeight="1">
-      <c r="A151" s="9" t="inlineStr">
+    <row r="150" ht="16" customHeight="1">
+      <c r="A150" s="60" t="inlineStr">
+        <is>
+          <t>W16-7  –  W16-8</t>
+        </is>
+      </c>
+      <c r="E150" s="17" t="inlineStr"/>
+      <c r="F150" s="17" t="inlineStr"/>
+      <c r="G150" s="17" t="inlineStr"/>
+    </row>
+    <row r="151" ht="6" customHeight="1"/>
+    <row r="152" ht="16" customHeight="1">
+      <c r="A152" s="9" t="inlineStr">
         <is>
           <t>Halve finales  ·  toto 11 pt / exact +6 pt</t>
         </is>
       </c>
     </row>
-    <row r="152" ht="14" customHeight="1">
-      <c r="A152" s="12" t="inlineStr">
+    <row r="153" ht="14" customHeight="1">
+      <c r="A153" s="12" t="inlineStr">
         <is>
           <t>Wedstrijd</t>
         </is>
       </c>
-      <c r="E152" s="12" t="inlineStr">
+      <c r="E153" s="12" t="inlineStr">
         <is>
           <t>voorsp.</t>
         </is>
       </c>
-      <c r="F152" s="12" t="inlineStr">
+      <c r="F153" s="12" t="inlineStr">
         <is>
           <t>uitslag</t>
         </is>
       </c>
-      <c r="G152" s="12" t="inlineStr">
+      <c r="G153" s="12" t="inlineStr">
         <is>
           <t>pt.</t>
         </is>
       </c>
-      <c r="H152" s="60" t="n"/>
-      <c r="I152" s="60" t="n"/>
-      <c r="J152" s="60" t="n"/>
-      <c r="K152" s="60" t="n"/>
-      <c r="L152" s="60" t="n"/>
-      <c r="M152" s="60" t="n"/>
-      <c r="N152" s="60" t="n"/>
-      <c r="O152" s="60" t="n"/>
-    </row>
-    <row r="153" ht="16" customHeight="1">
-      <c r="A153" s="61" t="inlineStr">
+      <c r="H153" s="59" t="n"/>
+      <c r="I153" s="59" t="n"/>
+      <c r="J153" s="59" t="n"/>
+      <c r="K153" s="59" t="n"/>
+      <c r="L153" s="59" t="n"/>
+      <c r="M153" s="59" t="n"/>
+      <c r="N153" s="59" t="n"/>
+      <c r="O153" s="59" t="n"/>
+    </row>
+    <row r="154" ht="16" customHeight="1">
+      <c r="A154" s="60" t="inlineStr">
         <is>
           <t>WKF-1  –  WKF-2</t>
-        </is>
-      </c>
-      <c r="E153" s="17" t="inlineStr"/>
-      <c r="F153" s="17" t="inlineStr"/>
-      <c r="G153" s="17" t="inlineStr"/>
-    </row>
-    <row r="154" ht="16" customHeight="1">
-      <c r="A154" s="61" t="inlineStr">
-        <is>
-          <t>WKF-3  –  WKF-4</t>
         </is>
       </c>
       <c r="E154" s="17" t="inlineStr"/>
       <c r="F154" s="17" t="inlineStr"/>
       <c r="G154" s="17" t="inlineStr"/>
     </row>
-    <row r="155" ht="6" customHeight="1"/>
-    <row r="156" ht="16" customHeight="1">
-      <c r="A156" s="9" t="inlineStr">
+    <row r="155" ht="16" customHeight="1">
+      <c r="A155" s="60" t="inlineStr">
+        <is>
+          <t>WKF-3  –  WKF-4</t>
+        </is>
+      </c>
+      <c r="E155" s="17" t="inlineStr"/>
+      <c r="F155" s="17" t="inlineStr"/>
+      <c r="G155" s="17" t="inlineStr"/>
+    </row>
+    <row r="156" ht="6" customHeight="1"/>
+    <row r="157" ht="16" customHeight="1">
+      <c r="A157" s="9" t="inlineStr">
         <is>
           <t>Finale  ·  toto 13 pt / exact +7 pt</t>
         </is>
       </c>
     </row>
-    <row r="157" ht="14" customHeight="1">
-      <c r="A157" s="12" t="inlineStr">
+    <row r="158" ht="14" customHeight="1">
+      <c r="A158" s="12" t="inlineStr">
         <is>
           <t>Wedstrijd</t>
         </is>
       </c>
-      <c r="E157" s="12" t="inlineStr">
+      <c r="E158" s="12" t="inlineStr">
         <is>
           <t>voorsp.</t>
         </is>
       </c>
-      <c r="F157" s="12" t="inlineStr">
+      <c r="F158" s="12" t="inlineStr">
         <is>
           <t>uitslag</t>
         </is>
       </c>
-      <c r="G157" s="12" t="inlineStr">
+      <c r="G158" s="12" t="inlineStr">
         <is>
           <t>pt.</t>
         </is>
       </c>
-      <c r="H157" s="60" t="n"/>
-      <c r="I157" s="60" t="n"/>
-      <c r="J157" s="60" t="n"/>
-      <c r="K157" s="60" t="n"/>
-      <c r="L157" s="60" t="n"/>
-      <c r="M157" s="60" t="n"/>
-      <c r="N157" s="60" t="n"/>
-      <c r="O157" s="60" t="n"/>
-    </row>
-    <row r="158" ht="16" customHeight="1">
-      <c r="A158" s="61" t="inlineStr">
+      <c r="H158" s="59" t="n"/>
+      <c r="I158" s="59" t="n"/>
+      <c r="J158" s="59" t="n"/>
+      <c r="K158" s="59" t="n"/>
+      <c r="L158" s="59" t="n"/>
+      <c r="M158" s="59" t="n"/>
+      <c r="N158" s="59" t="n"/>
+      <c r="O158" s="59" t="n"/>
+    </row>
+    <row r="159" ht="16" customHeight="1">
+      <c r="A159" s="60" t="inlineStr">
         <is>
           <t>WHF-1  –  WHF-2</t>
         </is>
       </c>
-      <c r="E158" s="17" t="inlineStr"/>
-      <c r="F158" s="17" t="inlineStr"/>
-      <c r="G158" s="17" t="inlineStr"/>
-    </row>
-    <row r="159" ht="6" customHeight="1"/>
-    <row r="160" ht="8" customHeight="1"/>
-    <row r="161" ht="18" customHeight="1">
-      <c r="A161" s="3" t="inlineStr">
+      <c r="E159" s="17" t="inlineStr"/>
+      <c r="F159" s="17" t="inlineStr"/>
+      <c r="G159" s="17" t="inlineStr"/>
+    </row>
+    <row r="160" ht="6" customHeight="1"/>
+    <row r="161" ht="8" customHeight="1"/>
+    <row r="162" ht="18" customHeight="1">
+      <c r="A162" s="3" t="inlineStr">
         <is>
           <t>▶  VERRASSING — kies een land BUITEN de top-12 · punten schalen met ranking en ronde</t>
         </is>
       </c>
     </row>
-    <row r="162" ht="14" customHeight="1">
-      <c r="A162" s="12" t="inlineStr">
+    <row r="163" ht="14" customHeight="1">
+      <c r="A163" s="12" t="inlineStr">
         <is>
           <t>Land (outsider)</t>
         </is>
       </c>
-      <c r="E162" s="12" t="inlineStr">
+      <c r="E163" s="12" t="inlineStr">
         <is>
           <t>R16</t>
         </is>
       </c>
-      <c r="F162" s="12" t="inlineStr">
+      <c r="F163" s="12" t="inlineStr">
         <is>
           <t>KF</t>
         </is>
       </c>
-      <c r="G162" s="12" t="inlineStr">
+      <c r="G163" s="12" t="inlineStr">
         <is>
           <t>HF</t>
         </is>
       </c>
-      <c r="H162" s="12" t="inlineStr">
+      <c r="H163" s="12" t="inlineStr">
         <is>
           <t>Finale</t>
         </is>
       </c>
-      <c r="I162" s="12" t="inlineStr">
+      <c r="I163" s="12" t="inlineStr">
         <is>
           <t>Winnaar</t>
         </is>
-      </c>
-    </row>
-    <row r="163" ht="15" customHeight="1">
-      <c r="A163" s="14" t="inlineStr">
-        <is>
-          <t>Senegal</t>
-        </is>
-      </c>
-      <c r="E163" s="62" t="n">
-        <v>7</v>
-      </c>
-      <c r="F163" s="62" t="n">
-        <v>12</v>
-      </c>
-      <c r="G163" s="62" t="n">
-        <v>19</v>
-      </c>
-      <c r="H163" s="62" t="n">
-        <v>26</v>
-      </c>
-      <c r="I163" s="62" t="n">
-        <v>34</v>
       </c>
     </row>
     <row r="164" ht="15" customHeight="1">
       <c r="A164" s="14" t="inlineStr">
         <is>
-          <t>Mexico</t>
-        </is>
-      </c>
-      <c r="E164" s="62" t="n">
+          <t>Senegal</t>
+        </is>
+      </c>
+      <c r="E164" s="61" t="n">
         <v>7</v>
       </c>
-      <c r="F164" s="62" t="n">
-        <v>13</v>
-      </c>
-      <c r="G164" s="62" t="n">
+      <c r="F164" s="61" t="n">
+        <v>12</v>
+      </c>
+      <c r="G164" s="61" t="n">
         <v>19</v>
       </c>
-      <c r="H164" s="62" t="n">
-        <v>27</v>
-      </c>
-      <c r="I164" s="62" t="n">
-        <v>35</v>
+      <c r="H164" s="61" t="n">
+        <v>26</v>
+      </c>
+      <c r="I164" s="61" t="n">
+        <v>34</v>
       </c>
     </row>
     <row r="165" ht="15" customHeight="1">
       <c r="A165" s="14" t="inlineStr">
         <is>
-          <t>Verenigde Staten</t>
-        </is>
-      </c>
-      <c r="E165" s="62" t="n">
-        <v>8</v>
-      </c>
-      <c r="F165" s="62" t="n">
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="E165" s="61" t="n">
+        <v>7</v>
+      </c>
+      <c r="F165" s="61" t="n">
         <v>13</v>
       </c>
-      <c r="G165" s="62" t="n">
-        <v>20</v>
-      </c>
-      <c r="H165" s="62" t="n">
+      <c r="G165" s="61" t="n">
+        <v>19</v>
+      </c>
+      <c r="H165" s="61" t="n">
         <v>27</v>
       </c>
-      <c r="I165" s="62" t="n">
-        <v>36</v>
+      <c r="I165" s="61" t="n">
+        <v>35</v>
       </c>
     </row>
     <row r="166" ht="15" customHeight="1">
       <c r="A166" s="14" t="inlineStr">
         <is>
-          <t>Uruguay</t>
-        </is>
-      </c>
-      <c r="E166" s="62" t="n">
+          <t>Verenigde Staten</t>
+        </is>
+      </c>
+      <c r="E166" s="61" t="n">
         <v>8</v>
       </c>
-      <c r="F166" s="62" t="n">
-        <v>14</v>
-      </c>
-      <c r="G166" s="62" t="n">
+      <c r="F166" s="61" t="n">
+        <v>13</v>
+      </c>
+      <c r="G166" s="61" t="n">
         <v>20</v>
       </c>
-      <c r="H166" s="62" t="n">
-        <v>28</v>
-      </c>
-      <c r="I166" s="62" t="n">
-        <v>37</v>
+      <c r="H166" s="61" t="n">
+        <v>27</v>
+      </c>
+      <c r="I166" s="61" t="n">
+        <v>36</v>
       </c>
     </row>
     <row r="167" ht="15" customHeight="1">
       <c r="A167" s="14" t="inlineStr">
         <is>
-          <t>Japan</t>
-        </is>
-      </c>
-      <c r="E167" s="62" t="n">
+          <t>Uruguay</t>
+        </is>
+      </c>
+      <c r="E167" s="61" t="n">
         <v>8</v>
       </c>
-      <c r="F167" s="62" t="n">
+      <c r="F167" s="61" t="n">
         <v>14</v>
       </c>
-      <c r="G167" s="62" t="n">
-        <v>21</v>
-      </c>
-      <c r="H167" s="62" t="n">
-        <v>29</v>
-      </c>
-      <c r="I167" s="62" t="n">
-        <v>38</v>
+      <c r="G167" s="61" t="n">
+        <v>20</v>
+      </c>
+      <c r="H167" s="61" t="n">
+        <v>28</v>
+      </c>
+      <c r="I167" s="61" t="n">
+        <v>37</v>
       </c>
     </row>
     <row r="168" ht="15" customHeight="1">
       <c r="A168" s="14" t="inlineStr">
         <is>
-          <t>Zwitserland</t>
-        </is>
-      </c>
-      <c r="E168" s="62" t="n">
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="E168" s="61" t="n">
         <v>8</v>
       </c>
-      <c r="F168" s="62" t="n">
+      <c r="F168" s="61" t="n">
         <v>14</v>
       </c>
-      <c r="G168" s="62" t="n">
+      <c r="G168" s="61" t="n">
         <v>21</v>
       </c>
-      <c r="H168" s="62" t="n">
-        <v>30</v>
-      </c>
-      <c r="I168" s="62" t="n">
-        <v>39</v>
+      <c r="H168" s="61" t="n">
+        <v>29</v>
+      </c>
+      <c r="I168" s="61" t="n">
+        <v>38</v>
       </c>
     </row>
     <row r="169" ht="15" customHeight="1">
       <c r="A169" s="14" t="inlineStr">
         <is>
-          <t>Iran</t>
-        </is>
-      </c>
-      <c r="E169" s="62" t="n">
-        <v>9</v>
-      </c>
-      <c r="F169" s="62" t="n">
-        <v>15</v>
-      </c>
-      <c r="G169" s="62" t="n">
-        <v>22</v>
-      </c>
-      <c r="H169" s="62" t="n">
-        <v>31</v>
-      </c>
-      <c r="I169" s="62" t="n">
-        <v>41</v>
+          <t>Zwitserland</t>
+        </is>
+      </c>
+      <c r="E169" s="61" t="n">
+        <v>8</v>
+      </c>
+      <c r="F169" s="61" t="n">
+        <v>14</v>
+      </c>
+      <c r="G169" s="61" t="n">
+        <v>21</v>
+      </c>
+      <c r="H169" s="61" t="n">
+        <v>30</v>
+      </c>
+      <c r="I169" s="61" t="n">
+        <v>39</v>
       </c>
     </row>
     <row r="170" ht="15" customHeight="1">
       <c r="A170" s="14" t="inlineStr">
         <is>
-          <t>Oostenrijk</t>
-        </is>
-      </c>
-      <c r="E170" s="62" t="n">
+          <t>Iran</t>
+        </is>
+      </c>
+      <c r="E170" s="61" t="n">
         <v>9</v>
       </c>
-      <c r="F170" s="62" t="n">
+      <c r="F170" s="61" t="n">
         <v>15</v>
       </c>
-      <c r="G170" s="62" t="n">
-        <v>23</v>
-      </c>
-      <c r="H170" s="62" t="n">
-        <v>32</v>
-      </c>
-      <c r="I170" s="62" t="n">
-        <v>42</v>
+      <c r="G170" s="61" t="n">
+        <v>22</v>
+      </c>
+      <c r="H170" s="61" t="n">
+        <v>31</v>
+      </c>
+      <c r="I170" s="61" t="n">
+        <v>41</v>
       </c>
     </row>
     <row r="171" ht="15" customHeight="1">
       <c r="A171" s="14" t="inlineStr">
         <is>
-          <t>Zuid-Korea</t>
-        </is>
-      </c>
-      <c r="E171" s="62" t="n">
+          <t>Oostenrijk</t>
+        </is>
+      </c>
+      <c r="E171" s="61" t="n">
         <v>9</v>
       </c>
-      <c r="F171" s="62" t="n">
-        <v>16</v>
-      </c>
-      <c r="G171" s="62" t="n">
+      <c r="F171" s="61" t="n">
+        <v>15</v>
+      </c>
+      <c r="G171" s="61" t="n">
         <v>23</v>
       </c>
-      <c r="H171" s="62" t="n">
+      <c r="H171" s="61" t="n">
         <v>32</v>
       </c>
-      <c r="I171" s="62" t="n">
-        <v>43</v>
+      <c r="I171" s="61" t="n">
+        <v>42</v>
       </c>
     </row>
     <row r="172" ht="15" customHeight="1">
       <c r="A172" s="14" t="inlineStr">
         <is>
-          <t>Australië</t>
-        </is>
-      </c>
-      <c r="E172" s="62" t="n">
+          <t>Zuid-Korea</t>
+        </is>
+      </c>
+      <c r="E172" s="61" t="n">
         <v>9</v>
       </c>
-      <c r="F172" s="62" t="n">
+      <c r="F172" s="61" t="n">
         <v>16</v>
       </c>
-      <c r="G172" s="62" t="n">
-        <v>24</v>
-      </c>
-      <c r="H172" s="62" t="n">
-        <v>33</v>
-      </c>
-      <c r="I172" s="62" t="n">
+      <c r="G172" s="61" t="n">
+        <v>23</v>
+      </c>
+      <c r="H172" s="61" t="n">
+        <v>32</v>
+      </c>
+      <c r="I172" s="61" t="n">
         <v>43</v>
       </c>
     </row>
     <row r="173" ht="15" customHeight="1">
       <c r="A173" s="14" t="inlineStr">
         <is>
-          <t>Ecuador</t>
-        </is>
-      </c>
-      <c r="E173" s="62" t="n">
+          <t>Australië</t>
+        </is>
+      </c>
+      <c r="E173" s="61" t="n">
         <v>9</v>
       </c>
-      <c r="F173" s="62" t="n">
+      <c r="F173" s="61" t="n">
         <v>16</v>
       </c>
-      <c r="G173" s="62" t="n">
+      <c r="G173" s="61" t="n">
         <v>24</v>
       </c>
-      <c r="H173" s="62" t="n">
-        <v>34</v>
-      </c>
-      <c r="I173" s="62" t="n">
-        <v>44</v>
+      <c r="H173" s="61" t="n">
+        <v>33</v>
+      </c>
+      <c r="I173" s="61" t="n">
+        <v>43</v>
       </c>
     </row>
     <row r="174" ht="15" customHeight="1">
       <c r="A174" s="14" t="inlineStr">
         <is>
-          <t>Noorwegen</t>
-        </is>
-      </c>
-      <c r="E174" s="62" t="n">
-        <v>10</v>
-      </c>
-      <c r="F174" s="62" t="n">
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="E174" s="61" t="n">
+        <v>9</v>
+      </c>
+      <c r="F174" s="61" t="n">
         <v>16</v>
       </c>
-      <c r="G174" s="62" t="n">
-        <v>25</v>
-      </c>
-      <c r="H174" s="62" t="n">
+      <c r="G174" s="61" t="n">
+        <v>24</v>
+      </c>
+      <c r="H174" s="61" t="n">
         <v>34</v>
       </c>
-      <c r="I174" s="62" t="n">
-        <v>45</v>
+      <c r="I174" s="61" t="n">
+        <v>44</v>
       </c>
     </row>
     <row r="175" ht="15" customHeight="1">
       <c r="A175" s="14" t="inlineStr">
         <is>
-          <t>Panama</t>
-        </is>
-      </c>
-      <c r="E175" s="62" t="n">
+          <t>Noorwegen</t>
+        </is>
+      </c>
+      <c r="E175" s="61" t="n">
         <v>10</v>
       </c>
-      <c r="F175" s="62" t="n">
-        <v>17</v>
-      </c>
-      <c r="G175" s="62" t="n">
-        <v>26</v>
-      </c>
-      <c r="H175" s="62" t="n">
-        <v>36</v>
-      </c>
-      <c r="I175" s="62" t="n">
-        <v>48</v>
+      <c r="F175" s="61" t="n">
+        <v>16</v>
+      </c>
+      <c r="G175" s="61" t="n">
+        <v>25</v>
+      </c>
+      <c r="H175" s="61" t="n">
+        <v>34</v>
+      </c>
+      <c r="I175" s="61" t="n">
+        <v>45</v>
       </c>
     </row>
     <row r="176" ht="15" customHeight="1">
       <c r="A176" s="14" t="inlineStr">
         <is>
-          <t>Egypte</t>
-        </is>
-      </c>
-      <c r="E176" s="62" t="n">
+          <t>Panama</t>
+        </is>
+      </c>
+      <c r="E176" s="61" t="n">
         <v>10</v>
       </c>
-      <c r="F176" s="62" t="n">
-        <v>18</v>
-      </c>
-      <c r="G176" s="62" t="n">
-        <v>27</v>
-      </c>
-      <c r="H176" s="62" t="n">
-        <v>37</v>
-      </c>
-      <c r="I176" s="62" t="n">
-        <v>49</v>
+      <c r="F176" s="61" t="n">
+        <v>17</v>
+      </c>
+      <c r="G176" s="61" t="n">
+        <v>26</v>
+      </c>
+      <c r="H176" s="61" t="n">
+        <v>36</v>
+      </c>
+      <c r="I176" s="61" t="n">
+        <v>48</v>
       </c>
     </row>
     <row r="177" ht="15" customHeight="1">
       <c r="A177" s="14" t="inlineStr">
         <is>
-          <t>Algerije</t>
-        </is>
-      </c>
-      <c r="E177" s="62" t="n">
-        <v>11</v>
-      </c>
-      <c r="F177" s="62" t="n">
-        <v>19</v>
-      </c>
-      <c r="G177" s="62" t="n">
-        <v>28</v>
-      </c>
-      <c r="H177" s="62" t="n">
-        <v>40</v>
-      </c>
-      <c r="I177" s="62" t="n">
-        <v>52</v>
+          <t>Egypte</t>
+        </is>
+      </c>
+      <c r="E177" s="61" t="n">
+        <v>10</v>
+      </c>
+      <c r="F177" s="61" t="n">
+        <v>18</v>
+      </c>
+      <c r="G177" s="61" t="n">
+        <v>27</v>
+      </c>
+      <c r="H177" s="61" t="n">
+        <v>37</v>
+      </c>
+      <c r="I177" s="61" t="n">
+        <v>49</v>
       </c>
     </row>
     <row r="178" ht="15" customHeight="1">
       <c r="A178" s="14" t="inlineStr">
         <is>
-          <t>Paraguay</t>
-        </is>
-      </c>
-      <c r="E178" s="62" t="n">
+          <t>Algerije</t>
+        </is>
+      </c>
+      <c r="E178" s="61" t="n">
         <v>11</v>
       </c>
-      <c r="F178" s="62" t="n">
+      <c r="F178" s="61" t="n">
         <v>19</v>
       </c>
-      <c r="G178" s="62" t="n">
-        <v>29</v>
-      </c>
-      <c r="H178" s="62" t="n">
-        <v>41</v>
-      </c>
-      <c r="I178" s="62" t="n">
-        <v>53</v>
+      <c r="G178" s="61" t="n">
+        <v>28</v>
+      </c>
+      <c r="H178" s="61" t="n">
+        <v>40</v>
+      </c>
+      <c r="I178" s="61" t="n">
+        <v>52</v>
       </c>
     </row>
     <row r="179" ht="15" customHeight="1">
       <c r="A179" s="14" t="inlineStr">
         <is>
-          <t>Ivoorkust</t>
-        </is>
-      </c>
-      <c r="E179" s="62" t="n">
-        <v>12</v>
-      </c>
-      <c r="F179" s="62" t="n">
-        <v>20</v>
-      </c>
-      <c r="G179" s="62" t="n">
-        <v>30</v>
-      </c>
-      <c r="H179" s="62" t="n">
+          <t>Paraguay</t>
+        </is>
+      </c>
+      <c r="E179" s="61" t="n">
+        <v>11</v>
+      </c>
+      <c r="F179" s="61" t="n">
+        <v>19</v>
+      </c>
+      <c r="G179" s="61" t="n">
+        <v>29</v>
+      </c>
+      <c r="H179" s="61" t="n">
         <v>41</v>
       </c>
-      <c r="I179" s="62" t="n">
-        <v>55</v>
+      <c r="I179" s="61" t="n">
+        <v>53</v>
       </c>
     </row>
     <row r="180" ht="15" customHeight="1">
       <c r="A180" s="14" t="inlineStr">
         <is>
-          <t>Tunesië</t>
-        </is>
-      </c>
-      <c r="E180" s="62" t="n">
+          <t>Ivoorkust</t>
+        </is>
+      </c>
+      <c r="E180" s="61" t="n">
         <v>12</v>
       </c>
-      <c r="F180" s="62" t="n">
+      <c r="F180" s="61" t="n">
         <v>20</v>
       </c>
-      <c r="G180" s="62" t="n">
+      <c r="G180" s="61" t="n">
         <v>30</v>
       </c>
-      <c r="H180" s="62" t="n">
-        <v>42</v>
-      </c>
-      <c r="I180" s="62" t="n">
+      <c r="H180" s="61" t="n">
+        <v>41</v>
+      </c>
+      <c r="I180" s="61" t="n">
         <v>55</v>
       </c>
     </row>
     <row r="181" ht="15" customHeight="1">
       <c r="A181" s="14" t="inlineStr">
         <is>
-          <t>Schotland</t>
-        </is>
-      </c>
-      <c r="E181" s="62" t="n">
+          <t>Tunesië</t>
+        </is>
+      </c>
+      <c r="E181" s="61" t="n">
         <v>12</v>
       </c>
-      <c r="F181" s="62" t="n">
+      <c r="F181" s="61" t="n">
         <v>20</v>
       </c>
-      <c r="G181" s="62" t="n">
-        <v>31</v>
-      </c>
-      <c r="H181" s="62" t="n">
+      <c r="G181" s="61" t="n">
+        <v>30</v>
+      </c>
+      <c r="H181" s="61" t="n">
         <v>42</v>
       </c>
-      <c r="I181" s="62" t="n">
-        <v>56</v>
+      <c r="I181" s="61" t="n">
+        <v>55</v>
       </c>
     </row>
     <row r="182" ht="15" customHeight="1">
       <c r="A182" s="14" t="inlineStr">
         <is>
-          <t>Zweden</t>
-        </is>
-      </c>
-      <c r="E182" s="62" t="n">
+          <t>Schotland</t>
+        </is>
+      </c>
+      <c r="E182" s="61" t="n">
         <v>12</v>
       </c>
-      <c r="F182" s="62" t="n">
-        <v>21</v>
-      </c>
-      <c r="G182" s="62" t="n">
+      <c r="F182" s="61" t="n">
+        <v>20</v>
+      </c>
+      <c r="G182" s="61" t="n">
         <v>31</v>
       </c>
-      <c r="H182" s="62" t="n">
-        <v>43</v>
-      </c>
-      <c r="I182" s="62" t="n">
-        <v>57</v>
+      <c r="H182" s="61" t="n">
+        <v>42</v>
+      </c>
+      <c r="I182" s="61" t="n">
+        <v>56</v>
       </c>
     </row>
     <row r="183" ht="15" customHeight="1">
       <c r="A183" s="14" t="inlineStr">
         <is>
-          <t>Tsjechië</t>
-        </is>
-      </c>
-      <c r="E183" s="62" t="n">
+          <t>Zweden</t>
+        </is>
+      </c>
+      <c r="E183" s="61" t="n">
         <v>12</v>
       </c>
-      <c r="F183" s="62" t="n">
+      <c r="F183" s="61" t="n">
         <v>21</v>
       </c>
-      <c r="G183" s="62" t="n">
+      <c r="G183" s="61" t="n">
         <v>31</v>
       </c>
-      <c r="H183" s="62" t="n">
+      <c r="H183" s="61" t="n">
         <v>43</v>
       </c>
-      <c r="I183" s="62" t="n">
+      <c r="I183" s="61" t="n">
         <v>57</v>
       </c>
     </row>
     <row r="184" ht="15" customHeight="1">
       <c r="A184" s="14" t="inlineStr">
         <is>
-          <t>Qatar</t>
-        </is>
-      </c>
-      <c r="E184" s="62" t="n">
-        <v>13</v>
-      </c>
-      <c r="F184" s="62" t="n">
-        <v>22</v>
-      </c>
-      <c r="G184" s="62" t="n">
-        <v>33</v>
-      </c>
-      <c r="H184" s="62" t="n">
-        <v>46</v>
-      </c>
-      <c r="I184" s="62" t="n">
-        <v>61</v>
+          <t>Tsjechië</t>
+        </is>
+      </c>
+      <c r="E184" s="61" t="n">
+        <v>12</v>
+      </c>
+      <c r="F184" s="61" t="n">
+        <v>21</v>
+      </c>
+      <c r="G184" s="61" t="n">
+        <v>31</v>
+      </c>
+      <c r="H184" s="61" t="n">
+        <v>43</v>
+      </c>
+      <c r="I184" s="61" t="n">
+        <v>57</v>
       </c>
     </row>
     <row r="185" ht="15" customHeight="1">
       <c r="A185" s="14" t="inlineStr">
         <is>
-          <t>Oezbekistan</t>
-        </is>
-      </c>
-      <c r="E185" s="62" t="n">
+          <t>Qatar</t>
+        </is>
+      </c>
+      <c r="E185" s="61" t="n">
         <v>13</v>
       </c>
-      <c r="F185" s="62" t="n">
-        <v>23</v>
-      </c>
-      <c r="G185" s="62" t="n">
-        <v>34</v>
-      </c>
-      <c r="H185" s="62" t="n">
-        <v>47</v>
-      </c>
-      <c r="I185" s="62" t="n">
-        <v>63</v>
+      <c r="F185" s="61" t="n">
+        <v>22</v>
+      </c>
+      <c r="G185" s="61" t="n">
+        <v>33</v>
+      </c>
+      <c r="H185" s="61" t="n">
+        <v>46</v>
+      </c>
+      <c r="I185" s="61" t="n">
+        <v>61</v>
       </c>
     </row>
     <row r="186" ht="15" customHeight="1">
       <c r="A186" s="14" t="inlineStr">
         <is>
-          <t>DR Congo</t>
-        </is>
-      </c>
-      <c r="E186" s="62" t="n">
-        <v>14</v>
-      </c>
-      <c r="F186" s="62" t="n">
+          <t>Oezbekistan</t>
+        </is>
+      </c>
+      <c r="E186" s="61" t="n">
+        <v>13</v>
+      </c>
+      <c r="F186" s="61" t="n">
         <v>23</v>
       </c>
-      <c r="G186" s="62" t="n">
-        <v>35</v>
-      </c>
-      <c r="H186" s="62" t="n">
-        <v>48</v>
-      </c>
-      <c r="I186" s="62" t="n">
-        <v>64</v>
+      <c r="G186" s="61" t="n">
+        <v>34</v>
+      </c>
+      <c r="H186" s="61" t="n">
+        <v>47</v>
+      </c>
+      <c r="I186" s="61" t="n">
+        <v>63</v>
       </c>
     </row>
     <row r="187" ht="15" customHeight="1">
       <c r="A187" s="14" t="inlineStr">
         <is>
-          <t>Saoedi-Arabië</t>
-        </is>
-      </c>
-      <c r="E187" s="62" t="n">
+          <t>DR Congo</t>
+        </is>
+      </c>
+      <c r="E187" s="61" t="n">
         <v>14</v>
       </c>
-      <c r="F187" s="62" t="n">
-        <v>24</v>
-      </c>
-      <c r="G187" s="62" t="n">
+      <c r="F187" s="61" t="n">
+        <v>23</v>
+      </c>
+      <c r="G187" s="61" t="n">
         <v>35</v>
       </c>
-      <c r="H187" s="62" t="n">
-        <v>49</v>
-      </c>
-      <c r="I187" s="62" t="n">
-        <v>65</v>
+      <c r="H187" s="61" t="n">
+        <v>48</v>
+      </c>
+      <c r="I187" s="61" t="n">
+        <v>64</v>
       </c>
     </row>
     <row r="188" ht="15" customHeight="1">
       <c r="A188" s="14" t="inlineStr">
         <is>
-          <t>Irak</t>
-        </is>
-      </c>
-      <c r="E188" s="62" t="n">
+          <t>Saoedi-Arabië</t>
+        </is>
+      </c>
+      <c r="E188" s="61" t="n">
         <v>14</v>
       </c>
-      <c r="F188" s="62" t="n">
+      <c r="F188" s="61" t="n">
         <v>24</v>
       </c>
-      <c r="G188" s="62" t="n">
-        <v>36</v>
-      </c>
-      <c r="H188" s="62" t="n">
+      <c r="G188" s="61" t="n">
+        <v>35</v>
+      </c>
+      <c r="H188" s="61" t="n">
         <v>49</v>
       </c>
-      <c r="I188" s="62" t="n">
+      <c r="I188" s="61" t="n">
         <v>65</v>
       </c>
     </row>
     <row r="189" ht="15" customHeight="1">
       <c r="A189" s="14" t="inlineStr">
         <is>
-          <t>Zuid-Afrika</t>
-        </is>
-      </c>
-      <c r="E189" s="62" t="n">
+          <t>Irak</t>
+        </is>
+      </c>
+      <c r="E189" s="61" t="n">
         <v>14</v>
       </c>
-      <c r="F189" s="62" t="n">
+      <c r="F189" s="61" t="n">
         <v>24</v>
       </c>
-      <c r="G189" s="62" t="n">
+      <c r="G189" s="61" t="n">
         <v>36</v>
       </c>
-      <c r="H189" s="62" t="n">
-        <v>50</v>
-      </c>
-      <c r="I189" s="62" t="n">
-        <v>66</v>
+      <c r="H189" s="61" t="n">
+        <v>49</v>
+      </c>
+      <c r="I189" s="61" t="n">
+        <v>65</v>
       </c>
     </row>
     <row r="190" ht="15" customHeight="1">
       <c r="A190" s="14" t="inlineStr">
         <is>
-          <t>Jordanië</t>
-        </is>
-      </c>
-      <c r="E190" s="62" t="n">
+          <t>Zuid-Afrika</t>
+        </is>
+      </c>
+      <c r="E190" s="61" t="n">
         <v>14</v>
       </c>
-      <c r="F190" s="62" t="n">
-        <v>25</v>
-      </c>
-      <c r="G190" s="62" t="n">
-        <v>37</v>
-      </c>
-      <c r="H190" s="62" t="n">
-        <v>51</v>
-      </c>
-      <c r="I190" s="62" t="n">
-        <v>68</v>
+      <c r="F190" s="61" t="n">
+        <v>24</v>
+      </c>
+      <c r="G190" s="61" t="n">
+        <v>36</v>
+      </c>
+      <c r="H190" s="61" t="n">
+        <v>50</v>
+      </c>
+      <c r="I190" s="61" t="n">
+        <v>66</v>
       </c>
     </row>
     <row r="191" ht="15" customHeight="1">
       <c r="A191" s="14" t="inlineStr">
         <is>
-          <t>Kaapverdië</t>
-        </is>
-      </c>
-      <c r="E191" s="62" t="n">
-        <v>15</v>
-      </c>
-      <c r="F191" s="62" t="n">
-        <v>26</v>
-      </c>
-      <c r="G191" s="62" t="n">
-        <v>38</v>
-      </c>
-      <c r="H191" s="62" t="n">
-        <v>53</v>
-      </c>
-      <c r="I191" s="62" t="n">
-        <v>70</v>
+          <t>Jordanië</t>
+        </is>
+      </c>
+      <c r="E191" s="61" t="n">
+        <v>14</v>
+      </c>
+      <c r="F191" s="61" t="n">
+        <v>25</v>
+      </c>
+      <c r="G191" s="61" t="n">
+        <v>37</v>
+      </c>
+      <c r="H191" s="61" t="n">
+        <v>51</v>
+      </c>
+      <c r="I191" s="61" t="n">
+        <v>68</v>
       </c>
     </row>
     <row r="192" ht="15" customHeight="1">
       <c r="A192" s="14" t="inlineStr">
         <is>
-          <t>Ghana</t>
-        </is>
-      </c>
-      <c r="E192" s="62" t="n">
+          <t>Kaapverdië</t>
+        </is>
+      </c>
+      <c r="E192" s="61" t="n">
         <v>15</v>
       </c>
-      <c r="F192" s="62" t="n">
+      <c r="F192" s="61" t="n">
         <v>26</v>
       </c>
-      <c r="G192" s="62" t="n">
-        <v>39</v>
-      </c>
-      <c r="H192" s="62" t="n">
-        <v>54</v>
-      </c>
-      <c r="I192" s="62" t="n">
-        <v>72</v>
+      <c r="G192" s="61" t="n">
+        <v>38</v>
+      </c>
+      <c r="H192" s="61" t="n">
+        <v>53</v>
+      </c>
+      <c r="I192" s="61" t="n">
+        <v>70</v>
       </c>
     </row>
     <row r="193" ht="15" customHeight="1">
       <c r="A193" s="14" t="inlineStr">
         <is>
-          <t>Bosnië-Herzegovina</t>
-        </is>
-      </c>
-      <c r="E193" s="62" t="n">
+          <t>Ghana</t>
+        </is>
+      </c>
+      <c r="E193" s="61" t="n">
         <v>15</v>
       </c>
-      <c r="F193" s="62" t="n">
+      <c r="F193" s="61" t="n">
         <v>26</v>
       </c>
-      <c r="G193" s="62" t="n">
+      <c r="G193" s="61" t="n">
         <v>39</v>
       </c>
-      <c r="H193" s="62" t="n">
-        <v>55</v>
-      </c>
-      <c r="I193" s="62" t="n">
+      <c r="H193" s="61" t="n">
+        <v>54</v>
+      </c>
+      <c r="I193" s="61" t="n">
         <v>72</v>
       </c>
     </row>
     <row r="194" ht="15" customHeight="1">
       <c r="A194" s="14" t="inlineStr">
         <is>
-          <t>Haïti</t>
-        </is>
-      </c>
-      <c r="E194" s="62" t="n">
-        <v>16</v>
-      </c>
-      <c r="F194" s="62" t="n">
-        <v>28</v>
-      </c>
-      <c r="G194" s="62" t="n">
-        <v>41</v>
-      </c>
-      <c r="H194" s="62" t="n">
-        <v>58</v>
-      </c>
-      <c r="I194" s="62" t="n">
-        <v>76</v>
+          <t>Bosnië-Herzegovina</t>
+        </is>
+      </c>
+      <c r="E194" s="61" t="n">
+        <v>15</v>
+      </c>
+      <c r="F194" s="61" t="n">
+        <v>26</v>
+      </c>
+      <c r="G194" s="61" t="n">
+        <v>39</v>
+      </c>
+      <c r="H194" s="61" t="n">
+        <v>55</v>
+      </c>
+      <c r="I194" s="61" t="n">
+        <v>72</v>
       </c>
     </row>
     <row r="195" ht="15" customHeight="1">
       <c r="A195" s="14" t="inlineStr">
         <is>
-          <t>Nieuw-Zeeland</t>
-        </is>
-      </c>
-      <c r="E195" s="62" t="n">
+          <t>Haïti</t>
+        </is>
+      </c>
+      <c r="E195" s="61" t="n">
         <v>16</v>
       </c>
-      <c r="F195" s="62" t="n">
+      <c r="F195" s="61" t="n">
         <v>28</v>
       </c>
-      <c r="G195" s="62" t="n">
-        <v>42</v>
-      </c>
-      <c r="H195" s="62" t="n">
-        <v>59</v>
-      </c>
-      <c r="I195" s="62" t="n">
-        <v>77</v>
+      <c r="G195" s="61" t="n">
+        <v>41</v>
+      </c>
+      <c r="H195" s="61" t="n">
+        <v>58</v>
+      </c>
+      <c r="I195" s="61" t="n">
+        <v>76</v>
       </c>
     </row>
     <row r="196" ht="15" customHeight="1">
       <c r="A196" s="14" t="inlineStr">
         <is>
-          <t>Curaçao</t>
-        </is>
-      </c>
-      <c r="E196" s="62" t="n">
-        <v>17</v>
-      </c>
-      <c r="F196" s="62" t="n">
-        <v>29</v>
-      </c>
-      <c r="G196" s="62" t="n">
-        <v>43</v>
-      </c>
-      <c r="H196" s="62" t="n">
-        <v>60</v>
-      </c>
-      <c r="I196" s="62" t="n">
-        <v>79</v>
+          <t>Nieuw-Zeeland</t>
+        </is>
+      </c>
+      <c r="E196" s="61" t="n">
+        <v>16</v>
+      </c>
+      <c r="F196" s="61" t="n">
+        <v>28</v>
+      </c>
+      <c r="G196" s="61" t="n">
+        <v>42</v>
+      </c>
+      <c r="H196" s="61" t="n">
+        <v>59</v>
+      </c>
+      <c r="I196" s="61" t="n">
+        <v>77</v>
       </c>
     </row>
     <row r="197" ht="15" customHeight="1">
       <c r="A197" s="14" t="inlineStr">
         <is>
-          <t>Canada</t>
-        </is>
-      </c>
-      <c r="E197" s="62" t="n">
-        <v>13</v>
-      </c>
-      <c r="F197" s="62" t="n">
-        <v>22</v>
-      </c>
-      <c r="G197" s="62" t="n">
-        <v>33</v>
-      </c>
-      <c r="H197" s="62" t="n">
-        <v>46</v>
-      </c>
-      <c r="I197" s="62" t="n">
-        <v>61</v>
+          <t>Curaçao</t>
+        </is>
+      </c>
+      <c r="E197" s="61" t="n">
+        <v>17</v>
+      </c>
+      <c r="F197" s="61" t="n">
+        <v>29</v>
+      </c>
+      <c r="G197" s="61" t="n">
+        <v>43</v>
+      </c>
+      <c r="H197" s="61" t="n">
+        <v>60</v>
+      </c>
+      <c r="I197" s="61" t="n">
+        <v>79</v>
       </c>
     </row>
     <row r="198" ht="15" customHeight="1">
       <c r="A198" s="14" t="inlineStr">
         <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="E198" s="61" t="n">
+        <v>13</v>
+      </c>
+      <c r="F198" s="61" t="n">
+        <v>22</v>
+      </c>
+      <c r="G198" s="61" t="n">
+        <v>33</v>
+      </c>
+      <c r="H198" s="61" t="n">
+        <v>46</v>
+      </c>
+      <c r="I198" s="61" t="n">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="199" ht="15" customHeight="1">
+      <c r="A199" s="14" t="inlineStr">
+        <is>
           <t>Turkije</t>
         </is>
       </c>
-      <c r="E198" s="62" t="n">
+      <c r="E199" s="61" t="n">
         <v>13</v>
       </c>
-      <c r="F198" s="62" t="n">
+      <c r="F199" s="61" t="n">
         <v>22</v>
       </c>
-      <c r="G198" s="62" t="n">
+      <c r="G199" s="61" t="n">
         <v>33</v>
       </c>
-      <c r="H198" s="62" t="n">
+      <c r="H199" s="61" t="n">
         <v>46</v>
       </c>
-      <c r="I198" s="62" t="n">
+      <c r="I199" s="61" t="n">
         <v>61</v>
       </c>
     </row>
-    <row r="199" ht="8" customHeight="1"/>
-    <row r="200" ht="18" customHeight="1">
-      <c r="A200" s="3" t="inlineStr">
+    <row r="200" ht="8" customHeight="1"/>
+    <row r="201" ht="18" customHeight="1">
+      <c r="A201" s="3" t="inlineStr">
         <is>
           <t>▶  DECEPTIE — kies een land UIT de top-12 · punten schalen met ranking en uitvalsronde</t>
         </is>
       </c>
     </row>
-    <row r="201" ht="14" customHeight="1">
-      <c r="A201" s="12" t="inlineStr">
+    <row r="202" ht="14" customHeight="1">
+      <c r="A202" s="12" t="inlineStr">
         <is>
           <t>Land (favoriet)</t>
         </is>
       </c>
-      <c r="E201" s="12" t="inlineStr">
+      <c r="E202" s="12" t="inlineStr">
         <is>
           <t>KF</t>
         </is>
       </c>
-      <c r="F201" s="12" t="inlineStr">
+      <c r="F202" s="12" t="inlineStr">
         <is>
           <t>R16</t>
         </is>
       </c>
-      <c r="G201" s="12" t="inlineStr">
+      <c r="G202" s="12" t="inlineStr">
         <is>
           <t>R32</t>
         </is>
       </c>
-      <c r="H201" s="12" t="inlineStr">
+      <c r="H202" s="12" t="inlineStr">
         <is>
           <t>Groep eruit</t>
         </is>
-      </c>
-    </row>
-    <row r="202" ht="15" customHeight="1">
-      <c r="A202" s="14" t="inlineStr">
-        <is>
-          <t>Frankrijk</t>
-        </is>
-      </c>
-      <c r="E202" s="62" t="n">
-        <v>8</v>
-      </c>
-      <c r="F202" s="62" t="n">
-        <v>14</v>
-      </c>
-      <c r="G202" s="62" t="n">
-        <v>20</v>
-      </c>
-      <c r="H202" s="62" t="n">
-        <v>30</v>
       </c>
     </row>
     <row r="203" ht="15" customHeight="1">
       <c r="A203" s="14" t="inlineStr">
         <is>
-          <t>Spanje</t>
-        </is>
-      </c>
-      <c r="E203" s="62" t="n">
-        <v>7</v>
-      </c>
-      <c r="F203" s="62" t="n">
-        <v>13</v>
-      </c>
-      <c r="G203" s="62" t="n">
-        <v>19</v>
-      </c>
-      <c r="H203" s="62" t="n">
-        <v>28</v>
+          <t>Frankrijk</t>
+        </is>
+      </c>
+      <c r="E203" s="61" t="n">
+        <v>8</v>
+      </c>
+      <c r="F203" s="61" t="n">
+        <v>14</v>
+      </c>
+      <c r="G203" s="61" t="n">
+        <v>20</v>
+      </c>
+      <c r="H203" s="61" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="204" ht="15" customHeight="1">
       <c r="A204" s="14" t="inlineStr">
         <is>
-          <t>Argentinië</t>
-        </is>
-      </c>
-      <c r="E204" s="62" t="n">
-        <v>6</v>
-      </c>
-      <c r="F204" s="62" t="n">
-        <v>12</v>
-      </c>
-      <c r="G204" s="62" t="n">
-        <v>17</v>
-      </c>
-      <c r="H204" s="62" t="n">
-        <v>26</v>
+          <t>Spanje</t>
+        </is>
+      </c>
+      <c r="E204" s="61" t="n">
+        <v>7</v>
+      </c>
+      <c r="F204" s="61" t="n">
+        <v>13</v>
+      </c>
+      <c r="G204" s="61" t="n">
+        <v>19</v>
+      </c>
+      <c r="H204" s="61" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="205" ht="15" customHeight="1">
       <c r="A205" s="14" t="inlineStr">
         <is>
-          <t>Engeland</t>
-        </is>
-      </c>
-      <c r="E205" s="62" t="n">
+          <t>Argentinië</t>
+        </is>
+      </c>
+      <c r="E205" s="61" t="n">
         <v>6</v>
       </c>
-      <c r="F205" s="62" t="n">
-        <v>11</v>
-      </c>
-      <c r="G205" s="62" t="n">
-        <v>16</v>
-      </c>
-      <c r="H205" s="62" t="n">
-        <v>24</v>
+      <c r="F205" s="61" t="n">
+        <v>12</v>
+      </c>
+      <c r="G205" s="61" t="n">
+        <v>17</v>
+      </c>
+      <c r="H205" s="61" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="206" ht="15" customHeight="1">
       <c r="A206" s="14" t="inlineStr">
         <is>
-          <t>Portugal</t>
-        </is>
-      </c>
-      <c r="E206" s="62" t="n">
+          <t>Engeland</t>
+        </is>
+      </c>
+      <c r="E206" s="61" t="n">
         <v>6</v>
       </c>
-      <c r="F206" s="62" t="n">
-        <v>10</v>
-      </c>
-      <c r="G206" s="62" t="n">
-        <v>15</v>
-      </c>
-      <c r="H206" s="62" t="n">
-        <v>22</v>
+      <c r="F206" s="61" t="n">
+        <v>11</v>
+      </c>
+      <c r="G206" s="61" t="n">
+        <v>16</v>
+      </c>
+      <c r="H206" s="61" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="207" ht="15" customHeight="1">
       <c r="A207" s="14" t="inlineStr">
         <is>
-          <t>Brazilië</t>
-        </is>
-      </c>
-      <c r="E207" s="62" t="n">
-        <v>5</v>
-      </c>
-      <c r="F207" s="62" t="n">
-        <v>9</v>
-      </c>
-      <c r="G207" s="62" t="n">
-        <v>13</v>
-      </c>
-      <c r="H207" s="62" t="n">
-        <v>20</v>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="E207" s="61" t="n">
+        <v>6</v>
+      </c>
+      <c r="F207" s="61" t="n">
+        <v>10</v>
+      </c>
+      <c r="G207" s="61" t="n">
+        <v>15</v>
+      </c>
+      <c r="H207" s="61" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="208" ht="15" customHeight="1">
       <c r="A208" s="14" t="inlineStr">
         <is>
-          <t>Nederland</t>
-        </is>
-      </c>
-      <c r="E208" s="62" t="n">
-        <v>4</v>
-      </c>
-      <c r="F208" s="62" t="n">
-        <v>8</v>
-      </c>
-      <c r="G208" s="62" t="n">
-        <v>12</v>
-      </c>
-      <c r="H208" s="62" t="n">
-        <v>18</v>
+          <t>Brazilië</t>
+        </is>
+      </c>
+      <c r="E208" s="61" t="n">
+        <v>5</v>
+      </c>
+      <c r="F208" s="61" t="n">
+        <v>9</v>
+      </c>
+      <c r="G208" s="61" t="n">
+        <v>13</v>
+      </c>
+      <c r="H208" s="61" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="209" ht="15" customHeight="1">
       <c r="A209" s="14" t="inlineStr">
         <is>
-          <t>Marokko</t>
-        </is>
-      </c>
-      <c r="E209" s="62" t="n">
+          <t>Nederland</t>
+        </is>
+      </c>
+      <c r="E209" s="61" t="n">
         <v>4</v>
       </c>
-      <c r="F209" s="62" t="n">
-        <v>7</v>
-      </c>
-      <c r="G209" s="62" t="n">
-        <v>11</v>
-      </c>
-      <c r="H209" s="62" t="n">
-        <v>16</v>
+      <c r="F209" s="61" t="n">
+        <v>8</v>
+      </c>
+      <c r="G209" s="61" t="n">
+        <v>12</v>
+      </c>
+      <c r="H209" s="61" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="210" ht="15" customHeight="1">
       <c r="A210" s="14" t="inlineStr">
         <is>
-          <t>België</t>
-        </is>
-      </c>
-      <c r="E210" s="62" t="n">
+          <t>Marokko</t>
+        </is>
+      </c>
+      <c r="E210" s="61" t="n">
         <v>4</v>
       </c>
-      <c r="F210" s="62" t="n">
-        <v>6</v>
-      </c>
-      <c r="G210" s="62" t="n">
-        <v>9</v>
-      </c>
-      <c r="H210" s="62" t="n">
-        <v>14</v>
+      <c r="F210" s="61" t="n">
+        <v>7</v>
+      </c>
+      <c r="G210" s="61" t="n">
+        <v>11</v>
+      </c>
+      <c r="H210" s="61" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="211" ht="15" customHeight="1">
       <c r="A211" s="14" t="inlineStr">
         <is>
-          <t>Duitsland</t>
-        </is>
-      </c>
-      <c r="E211" s="62" t="n">
-        <v>3</v>
-      </c>
-      <c r="F211" s="62" t="n">
+          <t>België</t>
+        </is>
+      </c>
+      <c r="E211" s="61" t="n">
+        <v>4</v>
+      </c>
+      <c r="F211" s="61" t="n">
         <v>6</v>
       </c>
-      <c r="G211" s="62" t="n">
-        <v>8</v>
-      </c>
-      <c r="H211" s="62" t="n">
-        <v>12</v>
+      <c r="G211" s="61" t="n">
+        <v>9</v>
+      </c>
+      <c r="H211" s="61" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="212" ht="15" customHeight="1">
       <c r="A212" s="14" t="inlineStr">
         <is>
-          <t>Kroatië</t>
-        </is>
-      </c>
-      <c r="E212" s="62" t="n">
-        <v>2</v>
-      </c>
-      <c r="F212" s="62" t="n">
-        <v>5</v>
-      </c>
-      <c r="G212" s="62" t="n">
-        <v>7</v>
-      </c>
-      <c r="H212" s="62" t="n">
-        <v>10</v>
+          <t>Duitsland</t>
+        </is>
+      </c>
+      <c r="E212" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="F212" s="61" t="n">
+        <v>6</v>
+      </c>
+      <c r="G212" s="61" t="n">
+        <v>8</v>
+      </c>
+      <c r="H212" s="61" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="213" ht="15" customHeight="1">
       <c r="A213" s="14" t="inlineStr">
         <is>
+          <t>Kroatië</t>
+        </is>
+      </c>
+      <c r="E213" s="61" t="n">
+        <v>2</v>
+      </c>
+      <c r="F213" s="61" t="n">
+        <v>5</v>
+      </c>
+      <c r="G213" s="61" t="n">
+        <v>7</v>
+      </c>
+      <c r="H213" s="61" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="214" ht="15" customHeight="1">
+      <c r="A214" s="14" t="inlineStr">
+        <is>
           <t>Colombia</t>
         </is>
       </c>
-      <c r="E213" s="62" t="n">
+      <c r="E214" s="61" t="n">
         <v>2</v>
       </c>
-      <c r="F213" s="62" t="n">
+      <c r="F214" s="61" t="n">
         <v>3</v>
       </c>
-      <c r="G213" s="62" t="n">
+      <c r="G214" s="61" t="n">
         <v>4</v>
       </c>
-      <c r="H213" s="62" t="n">
+      <c r="H214" s="61" t="n">
         <v>6</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="204">
+  <mergeCells count="187">
+    <mergeCell ref="A150:D150"/>
     <mergeCell ref="E13:G13"/>
     <mergeCell ref="A122:D122"/>
     <mergeCell ref="A97:D97"/>
-    <mergeCell ref="A133:O133"/>
-    <mergeCell ref="A134:D134"/>
-    <mergeCell ref="A152:D152"/>
+    <mergeCell ref="A159:D159"/>
+    <mergeCell ref="M111:N111"/>
+    <mergeCell ref="E111:F111"/>
     <mergeCell ref="A121:D121"/>
     <mergeCell ref="E15:G15"/>
     <mergeCell ref="A13:D13"/>
     <mergeCell ref="A202:D202"/>
     <mergeCell ref="A176:D176"/>
     <mergeCell ref="A15:D15"/>
-    <mergeCell ref="E57:G57"/>
     <mergeCell ref="A186:D186"/>
-    <mergeCell ref="M106:O106"/>
     <mergeCell ref="A107:D107"/>
     <mergeCell ref="A178:D178"/>
-    <mergeCell ref="M76:O76"/>
     <mergeCell ref="E16:G16"/>
     <mergeCell ref="A29:O29"/>
-    <mergeCell ref="A200:O200"/>
     <mergeCell ref="B44:O44"/>
-    <mergeCell ref="A161:O161"/>
-    <mergeCell ref="M66:O66"/>
+    <mergeCell ref="A152:O152"/>
     <mergeCell ref="I106:L106"/>
     <mergeCell ref="A124:D124"/>
     <mergeCell ref="A31:O31"/>
@@ -5143,19 +5367,18 @@
     <mergeCell ref="A172:D172"/>
     <mergeCell ref="A99:D99"/>
     <mergeCell ref="A164:D164"/>
-    <mergeCell ref="E106:G106"/>
     <mergeCell ref="A212:D212"/>
     <mergeCell ref="I66:L66"/>
     <mergeCell ref="A56:D56"/>
     <mergeCell ref="A24:O24"/>
     <mergeCell ref="A154:D154"/>
     <mergeCell ref="A149:D149"/>
+    <mergeCell ref="A214:D214"/>
     <mergeCell ref="A163:D163"/>
-    <mergeCell ref="M67:O67"/>
     <mergeCell ref="A6:C6"/>
+    <mergeCell ref="A111:B111"/>
     <mergeCell ref="A195:D195"/>
     <mergeCell ref="A204:D204"/>
-    <mergeCell ref="E107:G107"/>
     <mergeCell ref="A188:D188"/>
     <mergeCell ref="A126:D126"/>
     <mergeCell ref="A141:D141"/>
@@ -5166,36 +5389,28 @@
     <mergeCell ref="A190:D190"/>
     <mergeCell ref="A18:O18"/>
     <mergeCell ref="A117:D117"/>
-    <mergeCell ref="E77:G77"/>
-    <mergeCell ref="M86:O86"/>
+    <mergeCell ref="A199:D199"/>
     <mergeCell ref="A9:D9"/>
-    <mergeCell ref="E86:G86"/>
     <mergeCell ref="A127:D127"/>
     <mergeCell ref="A167:D167"/>
-    <mergeCell ref="A151:O151"/>
+    <mergeCell ref="I112:J112"/>
     <mergeCell ref="A59:D59"/>
     <mergeCell ref="I77:L77"/>
     <mergeCell ref="A142:D142"/>
-    <mergeCell ref="M57:O57"/>
     <mergeCell ref="A11:D11"/>
     <mergeCell ref="A22:O22"/>
     <mergeCell ref="B42:O42"/>
     <mergeCell ref="I86:L86"/>
-    <mergeCell ref="M97:O97"/>
-    <mergeCell ref="A144:O144"/>
+    <mergeCell ref="A182:D182"/>
+    <mergeCell ref="A191:D191"/>
     <mergeCell ref="A169:D169"/>
     <mergeCell ref="I89:L89"/>
-    <mergeCell ref="A182:D182"/>
-    <mergeCell ref="A191:D191"/>
     <mergeCell ref="A20:O20"/>
     <mergeCell ref="A79:D79"/>
-    <mergeCell ref="E97:G97"/>
+    <mergeCell ref="A134:O134"/>
+    <mergeCell ref="I111:J111"/>
     <mergeCell ref="I57:L57"/>
     <mergeCell ref="A153:D153"/>
-    <mergeCell ref="A162:D162"/>
-    <mergeCell ref="M56:O56"/>
-    <mergeCell ref="E56:G56"/>
-    <mergeCell ref="E96:G96"/>
     <mergeCell ref="B34:O34"/>
     <mergeCell ref="A128:D128"/>
     <mergeCell ref="B28:O28"/>
@@ -5207,8 +5422,6 @@
     <mergeCell ref="A136:D136"/>
     <mergeCell ref="I56:L56"/>
     <mergeCell ref="I96:L96"/>
-    <mergeCell ref="M107:O107"/>
-    <mergeCell ref="A145:D145"/>
     <mergeCell ref="A192:D192"/>
     <mergeCell ref="B30:O30"/>
     <mergeCell ref="A139:D139"/>
@@ -5217,6 +5430,7 @@
     <mergeCell ref="A129:D129"/>
     <mergeCell ref="A194:D194"/>
     <mergeCell ref="A76:D76"/>
+    <mergeCell ref="A162:O162"/>
     <mergeCell ref="I107:L107"/>
     <mergeCell ref="A116:D116"/>
     <mergeCell ref="A181:D181"/>
@@ -5232,16 +5446,16 @@
     <mergeCell ref="E9:G9"/>
     <mergeCell ref="A10:D10"/>
     <mergeCell ref="B46:O46"/>
-    <mergeCell ref="A115:D115"/>
+    <mergeCell ref="A145:O145"/>
+    <mergeCell ref="A155:D155"/>
     <mergeCell ref="I59:L59"/>
     <mergeCell ref="I99:L99"/>
     <mergeCell ref="A173:D173"/>
-    <mergeCell ref="M77:O77"/>
     <mergeCell ref="E11:G11"/>
     <mergeCell ref="A77:D77"/>
     <mergeCell ref="I69:L69"/>
+    <mergeCell ref="A143:D143"/>
     <mergeCell ref="A33:O33"/>
-    <mergeCell ref="A157:D157"/>
     <mergeCell ref="A166:D166"/>
     <mergeCell ref="A8:O8"/>
     <mergeCell ref="A49:D49"/>
@@ -5249,13 +5463,11 @@
     <mergeCell ref="A35:O35"/>
     <mergeCell ref="A168:D168"/>
     <mergeCell ref="A69:D69"/>
+    <mergeCell ref="A115:O115"/>
     <mergeCell ref="A19:O19"/>
     <mergeCell ref="A205:D205"/>
     <mergeCell ref="A87:D87"/>
     <mergeCell ref="E12:G12"/>
-    <mergeCell ref="A111:O111"/>
-    <mergeCell ref="M87:O87"/>
-    <mergeCell ref="M96:O96"/>
     <mergeCell ref="A193:D193"/>
     <mergeCell ref="A39:O39"/>
     <mergeCell ref="I97:L97"/>
@@ -5264,10 +5476,10 @@
     <mergeCell ref="E14:G14"/>
     <mergeCell ref="A12:D12"/>
     <mergeCell ref="I87:L87"/>
+    <mergeCell ref="E112:F112"/>
     <mergeCell ref="A45:O45"/>
     <mergeCell ref="A57:D57"/>
     <mergeCell ref="B36:O36"/>
-    <mergeCell ref="E87:G87"/>
     <mergeCell ref="A14:D14"/>
     <mergeCell ref="A185:D185"/>
     <mergeCell ref="A106:D106"/>
@@ -5281,20 +5493,16 @@
     <mergeCell ref="A211:D211"/>
     <mergeCell ref="A26:O26"/>
     <mergeCell ref="A67:D67"/>
-    <mergeCell ref="A113:O113"/>
     <mergeCell ref="A130:D130"/>
-    <mergeCell ref="A201:D201"/>
     <mergeCell ref="A148:D148"/>
     <mergeCell ref="A23:O23"/>
-    <mergeCell ref="E76:G76"/>
     <mergeCell ref="I49:L49"/>
     <mergeCell ref="A123:D123"/>
     <mergeCell ref="A138:D138"/>
+    <mergeCell ref="A132:D132"/>
     <mergeCell ref="A197:D197"/>
     <mergeCell ref="A43:O43"/>
     <mergeCell ref="A146:D146"/>
-    <mergeCell ref="A156:O156"/>
-    <mergeCell ref="E66:G66"/>
     <mergeCell ref="A119:D119"/>
     <mergeCell ref="B38:O38"/>
     <mergeCell ref="A187:D187"/>
@@ -5303,20 +5511,23 @@
     <mergeCell ref="A174:D174"/>
     <mergeCell ref="A183:D183"/>
     <mergeCell ref="A66:D66"/>
+    <mergeCell ref="A201:O201"/>
     <mergeCell ref="B40:O40"/>
     <mergeCell ref="A118:D118"/>
     <mergeCell ref="A189:D189"/>
+    <mergeCell ref="A157:O157"/>
     <mergeCell ref="A158:D158"/>
     <mergeCell ref="A198:D198"/>
-    <mergeCell ref="E67:G67"/>
+    <mergeCell ref="A112:B112"/>
     <mergeCell ref="A86:D86"/>
+    <mergeCell ref="M112:N112"/>
     <mergeCell ref="A110:O110"/>
     <mergeCell ref="A213:D213"/>
     <mergeCell ref="A175:D175"/>
     <mergeCell ref="I67:L67"/>
     <mergeCell ref="B32:O32"/>
   </mergeCells>
-  <dataValidations count="3">
+  <dataValidations count="35">
     <dataValidation sqref="E9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Landen!$A$1:$A$48</formula1>
     </dataValidation>
@@ -5326,6 +5537,102 @@
     <dataValidation sqref="E11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Landen!$C$1:$C$12</formula1>
     </dataValidation>
+    <dataValidation sqref="E56" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=Landen!$D$1:$D$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="M56" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=Landen!$E$1:$E$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="E57" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=Landen!$D$1:$D$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="M57" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=Landen!$E$1:$E$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="E66" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=Landen!$F$1:$F$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="M66" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=Landen!$G$1:$G$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="E67" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=Landen!$F$1:$F$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="M67" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=Landen!$G$1:$G$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="E76" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=Landen!$H$1:$H$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="M76" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=Landen!$I$1:$I$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="E77" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=Landen!$H$1:$H$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="M77" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=Landen!$I$1:$I$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="E86" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=Landen!$J$1:$J$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="M86" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=Landen!$K$1:$K$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="E87" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=Landen!$J$1:$J$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="M87" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=Landen!$K$1:$K$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="E96" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=Landen!$L$1:$L$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="M96" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=Landen!$M$1:$M$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="E97" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=Landen!$L$1:$L$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="M97" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=Landen!$M$1:$M$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="E106" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=Landen!$N$1:$N$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="M106" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=Landen!$O$1:$O$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="E107" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=Landen!$N$1:$N$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="M107" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=Landen!$O$1:$O$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="C111" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=Landen!$A$1:$A$48</formula1>
+    </dataValidation>
+    <dataValidation sqref="G111" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=Landen!$A$1:$A$48</formula1>
+    </dataValidation>
+    <dataValidation sqref="K111" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=Landen!$A$1:$A$48</formula1>
+    </dataValidation>
+    <dataValidation sqref="O111" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=Landen!$A$1:$A$48</formula1>
+    </dataValidation>
+    <dataValidation sqref="C112" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=Landen!$A$1:$A$48</formula1>
+    </dataValidation>
+    <dataValidation sqref="G112" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=Landen!$A$1:$A$48</formula1>
+    </dataValidation>
+    <dataValidation sqref="K112" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=Landen!$A$1:$A$48</formula1>
+    </dataValidation>
+    <dataValidation sqref="O112" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=Landen!$A$1:$A$48</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>